<commit_message>
0.6 Bindings gefixt (5.1.1.6)
</commit_message>
<xml_diff>
--- a/Projekttagebuch.xlsx
+++ b/Projekttagebuch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\projects\GW.Demo.Maui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4A69A8-43B1-4CCB-BFD7-CED0A21CD247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FEF5D-B9F5-4CEF-979F-DC51AEA9698A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1DD67F99-F2FF-45C7-A69A-922EBC32F5C0}"/>
   </bookViews>
@@ -235,9 +235,6 @@
 https://medium.com/@cristian_lopes/net-maui-flyout-navigation-tab-navigation-ca62913c98fa</t>
   </si>
   <si>
-    <t>166</t>
-  </si>
-  <si>
     <t>Menü-Commands feuern nicht, mühsam, Video und AI haben geholfen.
 Um das mit Commands zu machen, musste ich dann noch weiter rumzangeln. Richtiges VM haben wir so einmal nicht.</t>
   </si>
@@ -277,9 +274,6 @@
     <t>48</t>
   </si>
   <si>
-    <t>121</t>
-  </si>
-  <si>
     <t>https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/listview
 https://www.codemag.com/Article/2503021/Exploring-.NET-MAUI-Working-with-Lists-of-Data
 https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/collectionview
@@ -289,6 +283,12 @@
   </si>
   <si>
     <t>Im Großen und Ganzen wenig problematisch. Dokumentation ok. Wieder Binding-Fehler, wenn man das schon öfter gehabt hat, tut man sich leichter, CoPilot hilft zT. auch aus.</t>
+  </si>
+  <si>
+    <t>186</t>
+  </si>
+  <si>
+    <t>162</t>
   </si>
 </sst>
 </file>
@@ -3374,7 +3374,7 @@
       <c r="B46" s="44"/>
       <c r="C46" s="5"/>
       <c r="D46" s="41" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E46" s="42"/>
       <c r="F46" s="6" t="s">
@@ -3626,7 +3626,7 @@
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
       <c r="H54" s="32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I54" s="33"/>
       <c r="J54" s="33"/>
@@ -3930,7 +3930,7 @@
       <c r="B65" s="44"/>
       <c r="C65" s="5"/>
       <c r="D65" s="41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E65" s="42"/>
       <c r="F65" s="6" t="s">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I65" s="33"/>
       <c r="J65" s="33"/>
@@ -4272,7 +4272,7 @@
       <c r="F76" s="6"/>
       <c r="G76" s="6"/>
       <c r="H76" s="32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I76" s="33"/>
       <c r="J76" s="33"/>
@@ -4576,7 +4576,7 @@
       <c r="B87" s="44"/>
       <c r="C87" s="5"/>
       <c r="D87" s="41" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E87" s="42"/>
       <c r="F87" s="6" t="s">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="G87" s="6"/>
       <c r="H87" s="32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I87" s="33"/>
       <c r="J87" s="33"/>
@@ -4828,7 +4828,7 @@
       <c r="F95" s="6"/>
       <c r="G95" s="6"/>
       <c r="H95" s="32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I95" s="33"/>
       <c r="J95" s="33"/>
@@ -5132,7 +5132,7 @@
       <c r="B106" s="44"/>
       <c r="C106" s="5"/>
       <c r="D106" s="41" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E106" s="42"/>
       <c r="F106" s="6" t="s">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="G106" s="6"/>
       <c r="H106" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I106" s="33"/>
       <c r="J106" s="33"/>
@@ -5384,7 +5384,7 @@
       <c r="F114" s="6"/>
       <c r="G114" s="6"/>
       <c r="H114" s="32" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I114" s="33"/>
       <c r="J114" s="33"/>

</xml_diff>

<commit_message>
0.8 (5.1.1.7)  Video streamen
</commit_message>
<xml_diff>
--- a/Projekttagebuch.xlsx
+++ b/Projekttagebuch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\projects\GW.Demo.Maui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FEF5D-B9F5-4CEF-979F-DC51AEA9698A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DBF2A8D-30D6-4535-A3DB-09311CFBC2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1DD67F99-F2FF-45C7-A69A-922EBC32F5C0}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="71">
   <si>
     <t>Framework:</t>
   </si>
@@ -289,6 +289,17 @@
   </si>
   <si>
     <t>162</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/de-de/dotnet/communitytoolkit/maui/views/mediaelement
+https://www.c-sharpcorner.com/article/net-maui-video-player-using-community-toolkit/
+https://www.infoq.com/news/2023/02/dot-net-maui-mediaelement/</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>MediaElement ist eher komfortabel.</t>
   </si>
 </sst>
 </file>
@@ -620,12 +631,6 @@
     <xf numFmtId="49" fontId="1" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -652,6 +657,12 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2185,11 +2196,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>11</v>
       </c>
@@ -5687,33 +5698,37 @@
     <row r="125" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B125" s="44"/>
       <c r="C125" s="5"/>
-      <c r="D125" s="41"/>
+      <c r="D125" s="41" t="s">
+        <v>69</v>
+      </c>
       <c r="E125" s="42"/>
       <c r="F125" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G125" s="6"/>
-      <c r="H125" s="48"/>
-      <c r="I125" s="49"/>
-      <c r="J125" s="49"/>
-      <c r="K125" s="49"/>
-      <c r="L125" s="49"/>
-      <c r="M125" s="49"/>
-      <c r="N125" s="49"/>
-      <c r="O125" s="49"/>
-      <c r="P125" s="49"/>
-      <c r="Q125" s="49"/>
-      <c r="R125" s="49"/>
-      <c r="S125" s="49"/>
-      <c r="T125" s="49"/>
-      <c r="U125" s="49"/>
-      <c r="V125" s="49"/>
-      <c r="W125" s="49"/>
-      <c r="X125" s="49"/>
-      <c r="Y125" s="49"/>
-      <c r="Z125" s="49"/>
-      <c r="AA125" s="49"/>
-      <c r="AB125" s="50"/>
+      <c r="H125" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="I125" s="33"/>
+      <c r="J125" s="33"/>
+      <c r="K125" s="33"/>
+      <c r="L125" s="33"/>
+      <c r="M125" s="33"/>
+      <c r="N125" s="33"/>
+      <c r="O125" s="33"/>
+      <c r="P125" s="33"/>
+      <c r="Q125" s="33"/>
+      <c r="R125" s="33"/>
+      <c r="S125" s="33"/>
+      <c r="T125" s="33"/>
+      <c r="U125" s="33"/>
+      <c r="V125" s="33"/>
+      <c r="W125" s="33"/>
+      <c r="X125" s="33"/>
+      <c r="Y125" s="33"/>
+      <c r="Z125" s="33"/>
+      <c r="AA125" s="33"/>
+      <c r="AB125" s="34"/>
       <c r="AC125" s="11"/>
     </row>
     <row r="126" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5723,27 +5738,27 @@
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
       <c r="G126" s="6"/>
-      <c r="H126" s="51"/>
-      <c r="I126" s="52"/>
-      <c r="J126" s="52"/>
-      <c r="K126" s="52"/>
-      <c r="L126" s="52"/>
-      <c r="M126" s="52"/>
-      <c r="N126" s="52"/>
-      <c r="O126" s="52"/>
-      <c r="P126" s="52"/>
-      <c r="Q126" s="52"/>
-      <c r="R126" s="52"/>
-      <c r="S126" s="52"/>
-      <c r="T126" s="52"/>
-      <c r="U126" s="52"/>
-      <c r="V126" s="52"/>
-      <c r="W126" s="52"/>
-      <c r="X126" s="52"/>
-      <c r="Y126" s="52"/>
-      <c r="Z126" s="52"/>
-      <c r="AA126" s="52"/>
-      <c r="AB126" s="53"/>
+      <c r="H126" s="35"/>
+      <c r="I126" s="36"/>
+      <c r="J126" s="36"/>
+      <c r="K126" s="36"/>
+      <c r="L126" s="36"/>
+      <c r="M126" s="36"/>
+      <c r="N126" s="36"/>
+      <c r="O126" s="36"/>
+      <c r="P126" s="36"/>
+      <c r="Q126" s="36"/>
+      <c r="R126" s="36"/>
+      <c r="S126" s="36"/>
+      <c r="T126" s="36"/>
+      <c r="U126" s="36"/>
+      <c r="V126" s="36"/>
+      <c r="W126" s="36"/>
+      <c r="X126" s="36"/>
+      <c r="Y126" s="36"/>
+      <c r="Z126" s="36"/>
+      <c r="AA126" s="36"/>
+      <c r="AB126" s="37"/>
       <c r="AC126" s="11"/>
     </row>
     <row r="127" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5753,27 +5768,27 @@
       <c r="E127" s="6"/>
       <c r="F127" s="6"/>
       <c r="G127" s="6"/>
-      <c r="H127" s="51"/>
-      <c r="I127" s="52"/>
-      <c r="J127" s="52"/>
-      <c r="K127" s="52"/>
-      <c r="L127" s="52"/>
-      <c r="M127" s="52"/>
-      <c r="N127" s="52"/>
-      <c r="O127" s="52"/>
-      <c r="P127" s="52"/>
-      <c r="Q127" s="52"/>
-      <c r="R127" s="52"/>
-      <c r="S127" s="52"/>
-      <c r="T127" s="52"/>
-      <c r="U127" s="52"/>
-      <c r="V127" s="52"/>
-      <c r="W127" s="52"/>
-      <c r="X127" s="52"/>
-      <c r="Y127" s="52"/>
-      <c r="Z127" s="52"/>
-      <c r="AA127" s="52"/>
-      <c r="AB127" s="53"/>
+      <c r="H127" s="35"/>
+      <c r="I127" s="36"/>
+      <c r="J127" s="36"/>
+      <c r="K127" s="36"/>
+      <c r="L127" s="36"/>
+      <c r="M127" s="36"/>
+      <c r="N127" s="36"/>
+      <c r="O127" s="36"/>
+      <c r="P127" s="36"/>
+      <c r="Q127" s="36"/>
+      <c r="R127" s="36"/>
+      <c r="S127" s="36"/>
+      <c r="T127" s="36"/>
+      <c r="U127" s="36"/>
+      <c r="V127" s="36"/>
+      <c r="W127" s="36"/>
+      <c r="X127" s="36"/>
+      <c r="Y127" s="36"/>
+      <c r="Z127" s="36"/>
+      <c r="AA127" s="36"/>
+      <c r="AB127" s="37"/>
       <c r="AC127" s="11"/>
     </row>
     <row r="128" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5783,27 +5798,27 @@
       <c r="E128" s="6"/>
       <c r="F128" s="6"/>
       <c r="G128" s="6"/>
-      <c r="H128" s="51"/>
-      <c r="I128" s="52"/>
-      <c r="J128" s="52"/>
-      <c r="K128" s="52"/>
-      <c r="L128" s="52"/>
-      <c r="M128" s="52"/>
-      <c r="N128" s="52"/>
-      <c r="O128" s="52"/>
-      <c r="P128" s="52"/>
-      <c r="Q128" s="52"/>
-      <c r="R128" s="52"/>
-      <c r="S128" s="52"/>
-      <c r="T128" s="52"/>
-      <c r="U128" s="52"/>
-      <c r="V128" s="52"/>
-      <c r="W128" s="52"/>
-      <c r="X128" s="52"/>
-      <c r="Y128" s="52"/>
-      <c r="Z128" s="52"/>
-      <c r="AA128" s="52"/>
-      <c r="AB128" s="53"/>
+      <c r="H128" s="35"/>
+      <c r="I128" s="36"/>
+      <c r="J128" s="36"/>
+      <c r="K128" s="36"/>
+      <c r="L128" s="36"/>
+      <c r="M128" s="36"/>
+      <c r="N128" s="36"/>
+      <c r="O128" s="36"/>
+      <c r="P128" s="36"/>
+      <c r="Q128" s="36"/>
+      <c r="R128" s="36"/>
+      <c r="S128" s="36"/>
+      <c r="T128" s="36"/>
+      <c r="U128" s="36"/>
+      <c r="V128" s="36"/>
+      <c r="W128" s="36"/>
+      <c r="X128" s="36"/>
+      <c r="Y128" s="36"/>
+      <c r="Z128" s="36"/>
+      <c r="AA128" s="36"/>
+      <c r="AB128" s="37"/>
       <c r="AC128" s="11"/>
     </row>
     <row r="129" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5813,27 +5828,27 @@
       <c r="E129" s="6"/>
       <c r="F129" s="6"/>
       <c r="G129" s="6"/>
-      <c r="H129" s="51"/>
-      <c r="I129" s="52"/>
-      <c r="J129" s="52"/>
-      <c r="K129" s="52"/>
-      <c r="L129" s="52"/>
-      <c r="M129" s="52"/>
-      <c r="N129" s="52"/>
-      <c r="O129" s="52"/>
-      <c r="P129" s="52"/>
-      <c r="Q129" s="52"/>
-      <c r="R129" s="52"/>
-      <c r="S129" s="52"/>
-      <c r="T129" s="52"/>
-      <c r="U129" s="52"/>
-      <c r="V129" s="52"/>
-      <c r="W129" s="52"/>
-      <c r="X129" s="52"/>
-      <c r="Y129" s="52"/>
-      <c r="Z129" s="52"/>
-      <c r="AA129" s="52"/>
-      <c r="AB129" s="53"/>
+      <c r="H129" s="35"/>
+      <c r="I129" s="36"/>
+      <c r="J129" s="36"/>
+      <c r="K129" s="36"/>
+      <c r="L129" s="36"/>
+      <c r="M129" s="36"/>
+      <c r="N129" s="36"/>
+      <c r="O129" s="36"/>
+      <c r="P129" s="36"/>
+      <c r="Q129" s="36"/>
+      <c r="R129" s="36"/>
+      <c r="S129" s="36"/>
+      <c r="T129" s="36"/>
+      <c r="U129" s="36"/>
+      <c r="V129" s="36"/>
+      <c r="W129" s="36"/>
+      <c r="X129" s="36"/>
+      <c r="Y129" s="36"/>
+      <c r="Z129" s="36"/>
+      <c r="AA129" s="36"/>
+      <c r="AB129" s="37"/>
       <c r="AC129" s="11"/>
     </row>
     <row r="130" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5843,27 +5858,27 @@
       <c r="E130" s="6"/>
       <c r="F130" s="6"/>
       <c r="G130" s="6"/>
-      <c r="H130" s="51"/>
-      <c r="I130" s="52"/>
-      <c r="J130" s="52"/>
-      <c r="K130" s="52"/>
-      <c r="L130" s="52"/>
-      <c r="M130" s="52"/>
-      <c r="N130" s="52"/>
-      <c r="O130" s="52"/>
-      <c r="P130" s="52"/>
-      <c r="Q130" s="52"/>
-      <c r="R130" s="52"/>
-      <c r="S130" s="52"/>
-      <c r="T130" s="52"/>
-      <c r="U130" s="52"/>
-      <c r="V130" s="52"/>
-      <c r="W130" s="52"/>
-      <c r="X130" s="52"/>
-      <c r="Y130" s="52"/>
-      <c r="Z130" s="52"/>
-      <c r="AA130" s="52"/>
-      <c r="AB130" s="53"/>
+      <c r="H130" s="35"/>
+      <c r="I130" s="36"/>
+      <c r="J130" s="36"/>
+      <c r="K130" s="36"/>
+      <c r="L130" s="36"/>
+      <c r="M130" s="36"/>
+      <c r="N130" s="36"/>
+      <c r="O130" s="36"/>
+      <c r="P130" s="36"/>
+      <c r="Q130" s="36"/>
+      <c r="R130" s="36"/>
+      <c r="S130" s="36"/>
+      <c r="T130" s="36"/>
+      <c r="U130" s="36"/>
+      <c r="V130" s="36"/>
+      <c r="W130" s="36"/>
+      <c r="X130" s="36"/>
+      <c r="Y130" s="36"/>
+      <c r="Z130" s="36"/>
+      <c r="AA130" s="36"/>
+      <c r="AB130" s="37"/>
       <c r="AC130" s="11"/>
     </row>
     <row r="131" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5873,27 +5888,27 @@
       <c r="E131" s="6"/>
       <c r="F131" s="6"/>
       <c r="G131" s="6"/>
-      <c r="H131" s="54"/>
-      <c r="I131" s="55"/>
-      <c r="J131" s="55"/>
-      <c r="K131" s="55"/>
-      <c r="L131" s="55"/>
-      <c r="M131" s="55"/>
-      <c r="N131" s="55"/>
-      <c r="O131" s="55"/>
-      <c r="P131" s="55"/>
-      <c r="Q131" s="55"/>
-      <c r="R131" s="55"/>
-      <c r="S131" s="55"/>
-      <c r="T131" s="55"/>
-      <c r="U131" s="55"/>
-      <c r="V131" s="55"/>
-      <c r="W131" s="55"/>
-      <c r="X131" s="55"/>
-      <c r="Y131" s="55"/>
-      <c r="Z131" s="55"/>
-      <c r="AA131" s="55"/>
-      <c r="AB131" s="56"/>
+      <c r="H131" s="38"/>
+      <c r="I131" s="39"/>
+      <c r="J131" s="39"/>
+      <c r="K131" s="39"/>
+      <c r="L131" s="39"/>
+      <c r="M131" s="39"/>
+      <c r="N131" s="39"/>
+      <c r="O131" s="39"/>
+      <c r="P131" s="39"/>
+      <c r="Q131" s="39"/>
+      <c r="R131" s="39"/>
+      <c r="S131" s="39"/>
+      <c r="T131" s="39"/>
+      <c r="U131" s="39"/>
+      <c r="V131" s="39"/>
+      <c r="W131" s="39"/>
+      <c r="X131" s="39"/>
+      <c r="Y131" s="39"/>
+      <c r="Z131" s="39"/>
+      <c r="AA131" s="39"/>
+      <c r="AB131" s="40"/>
       <c r="AC131" s="11"/>
     </row>
     <row r="132" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5935,27 +5950,29 @@
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
       <c r="G133" s="6"/>
-      <c r="H133" s="48"/>
-      <c r="I133" s="49"/>
-      <c r="J133" s="49"/>
-      <c r="K133" s="49"/>
-      <c r="L133" s="49"/>
-      <c r="M133" s="49"/>
-      <c r="N133" s="49"/>
-      <c r="O133" s="49"/>
-      <c r="P133" s="49"/>
-      <c r="Q133" s="49"/>
-      <c r="R133" s="49"/>
-      <c r="S133" s="49"/>
-      <c r="T133" s="49"/>
-      <c r="U133" s="49"/>
-      <c r="V133" s="49"/>
-      <c r="W133" s="49"/>
-      <c r="X133" s="49"/>
-      <c r="Y133" s="49"/>
-      <c r="Z133" s="49"/>
-      <c r="AA133" s="49"/>
-      <c r="AB133" s="50"/>
+      <c r="H133" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="I133" s="33"/>
+      <c r="J133" s="33"/>
+      <c r="K133" s="33"/>
+      <c r="L133" s="33"/>
+      <c r="M133" s="33"/>
+      <c r="N133" s="33"/>
+      <c r="O133" s="33"/>
+      <c r="P133" s="33"/>
+      <c r="Q133" s="33"/>
+      <c r="R133" s="33"/>
+      <c r="S133" s="33"/>
+      <c r="T133" s="33"/>
+      <c r="U133" s="33"/>
+      <c r="V133" s="33"/>
+      <c r="W133" s="33"/>
+      <c r="X133" s="33"/>
+      <c r="Y133" s="33"/>
+      <c r="Z133" s="33"/>
+      <c r="AA133" s="33"/>
+      <c r="AB133" s="34"/>
       <c r="AC133" s="11"/>
     </row>
     <row r="134" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5965,27 +5982,27 @@
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
       <c r="G134" s="6"/>
-      <c r="H134" s="51"/>
-      <c r="I134" s="52"/>
-      <c r="J134" s="52"/>
-      <c r="K134" s="52"/>
-      <c r="L134" s="52"/>
-      <c r="M134" s="52"/>
-      <c r="N134" s="52"/>
-      <c r="O134" s="52"/>
-      <c r="P134" s="52"/>
-      <c r="Q134" s="52"/>
-      <c r="R134" s="52"/>
-      <c r="S134" s="52"/>
-      <c r="T134" s="52"/>
-      <c r="U134" s="52"/>
-      <c r="V134" s="52"/>
-      <c r="W134" s="52"/>
-      <c r="X134" s="52"/>
-      <c r="Y134" s="52"/>
-      <c r="Z134" s="52"/>
-      <c r="AA134" s="52"/>
-      <c r="AB134" s="53"/>
+      <c r="H134" s="35"/>
+      <c r="I134" s="36"/>
+      <c r="J134" s="36"/>
+      <c r="K134" s="36"/>
+      <c r="L134" s="36"/>
+      <c r="M134" s="36"/>
+      <c r="N134" s="36"/>
+      <c r="O134" s="36"/>
+      <c r="P134" s="36"/>
+      <c r="Q134" s="36"/>
+      <c r="R134" s="36"/>
+      <c r="S134" s="36"/>
+      <c r="T134" s="36"/>
+      <c r="U134" s="36"/>
+      <c r="V134" s="36"/>
+      <c r="W134" s="36"/>
+      <c r="X134" s="36"/>
+      <c r="Y134" s="36"/>
+      <c r="Z134" s="36"/>
+      <c r="AA134" s="36"/>
+      <c r="AB134" s="37"/>
       <c r="AC134" s="11"/>
     </row>
     <row r="135" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5995,27 +6012,27 @@
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
       <c r="G135" s="6"/>
-      <c r="H135" s="51"/>
-      <c r="I135" s="52"/>
-      <c r="J135" s="52"/>
-      <c r="K135" s="52"/>
-      <c r="L135" s="52"/>
-      <c r="M135" s="52"/>
-      <c r="N135" s="52"/>
-      <c r="O135" s="52"/>
-      <c r="P135" s="52"/>
-      <c r="Q135" s="52"/>
-      <c r="R135" s="52"/>
-      <c r="S135" s="52"/>
-      <c r="T135" s="52"/>
-      <c r="U135" s="52"/>
-      <c r="V135" s="52"/>
-      <c r="W135" s="52"/>
-      <c r="X135" s="52"/>
-      <c r="Y135" s="52"/>
-      <c r="Z135" s="52"/>
-      <c r="AA135" s="52"/>
-      <c r="AB135" s="53"/>
+      <c r="H135" s="35"/>
+      <c r="I135" s="36"/>
+      <c r="J135" s="36"/>
+      <c r="K135" s="36"/>
+      <c r="L135" s="36"/>
+      <c r="M135" s="36"/>
+      <c r="N135" s="36"/>
+      <c r="O135" s="36"/>
+      <c r="P135" s="36"/>
+      <c r="Q135" s="36"/>
+      <c r="R135" s="36"/>
+      <c r="S135" s="36"/>
+      <c r="T135" s="36"/>
+      <c r="U135" s="36"/>
+      <c r="V135" s="36"/>
+      <c r="W135" s="36"/>
+      <c r="X135" s="36"/>
+      <c r="Y135" s="36"/>
+      <c r="Z135" s="36"/>
+      <c r="AA135" s="36"/>
+      <c r="AB135" s="37"/>
       <c r="AC135" s="11"/>
     </row>
     <row r="136" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6025,27 +6042,27 @@
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
       <c r="G136" s="6"/>
-      <c r="H136" s="51"/>
-      <c r="I136" s="52"/>
-      <c r="J136" s="52"/>
-      <c r="K136" s="52"/>
-      <c r="L136" s="52"/>
-      <c r="M136" s="52"/>
-      <c r="N136" s="52"/>
-      <c r="O136" s="52"/>
-      <c r="P136" s="52"/>
-      <c r="Q136" s="52"/>
-      <c r="R136" s="52"/>
-      <c r="S136" s="52"/>
-      <c r="T136" s="52"/>
-      <c r="U136" s="52"/>
-      <c r="V136" s="52"/>
-      <c r="W136" s="52"/>
-      <c r="X136" s="52"/>
-      <c r="Y136" s="52"/>
-      <c r="Z136" s="52"/>
-      <c r="AA136" s="52"/>
-      <c r="AB136" s="53"/>
+      <c r="H136" s="35"/>
+      <c r="I136" s="36"/>
+      <c r="J136" s="36"/>
+      <c r="K136" s="36"/>
+      <c r="L136" s="36"/>
+      <c r="M136" s="36"/>
+      <c r="N136" s="36"/>
+      <c r="O136" s="36"/>
+      <c r="P136" s="36"/>
+      <c r="Q136" s="36"/>
+      <c r="R136" s="36"/>
+      <c r="S136" s="36"/>
+      <c r="T136" s="36"/>
+      <c r="U136" s="36"/>
+      <c r="V136" s="36"/>
+      <c r="W136" s="36"/>
+      <c r="X136" s="36"/>
+      <c r="Y136" s="36"/>
+      <c r="Z136" s="36"/>
+      <c r="AA136" s="36"/>
+      <c r="AB136" s="37"/>
       <c r="AC136" s="11"/>
     </row>
     <row r="137" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6055,27 +6072,27 @@
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
       <c r="G137" s="6"/>
-      <c r="H137" s="51"/>
-      <c r="I137" s="52"/>
-      <c r="J137" s="52"/>
-      <c r="K137" s="52"/>
-      <c r="L137" s="52"/>
-      <c r="M137" s="52"/>
-      <c r="N137" s="52"/>
-      <c r="O137" s="52"/>
-      <c r="P137" s="52"/>
-      <c r="Q137" s="52"/>
-      <c r="R137" s="52"/>
-      <c r="S137" s="52"/>
-      <c r="T137" s="52"/>
-      <c r="U137" s="52"/>
-      <c r="V137" s="52"/>
-      <c r="W137" s="52"/>
-      <c r="X137" s="52"/>
-      <c r="Y137" s="52"/>
-      <c r="Z137" s="52"/>
-      <c r="AA137" s="52"/>
-      <c r="AB137" s="53"/>
+      <c r="H137" s="35"/>
+      <c r="I137" s="36"/>
+      <c r="J137" s="36"/>
+      <c r="K137" s="36"/>
+      <c r="L137" s="36"/>
+      <c r="M137" s="36"/>
+      <c r="N137" s="36"/>
+      <c r="O137" s="36"/>
+      <c r="P137" s="36"/>
+      <c r="Q137" s="36"/>
+      <c r="R137" s="36"/>
+      <c r="S137" s="36"/>
+      <c r="T137" s="36"/>
+      <c r="U137" s="36"/>
+      <c r="V137" s="36"/>
+      <c r="W137" s="36"/>
+      <c r="X137" s="36"/>
+      <c r="Y137" s="36"/>
+      <c r="Z137" s="36"/>
+      <c r="AA137" s="36"/>
+      <c r="AB137" s="37"/>
       <c r="AC137" s="11"/>
     </row>
     <row r="138" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6085,27 +6102,27 @@
       <c r="E138" s="6"/>
       <c r="F138" s="6"/>
       <c r="G138" s="6"/>
-      <c r="H138" s="51"/>
-      <c r="I138" s="52"/>
-      <c r="J138" s="52"/>
-      <c r="K138" s="52"/>
-      <c r="L138" s="52"/>
-      <c r="M138" s="52"/>
-      <c r="N138" s="52"/>
-      <c r="O138" s="52"/>
-      <c r="P138" s="52"/>
-      <c r="Q138" s="52"/>
-      <c r="R138" s="52"/>
-      <c r="S138" s="52"/>
-      <c r="T138" s="52"/>
-      <c r="U138" s="52"/>
-      <c r="V138" s="52"/>
-      <c r="W138" s="52"/>
-      <c r="X138" s="52"/>
-      <c r="Y138" s="52"/>
-      <c r="Z138" s="52"/>
-      <c r="AA138" s="52"/>
-      <c r="AB138" s="53"/>
+      <c r="H138" s="35"/>
+      <c r="I138" s="36"/>
+      <c r="J138" s="36"/>
+      <c r="K138" s="36"/>
+      <c r="L138" s="36"/>
+      <c r="M138" s="36"/>
+      <c r="N138" s="36"/>
+      <c r="O138" s="36"/>
+      <c r="P138" s="36"/>
+      <c r="Q138" s="36"/>
+      <c r="R138" s="36"/>
+      <c r="S138" s="36"/>
+      <c r="T138" s="36"/>
+      <c r="U138" s="36"/>
+      <c r="V138" s="36"/>
+      <c r="W138" s="36"/>
+      <c r="X138" s="36"/>
+      <c r="Y138" s="36"/>
+      <c r="Z138" s="36"/>
+      <c r="AA138" s="36"/>
+      <c r="AB138" s="37"/>
       <c r="AC138" s="11"/>
     </row>
     <row r="139" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6115,27 +6132,27 @@
       <c r="E139" s="6"/>
       <c r="F139" s="6"/>
       <c r="G139" s="6"/>
-      <c r="H139" s="54"/>
-      <c r="I139" s="55"/>
-      <c r="J139" s="55"/>
-      <c r="K139" s="55"/>
-      <c r="L139" s="55"/>
-      <c r="M139" s="55"/>
-      <c r="N139" s="55"/>
-      <c r="O139" s="55"/>
-      <c r="P139" s="55"/>
-      <c r="Q139" s="55"/>
-      <c r="R139" s="55"/>
-      <c r="S139" s="55"/>
-      <c r="T139" s="55"/>
-      <c r="U139" s="55"/>
-      <c r="V139" s="55"/>
-      <c r="W139" s="55"/>
-      <c r="X139" s="55"/>
-      <c r="Y139" s="55"/>
-      <c r="Z139" s="55"/>
-      <c r="AA139" s="55"/>
-      <c r="AB139" s="56"/>
+      <c r="H139" s="38"/>
+      <c r="I139" s="39"/>
+      <c r="J139" s="39"/>
+      <c r="K139" s="39"/>
+      <c r="L139" s="39"/>
+      <c r="M139" s="39"/>
+      <c r="N139" s="39"/>
+      <c r="O139" s="39"/>
+      <c r="P139" s="39"/>
+      <c r="Q139" s="39"/>
+      <c r="R139" s="39"/>
+      <c r="S139" s="39"/>
+      <c r="T139" s="39"/>
+      <c r="U139" s="39"/>
+      <c r="V139" s="39"/>
+      <c r="W139" s="39"/>
+      <c r="X139" s="39"/>
+      <c r="Y139" s="39"/>
+      <c r="Z139" s="39"/>
+      <c r="AA139" s="39"/>
+      <c r="AB139" s="40"/>
       <c r="AC139" s="11"/>
     </row>
     <row r="140" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6243,27 +6260,27 @@
         <v>2</v>
       </c>
       <c r="G144" s="6"/>
-      <c r="H144" s="48"/>
-      <c r="I144" s="49"/>
-      <c r="J144" s="49"/>
-      <c r="K144" s="49"/>
-      <c r="L144" s="49"/>
-      <c r="M144" s="49"/>
-      <c r="N144" s="49"/>
-      <c r="O144" s="49"/>
-      <c r="P144" s="49"/>
-      <c r="Q144" s="49"/>
-      <c r="R144" s="49"/>
-      <c r="S144" s="49"/>
-      <c r="T144" s="49"/>
-      <c r="U144" s="49"/>
-      <c r="V144" s="49"/>
-      <c r="W144" s="49"/>
-      <c r="X144" s="49"/>
-      <c r="Y144" s="49"/>
-      <c r="Z144" s="49"/>
-      <c r="AA144" s="49"/>
-      <c r="AB144" s="50"/>
+      <c r="H144" s="46"/>
+      <c r="I144" s="47"/>
+      <c r="J144" s="47"/>
+      <c r="K144" s="47"/>
+      <c r="L144" s="47"/>
+      <c r="M144" s="47"/>
+      <c r="N144" s="47"/>
+      <c r="O144" s="47"/>
+      <c r="P144" s="47"/>
+      <c r="Q144" s="47"/>
+      <c r="R144" s="47"/>
+      <c r="S144" s="47"/>
+      <c r="T144" s="47"/>
+      <c r="U144" s="47"/>
+      <c r="V144" s="47"/>
+      <c r="W144" s="47"/>
+      <c r="X144" s="47"/>
+      <c r="Y144" s="47"/>
+      <c r="Z144" s="47"/>
+      <c r="AA144" s="47"/>
+      <c r="AB144" s="48"/>
       <c r="AC144" s="11"/>
     </row>
     <row r="145" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6273,27 +6290,27 @@
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
       <c r="G145" s="6"/>
-      <c r="H145" s="51"/>
-      <c r="I145" s="52"/>
-      <c r="J145" s="52"/>
-      <c r="K145" s="52"/>
-      <c r="L145" s="52"/>
-      <c r="M145" s="52"/>
-      <c r="N145" s="52"/>
-      <c r="O145" s="52"/>
-      <c r="P145" s="52"/>
-      <c r="Q145" s="52"/>
-      <c r="R145" s="52"/>
-      <c r="S145" s="52"/>
-      <c r="T145" s="52"/>
-      <c r="U145" s="52"/>
-      <c r="V145" s="52"/>
-      <c r="W145" s="52"/>
-      <c r="X145" s="52"/>
-      <c r="Y145" s="52"/>
-      <c r="Z145" s="52"/>
-      <c r="AA145" s="52"/>
-      <c r="AB145" s="53"/>
+      <c r="H145" s="49"/>
+      <c r="I145" s="50"/>
+      <c r="J145" s="50"/>
+      <c r="K145" s="50"/>
+      <c r="L145" s="50"/>
+      <c r="M145" s="50"/>
+      <c r="N145" s="50"/>
+      <c r="O145" s="50"/>
+      <c r="P145" s="50"/>
+      <c r="Q145" s="50"/>
+      <c r="R145" s="50"/>
+      <c r="S145" s="50"/>
+      <c r="T145" s="50"/>
+      <c r="U145" s="50"/>
+      <c r="V145" s="50"/>
+      <c r="W145" s="50"/>
+      <c r="X145" s="50"/>
+      <c r="Y145" s="50"/>
+      <c r="Z145" s="50"/>
+      <c r="AA145" s="50"/>
+      <c r="AB145" s="51"/>
       <c r="AC145" s="11"/>
     </row>
     <row r="146" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6303,27 +6320,27 @@
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
       <c r="G146" s="6"/>
-      <c r="H146" s="51"/>
-      <c r="I146" s="52"/>
-      <c r="J146" s="52"/>
-      <c r="K146" s="52"/>
-      <c r="L146" s="52"/>
-      <c r="M146" s="52"/>
-      <c r="N146" s="52"/>
-      <c r="O146" s="52"/>
-      <c r="P146" s="52"/>
-      <c r="Q146" s="52"/>
-      <c r="R146" s="52"/>
-      <c r="S146" s="52"/>
-      <c r="T146" s="52"/>
-      <c r="U146" s="52"/>
-      <c r="V146" s="52"/>
-      <c r="W146" s="52"/>
-      <c r="X146" s="52"/>
-      <c r="Y146" s="52"/>
-      <c r="Z146" s="52"/>
-      <c r="AA146" s="52"/>
-      <c r="AB146" s="53"/>
+      <c r="H146" s="49"/>
+      <c r="I146" s="50"/>
+      <c r="J146" s="50"/>
+      <c r="K146" s="50"/>
+      <c r="L146" s="50"/>
+      <c r="M146" s="50"/>
+      <c r="N146" s="50"/>
+      <c r="O146" s="50"/>
+      <c r="P146" s="50"/>
+      <c r="Q146" s="50"/>
+      <c r="R146" s="50"/>
+      <c r="S146" s="50"/>
+      <c r="T146" s="50"/>
+      <c r="U146" s="50"/>
+      <c r="V146" s="50"/>
+      <c r="W146" s="50"/>
+      <c r="X146" s="50"/>
+      <c r="Y146" s="50"/>
+      <c r="Z146" s="50"/>
+      <c r="AA146" s="50"/>
+      <c r="AB146" s="51"/>
       <c r="AC146" s="11"/>
     </row>
     <row r="147" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6333,27 +6350,27 @@
       <c r="E147" s="6"/>
       <c r="F147" s="6"/>
       <c r="G147" s="6"/>
-      <c r="H147" s="51"/>
-      <c r="I147" s="52"/>
-      <c r="J147" s="52"/>
-      <c r="K147" s="52"/>
-      <c r="L147" s="52"/>
-      <c r="M147" s="52"/>
-      <c r="N147" s="52"/>
-      <c r="O147" s="52"/>
-      <c r="P147" s="52"/>
-      <c r="Q147" s="52"/>
-      <c r="R147" s="52"/>
-      <c r="S147" s="52"/>
-      <c r="T147" s="52"/>
-      <c r="U147" s="52"/>
-      <c r="V147" s="52"/>
-      <c r="W147" s="52"/>
-      <c r="X147" s="52"/>
-      <c r="Y147" s="52"/>
-      <c r="Z147" s="52"/>
-      <c r="AA147" s="52"/>
-      <c r="AB147" s="53"/>
+      <c r="H147" s="49"/>
+      <c r="I147" s="50"/>
+      <c r="J147" s="50"/>
+      <c r="K147" s="50"/>
+      <c r="L147" s="50"/>
+      <c r="M147" s="50"/>
+      <c r="N147" s="50"/>
+      <c r="O147" s="50"/>
+      <c r="P147" s="50"/>
+      <c r="Q147" s="50"/>
+      <c r="R147" s="50"/>
+      <c r="S147" s="50"/>
+      <c r="T147" s="50"/>
+      <c r="U147" s="50"/>
+      <c r="V147" s="50"/>
+      <c r="W147" s="50"/>
+      <c r="X147" s="50"/>
+      <c r="Y147" s="50"/>
+      <c r="Z147" s="50"/>
+      <c r="AA147" s="50"/>
+      <c r="AB147" s="51"/>
       <c r="AC147" s="11"/>
     </row>
     <row r="148" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6363,27 +6380,27 @@
       <c r="E148" s="6"/>
       <c r="F148" s="6"/>
       <c r="G148" s="6"/>
-      <c r="H148" s="51"/>
-      <c r="I148" s="52"/>
-      <c r="J148" s="52"/>
-      <c r="K148" s="52"/>
-      <c r="L148" s="52"/>
-      <c r="M148" s="52"/>
-      <c r="N148" s="52"/>
-      <c r="O148" s="52"/>
-      <c r="P148" s="52"/>
-      <c r="Q148" s="52"/>
-      <c r="R148" s="52"/>
-      <c r="S148" s="52"/>
-      <c r="T148" s="52"/>
-      <c r="U148" s="52"/>
-      <c r="V148" s="52"/>
-      <c r="W148" s="52"/>
-      <c r="X148" s="52"/>
-      <c r="Y148" s="52"/>
-      <c r="Z148" s="52"/>
-      <c r="AA148" s="52"/>
-      <c r="AB148" s="53"/>
+      <c r="H148" s="49"/>
+      <c r="I148" s="50"/>
+      <c r="J148" s="50"/>
+      <c r="K148" s="50"/>
+      <c r="L148" s="50"/>
+      <c r="M148" s="50"/>
+      <c r="N148" s="50"/>
+      <c r="O148" s="50"/>
+      <c r="P148" s="50"/>
+      <c r="Q148" s="50"/>
+      <c r="R148" s="50"/>
+      <c r="S148" s="50"/>
+      <c r="T148" s="50"/>
+      <c r="U148" s="50"/>
+      <c r="V148" s="50"/>
+      <c r="W148" s="50"/>
+      <c r="X148" s="50"/>
+      <c r="Y148" s="50"/>
+      <c r="Z148" s="50"/>
+      <c r="AA148" s="50"/>
+      <c r="AB148" s="51"/>
       <c r="AC148" s="11"/>
     </row>
     <row r="149" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6393,27 +6410,27 @@
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
       <c r="G149" s="6"/>
-      <c r="H149" s="51"/>
-      <c r="I149" s="52"/>
-      <c r="J149" s="52"/>
-      <c r="K149" s="52"/>
-      <c r="L149" s="52"/>
-      <c r="M149" s="52"/>
-      <c r="N149" s="52"/>
-      <c r="O149" s="52"/>
-      <c r="P149" s="52"/>
-      <c r="Q149" s="52"/>
-      <c r="R149" s="52"/>
-      <c r="S149" s="52"/>
-      <c r="T149" s="52"/>
-      <c r="U149" s="52"/>
-      <c r="V149" s="52"/>
-      <c r="W149" s="52"/>
-      <c r="X149" s="52"/>
-      <c r="Y149" s="52"/>
-      <c r="Z149" s="52"/>
-      <c r="AA149" s="52"/>
-      <c r="AB149" s="53"/>
+      <c r="H149" s="49"/>
+      <c r="I149" s="50"/>
+      <c r="J149" s="50"/>
+      <c r="K149" s="50"/>
+      <c r="L149" s="50"/>
+      <c r="M149" s="50"/>
+      <c r="N149" s="50"/>
+      <c r="O149" s="50"/>
+      <c r="P149" s="50"/>
+      <c r="Q149" s="50"/>
+      <c r="R149" s="50"/>
+      <c r="S149" s="50"/>
+      <c r="T149" s="50"/>
+      <c r="U149" s="50"/>
+      <c r="V149" s="50"/>
+      <c r="W149" s="50"/>
+      <c r="X149" s="50"/>
+      <c r="Y149" s="50"/>
+      <c r="Z149" s="50"/>
+      <c r="AA149" s="50"/>
+      <c r="AB149" s="51"/>
       <c r="AC149" s="11"/>
     </row>
     <row r="150" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6423,27 +6440,27 @@
       <c r="E150" s="6"/>
       <c r="F150" s="6"/>
       <c r="G150" s="6"/>
-      <c r="H150" s="54"/>
-      <c r="I150" s="55"/>
-      <c r="J150" s="55"/>
-      <c r="K150" s="55"/>
-      <c r="L150" s="55"/>
-      <c r="M150" s="55"/>
-      <c r="N150" s="55"/>
-      <c r="O150" s="55"/>
-      <c r="P150" s="55"/>
-      <c r="Q150" s="55"/>
-      <c r="R150" s="55"/>
-      <c r="S150" s="55"/>
-      <c r="T150" s="55"/>
-      <c r="U150" s="55"/>
-      <c r="V150" s="55"/>
-      <c r="W150" s="55"/>
-      <c r="X150" s="55"/>
-      <c r="Y150" s="55"/>
-      <c r="Z150" s="55"/>
-      <c r="AA150" s="55"/>
-      <c r="AB150" s="56"/>
+      <c r="H150" s="52"/>
+      <c r="I150" s="53"/>
+      <c r="J150" s="53"/>
+      <c r="K150" s="53"/>
+      <c r="L150" s="53"/>
+      <c r="M150" s="53"/>
+      <c r="N150" s="53"/>
+      <c r="O150" s="53"/>
+      <c r="P150" s="53"/>
+      <c r="Q150" s="53"/>
+      <c r="R150" s="53"/>
+      <c r="S150" s="53"/>
+      <c r="T150" s="53"/>
+      <c r="U150" s="53"/>
+      <c r="V150" s="53"/>
+      <c r="W150" s="53"/>
+      <c r="X150" s="53"/>
+      <c r="Y150" s="53"/>
+      <c r="Z150" s="53"/>
+      <c r="AA150" s="53"/>
+      <c r="AB150" s="54"/>
       <c r="AC150" s="11"/>
     </row>
     <row r="151" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6485,27 +6502,27 @@
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6"/>
-      <c r="H152" s="48"/>
-      <c r="I152" s="49"/>
-      <c r="J152" s="49"/>
-      <c r="K152" s="49"/>
-      <c r="L152" s="49"/>
-      <c r="M152" s="49"/>
-      <c r="N152" s="49"/>
-      <c r="O152" s="49"/>
-      <c r="P152" s="49"/>
-      <c r="Q152" s="49"/>
-      <c r="R152" s="49"/>
-      <c r="S152" s="49"/>
-      <c r="T152" s="49"/>
-      <c r="U152" s="49"/>
-      <c r="V152" s="49"/>
-      <c r="W152" s="49"/>
-      <c r="X152" s="49"/>
-      <c r="Y152" s="49"/>
-      <c r="Z152" s="49"/>
-      <c r="AA152" s="49"/>
-      <c r="AB152" s="50"/>
+      <c r="H152" s="46"/>
+      <c r="I152" s="47"/>
+      <c r="J152" s="47"/>
+      <c r="K152" s="47"/>
+      <c r="L152" s="47"/>
+      <c r="M152" s="47"/>
+      <c r="N152" s="47"/>
+      <c r="O152" s="47"/>
+      <c r="P152" s="47"/>
+      <c r="Q152" s="47"/>
+      <c r="R152" s="47"/>
+      <c r="S152" s="47"/>
+      <c r="T152" s="47"/>
+      <c r="U152" s="47"/>
+      <c r="V152" s="47"/>
+      <c r="W152" s="47"/>
+      <c r="X152" s="47"/>
+      <c r="Y152" s="47"/>
+      <c r="Z152" s="47"/>
+      <c r="AA152" s="47"/>
+      <c r="AB152" s="48"/>
       <c r="AC152" s="11"/>
     </row>
     <row r="153" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6515,27 +6532,27 @@
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
       <c r="G153" s="6"/>
-      <c r="H153" s="51"/>
-      <c r="I153" s="52"/>
-      <c r="J153" s="52"/>
-      <c r="K153" s="52"/>
-      <c r="L153" s="52"/>
-      <c r="M153" s="52"/>
-      <c r="N153" s="52"/>
-      <c r="O153" s="52"/>
-      <c r="P153" s="52"/>
-      <c r="Q153" s="52"/>
-      <c r="R153" s="52"/>
-      <c r="S153" s="52"/>
-      <c r="T153" s="52"/>
-      <c r="U153" s="52"/>
-      <c r="V153" s="52"/>
-      <c r="W153" s="52"/>
-      <c r="X153" s="52"/>
-      <c r="Y153" s="52"/>
-      <c r="Z153" s="52"/>
-      <c r="AA153" s="52"/>
-      <c r="AB153" s="53"/>
+      <c r="H153" s="49"/>
+      <c r="I153" s="50"/>
+      <c r="J153" s="50"/>
+      <c r="K153" s="50"/>
+      <c r="L153" s="50"/>
+      <c r="M153" s="50"/>
+      <c r="N153" s="50"/>
+      <c r="O153" s="50"/>
+      <c r="P153" s="50"/>
+      <c r="Q153" s="50"/>
+      <c r="R153" s="50"/>
+      <c r="S153" s="50"/>
+      <c r="T153" s="50"/>
+      <c r="U153" s="50"/>
+      <c r="V153" s="50"/>
+      <c r="W153" s="50"/>
+      <c r="X153" s="50"/>
+      <c r="Y153" s="50"/>
+      <c r="Z153" s="50"/>
+      <c r="AA153" s="50"/>
+      <c r="AB153" s="51"/>
       <c r="AC153" s="11"/>
     </row>
     <row r="154" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6545,27 +6562,27 @@
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
       <c r="G154" s="6"/>
-      <c r="H154" s="51"/>
-      <c r="I154" s="52"/>
-      <c r="J154" s="52"/>
-      <c r="K154" s="52"/>
-      <c r="L154" s="52"/>
-      <c r="M154" s="52"/>
-      <c r="N154" s="52"/>
-      <c r="O154" s="52"/>
-      <c r="P154" s="52"/>
-      <c r="Q154" s="52"/>
-      <c r="R154" s="52"/>
-      <c r="S154" s="52"/>
-      <c r="T154" s="52"/>
-      <c r="U154" s="52"/>
-      <c r="V154" s="52"/>
-      <c r="W154" s="52"/>
-      <c r="X154" s="52"/>
-      <c r="Y154" s="52"/>
-      <c r="Z154" s="52"/>
-      <c r="AA154" s="52"/>
-      <c r="AB154" s="53"/>
+      <c r="H154" s="49"/>
+      <c r="I154" s="50"/>
+      <c r="J154" s="50"/>
+      <c r="K154" s="50"/>
+      <c r="L154" s="50"/>
+      <c r="M154" s="50"/>
+      <c r="N154" s="50"/>
+      <c r="O154" s="50"/>
+      <c r="P154" s="50"/>
+      <c r="Q154" s="50"/>
+      <c r="R154" s="50"/>
+      <c r="S154" s="50"/>
+      <c r="T154" s="50"/>
+      <c r="U154" s="50"/>
+      <c r="V154" s="50"/>
+      <c r="W154" s="50"/>
+      <c r="X154" s="50"/>
+      <c r="Y154" s="50"/>
+      <c r="Z154" s="50"/>
+      <c r="AA154" s="50"/>
+      <c r="AB154" s="51"/>
       <c r="AC154" s="11"/>
     </row>
     <row r="155" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6575,27 +6592,27 @@
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
       <c r="G155" s="6"/>
-      <c r="H155" s="51"/>
-      <c r="I155" s="52"/>
-      <c r="J155" s="52"/>
-      <c r="K155" s="52"/>
-      <c r="L155" s="52"/>
-      <c r="M155" s="52"/>
-      <c r="N155" s="52"/>
-      <c r="O155" s="52"/>
-      <c r="P155" s="52"/>
-      <c r="Q155" s="52"/>
-      <c r="R155" s="52"/>
-      <c r="S155" s="52"/>
-      <c r="T155" s="52"/>
-      <c r="U155" s="52"/>
-      <c r="V155" s="52"/>
-      <c r="W155" s="52"/>
-      <c r="X155" s="52"/>
-      <c r="Y155" s="52"/>
-      <c r="Z155" s="52"/>
-      <c r="AA155" s="52"/>
-      <c r="AB155" s="53"/>
+      <c r="H155" s="49"/>
+      <c r="I155" s="50"/>
+      <c r="J155" s="50"/>
+      <c r="K155" s="50"/>
+      <c r="L155" s="50"/>
+      <c r="M155" s="50"/>
+      <c r="N155" s="50"/>
+      <c r="O155" s="50"/>
+      <c r="P155" s="50"/>
+      <c r="Q155" s="50"/>
+      <c r="R155" s="50"/>
+      <c r="S155" s="50"/>
+      <c r="T155" s="50"/>
+      <c r="U155" s="50"/>
+      <c r="V155" s="50"/>
+      <c r="W155" s="50"/>
+      <c r="X155" s="50"/>
+      <c r="Y155" s="50"/>
+      <c r="Z155" s="50"/>
+      <c r="AA155" s="50"/>
+      <c r="AB155" s="51"/>
       <c r="AC155" s="11"/>
     </row>
     <row r="156" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6605,27 +6622,27 @@
       <c r="E156" s="6"/>
       <c r="F156" s="6"/>
       <c r="G156" s="6"/>
-      <c r="H156" s="51"/>
-      <c r="I156" s="52"/>
-      <c r="J156" s="52"/>
-      <c r="K156" s="52"/>
-      <c r="L156" s="52"/>
-      <c r="M156" s="52"/>
-      <c r="N156" s="52"/>
-      <c r="O156" s="52"/>
-      <c r="P156" s="52"/>
-      <c r="Q156" s="52"/>
-      <c r="R156" s="52"/>
-      <c r="S156" s="52"/>
-      <c r="T156" s="52"/>
-      <c r="U156" s="52"/>
-      <c r="V156" s="52"/>
-      <c r="W156" s="52"/>
-      <c r="X156" s="52"/>
-      <c r="Y156" s="52"/>
-      <c r="Z156" s="52"/>
-      <c r="AA156" s="52"/>
-      <c r="AB156" s="53"/>
+      <c r="H156" s="49"/>
+      <c r="I156" s="50"/>
+      <c r="J156" s="50"/>
+      <c r="K156" s="50"/>
+      <c r="L156" s="50"/>
+      <c r="M156" s="50"/>
+      <c r="N156" s="50"/>
+      <c r="O156" s="50"/>
+      <c r="P156" s="50"/>
+      <c r="Q156" s="50"/>
+      <c r="R156" s="50"/>
+      <c r="S156" s="50"/>
+      <c r="T156" s="50"/>
+      <c r="U156" s="50"/>
+      <c r="V156" s="50"/>
+      <c r="W156" s="50"/>
+      <c r="X156" s="50"/>
+      <c r="Y156" s="50"/>
+      <c r="Z156" s="50"/>
+      <c r="AA156" s="50"/>
+      <c r="AB156" s="51"/>
       <c r="AC156" s="11"/>
     </row>
     <row r="157" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6635,27 +6652,27 @@
       <c r="E157" s="6"/>
       <c r="F157" s="6"/>
       <c r="G157" s="6"/>
-      <c r="H157" s="51"/>
-      <c r="I157" s="52"/>
-      <c r="J157" s="52"/>
-      <c r="K157" s="52"/>
-      <c r="L157" s="52"/>
-      <c r="M157" s="52"/>
-      <c r="N157" s="52"/>
-      <c r="O157" s="52"/>
-      <c r="P157" s="52"/>
-      <c r="Q157" s="52"/>
-      <c r="R157" s="52"/>
-      <c r="S157" s="52"/>
-      <c r="T157" s="52"/>
-      <c r="U157" s="52"/>
-      <c r="V157" s="52"/>
-      <c r="W157" s="52"/>
-      <c r="X157" s="52"/>
-      <c r="Y157" s="52"/>
-      <c r="Z157" s="52"/>
-      <c r="AA157" s="52"/>
-      <c r="AB157" s="53"/>
+      <c r="H157" s="49"/>
+      <c r="I157" s="50"/>
+      <c r="J157" s="50"/>
+      <c r="K157" s="50"/>
+      <c r="L157" s="50"/>
+      <c r="M157" s="50"/>
+      <c r="N157" s="50"/>
+      <c r="O157" s="50"/>
+      <c r="P157" s="50"/>
+      <c r="Q157" s="50"/>
+      <c r="R157" s="50"/>
+      <c r="S157" s="50"/>
+      <c r="T157" s="50"/>
+      <c r="U157" s="50"/>
+      <c r="V157" s="50"/>
+      <c r="W157" s="50"/>
+      <c r="X157" s="50"/>
+      <c r="Y157" s="50"/>
+      <c r="Z157" s="50"/>
+      <c r="AA157" s="50"/>
+      <c r="AB157" s="51"/>
       <c r="AC157" s="11"/>
     </row>
     <row r="158" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6665,27 +6682,27 @@
       <c r="E158" s="6"/>
       <c r="F158" s="6"/>
       <c r="G158" s="6"/>
-      <c r="H158" s="54"/>
-      <c r="I158" s="55"/>
-      <c r="J158" s="55"/>
-      <c r="K158" s="55"/>
-      <c r="L158" s="55"/>
-      <c r="M158" s="55"/>
-      <c r="N158" s="55"/>
-      <c r="O158" s="55"/>
-      <c r="P158" s="55"/>
-      <c r="Q158" s="55"/>
-      <c r="R158" s="55"/>
-      <c r="S158" s="55"/>
-      <c r="T158" s="55"/>
-      <c r="U158" s="55"/>
-      <c r="V158" s="55"/>
-      <c r="W158" s="55"/>
-      <c r="X158" s="55"/>
-      <c r="Y158" s="55"/>
-      <c r="Z158" s="55"/>
-      <c r="AA158" s="55"/>
-      <c r="AB158" s="56"/>
+      <c r="H158" s="52"/>
+      <c r="I158" s="53"/>
+      <c r="J158" s="53"/>
+      <c r="K158" s="53"/>
+      <c r="L158" s="53"/>
+      <c r="M158" s="53"/>
+      <c r="N158" s="53"/>
+      <c r="O158" s="53"/>
+      <c r="P158" s="53"/>
+      <c r="Q158" s="53"/>
+      <c r="R158" s="53"/>
+      <c r="S158" s="53"/>
+      <c r="T158" s="53"/>
+      <c r="U158" s="53"/>
+      <c r="V158" s="53"/>
+      <c r="W158" s="53"/>
+      <c r="X158" s="53"/>
+      <c r="Y158" s="53"/>
+      <c r="Z158" s="53"/>
+      <c r="AA158" s="53"/>
+      <c r="AB158" s="54"/>
       <c r="AC158" s="11"/>
     </row>
     <row r="159" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6793,27 +6810,27 @@
         <v>2</v>
       </c>
       <c r="G163" s="6"/>
-      <c r="H163" s="48"/>
-      <c r="I163" s="49"/>
-      <c r="J163" s="49"/>
-      <c r="K163" s="49"/>
-      <c r="L163" s="49"/>
-      <c r="M163" s="49"/>
-      <c r="N163" s="49"/>
-      <c r="O163" s="49"/>
-      <c r="P163" s="49"/>
-      <c r="Q163" s="49"/>
-      <c r="R163" s="49"/>
-      <c r="S163" s="49"/>
-      <c r="T163" s="49"/>
-      <c r="U163" s="49"/>
-      <c r="V163" s="49"/>
-      <c r="W163" s="49"/>
-      <c r="X163" s="49"/>
-      <c r="Y163" s="49"/>
-      <c r="Z163" s="49"/>
-      <c r="AA163" s="49"/>
-      <c r="AB163" s="50"/>
+      <c r="H163" s="46"/>
+      <c r="I163" s="47"/>
+      <c r="J163" s="47"/>
+      <c r="K163" s="47"/>
+      <c r="L163" s="47"/>
+      <c r="M163" s="47"/>
+      <c r="N163" s="47"/>
+      <c r="O163" s="47"/>
+      <c r="P163" s="47"/>
+      <c r="Q163" s="47"/>
+      <c r="R163" s="47"/>
+      <c r="S163" s="47"/>
+      <c r="T163" s="47"/>
+      <c r="U163" s="47"/>
+      <c r="V163" s="47"/>
+      <c r="W163" s="47"/>
+      <c r="X163" s="47"/>
+      <c r="Y163" s="47"/>
+      <c r="Z163" s="47"/>
+      <c r="AA163" s="47"/>
+      <c r="AB163" s="48"/>
       <c r="AC163" s="11"/>
     </row>
     <row r="164" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6823,27 +6840,27 @@
       <c r="E164" s="6"/>
       <c r="F164" s="6"/>
       <c r="G164" s="6"/>
-      <c r="H164" s="51"/>
-      <c r="I164" s="52"/>
-      <c r="J164" s="52"/>
-      <c r="K164" s="52"/>
-      <c r="L164" s="52"/>
-      <c r="M164" s="52"/>
-      <c r="N164" s="52"/>
-      <c r="O164" s="52"/>
-      <c r="P164" s="52"/>
-      <c r="Q164" s="52"/>
-      <c r="R164" s="52"/>
-      <c r="S164" s="52"/>
-      <c r="T164" s="52"/>
-      <c r="U164" s="52"/>
-      <c r="V164" s="52"/>
-      <c r="W164" s="52"/>
-      <c r="X164" s="52"/>
-      <c r="Y164" s="52"/>
-      <c r="Z164" s="52"/>
-      <c r="AA164" s="52"/>
-      <c r="AB164" s="53"/>
+      <c r="H164" s="49"/>
+      <c r="I164" s="50"/>
+      <c r="J164" s="50"/>
+      <c r="K164" s="50"/>
+      <c r="L164" s="50"/>
+      <c r="M164" s="50"/>
+      <c r="N164" s="50"/>
+      <c r="O164" s="50"/>
+      <c r="P164" s="50"/>
+      <c r="Q164" s="50"/>
+      <c r="R164" s="50"/>
+      <c r="S164" s="50"/>
+      <c r="T164" s="50"/>
+      <c r="U164" s="50"/>
+      <c r="V164" s="50"/>
+      <c r="W164" s="50"/>
+      <c r="X164" s="50"/>
+      <c r="Y164" s="50"/>
+      <c r="Z164" s="50"/>
+      <c r="AA164" s="50"/>
+      <c r="AB164" s="51"/>
       <c r="AC164" s="11"/>
     </row>
     <row r="165" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6853,27 +6870,27 @@
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
       <c r="G165" s="6"/>
-      <c r="H165" s="51"/>
-      <c r="I165" s="52"/>
-      <c r="J165" s="52"/>
-      <c r="K165" s="52"/>
-      <c r="L165" s="52"/>
-      <c r="M165" s="52"/>
-      <c r="N165" s="52"/>
-      <c r="O165" s="52"/>
-      <c r="P165" s="52"/>
-      <c r="Q165" s="52"/>
-      <c r="R165" s="52"/>
-      <c r="S165" s="52"/>
-      <c r="T165" s="52"/>
-      <c r="U165" s="52"/>
-      <c r="V165" s="52"/>
-      <c r="W165" s="52"/>
-      <c r="X165" s="52"/>
-      <c r="Y165" s="52"/>
-      <c r="Z165" s="52"/>
-      <c r="AA165" s="52"/>
-      <c r="AB165" s="53"/>
+      <c r="H165" s="49"/>
+      <c r="I165" s="50"/>
+      <c r="J165" s="50"/>
+      <c r="K165" s="50"/>
+      <c r="L165" s="50"/>
+      <c r="M165" s="50"/>
+      <c r="N165" s="50"/>
+      <c r="O165" s="50"/>
+      <c r="P165" s="50"/>
+      <c r="Q165" s="50"/>
+      <c r="R165" s="50"/>
+      <c r="S165" s="50"/>
+      <c r="T165" s="50"/>
+      <c r="U165" s="50"/>
+      <c r="V165" s="50"/>
+      <c r="W165" s="50"/>
+      <c r="X165" s="50"/>
+      <c r="Y165" s="50"/>
+      <c r="Z165" s="50"/>
+      <c r="AA165" s="50"/>
+      <c r="AB165" s="51"/>
       <c r="AC165" s="11"/>
     </row>
     <row r="166" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6883,27 +6900,27 @@
       <c r="E166" s="6"/>
       <c r="F166" s="6"/>
       <c r="G166" s="6"/>
-      <c r="H166" s="51"/>
-      <c r="I166" s="52"/>
-      <c r="J166" s="52"/>
-      <c r="K166" s="52"/>
-      <c r="L166" s="52"/>
-      <c r="M166" s="52"/>
-      <c r="N166" s="52"/>
-      <c r="O166" s="52"/>
-      <c r="P166" s="52"/>
-      <c r="Q166" s="52"/>
-      <c r="R166" s="52"/>
-      <c r="S166" s="52"/>
-      <c r="T166" s="52"/>
-      <c r="U166" s="52"/>
-      <c r="V166" s="52"/>
-      <c r="W166" s="52"/>
-      <c r="X166" s="52"/>
-      <c r="Y166" s="52"/>
-      <c r="Z166" s="52"/>
-      <c r="AA166" s="52"/>
-      <c r="AB166" s="53"/>
+      <c r="H166" s="49"/>
+      <c r="I166" s="50"/>
+      <c r="J166" s="50"/>
+      <c r="K166" s="50"/>
+      <c r="L166" s="50"/>
+      <c r="M166" s="50"/>
+      <c r="N166" s="50"/>
+      <c r="O166" s="50"/>
+      <c r="P166" s="50"/>
+      <c r="Q166" s="50"/>
+      <c r="R166" s="50"/>
+      <c r="S166" s="50"/>
+      <c r="T166" s="50"/>
+      <c r="U166" s="50"/>
+      <c r="V166" s="50"/>
+      <c r="W166" s="50"/>
+      <c r="X166" s="50"/>
+      <c r="Y166" s="50"/>
+      <c r="Z166" s="50"/>
+      <c r="AA166" s="50"/>
+      <c r="AB166" s="51"/>
       <c r="AC166" s="11"/>
     </row>
     <row r="167" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6913,27 +6930,27 @@
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
       <c r="G167" s="6"/>
-      <c r="H167" s="51"/>
-      <c r="I167" s="52"/>
-      <c r="J167" s="52"/>
-      <c r="K167" s="52"/>
-      <c r="L167" s="52"/>
-      <c r="M167" s="52"/>
-      <c r="N167" s="52"/>
-      <c r="O167" s="52"/>
-      <c r="P167" s="52"/>
-      <c r="Q167" s="52"/>
-      <c r="R167" s="52"/>
-      <c r="S167" s="52"/>
-      <c r="T167" s="52"/>
-      <c r="U167" s="52"/>
-      <c r="V167" s="52"/>
-      <c r="W167" s="52"/>
-      <c r="X167" s="52"/>
-      <c r="Y167" s="52"/>
-      <c r="Z167" s="52"/>
-      <c r="AA167" s="52"/>
-      <c r="AB167" s="53"/>
+      <c r="H167" s="49"/>
+      <c r="I167" s="50"/>
+      <c r="J167" s="50"/>
+      <c r="K167" s="50"/>
+      <c r="L167" s="50"/>
+      <c r="M167" s="50"/>
+      <c r="N167" s="50"/>
+      <c r="O167" s="50"/>
+      <c r="P167" s="50"/>
+      <c r="Q167" s="50"/>
+      <c r="R167" s="50"/>
+      <c r="S167" s="50"/>
+      <c r="T167" s="50"/>
+      <c r="U167" s="50"/>
+      <c r="V167" s="50"/>
+      <c r="W167" s="50"/>
+      <c r="X167" s="50"/>
+      <c r="Y167" s="50"/>
+      <c r="Z167" s="50"/>
+      <c r="AA167" s="50"/>
+      <c r="AB167" s="51"/>
       <c r="AC167" s="11"/>
     </row>
     <row r="168" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6943,27 +6960,27 @@
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
       <c r="G168" s="6"/>
-      <c r="H168" s="51"/>
-      <c r="I168" s="52"/>
-      <c r="J168" s="52"/>
-      <c r="K168" s="52"/>
-      <c r="L168" s="52"/>
-      <c r="M168" s="52"/>
-      <c r="N168" s="52"/>
-      <c r="O168" s="52"/>
-      <c r="P168" s="52"/>
-      <c r="Q168" s="52"/>
-      <c r="R168" s="52"/>
-      <c r="S168" s="52"/>
-      <c r="T168" s="52"/>
-      <c r="U168" s="52"/>
-      <c r="V168" s="52"/>
-      <c r="W168" s="52"/>
-      <c r="X168" s="52"/>
-      <c r="Y168" s="52"/>
-      <c r="Z168" s="52"/>
-      <c r="AA168" s="52"/>
-      <c r="AB168" s="53"/>
+      <c r="H168" s="49"/>
+      <c r="I168" s="50"/>
+      <c r="J168" s="50"/>
+      <c r="K168" s="50"/>
+      <c r="L168" s="50"/>
+      <c r="M168" s="50"/>
+      <c r="N168" s="50"/>
+      <c r="O168" s="50"/>
+      <c r="P168" s="50"/>
+      <c r="Q168" s="50"/>
+      <c r="R168" s="50"/>
+      <c r="S168" s="50"/>
+      <c r="T168" s="50"/>
+      <c r="U168" s="50"/>
+      <c r="V168" s="50"/>
+      <c r="W168" s="50"/>
+      <c r="X168" s="50"/>
+      <c r="Y168" s="50"/>
+      <c r="Z168" s="50"/>
+      <c r="AA168" s="50"/>
+      <c r="AB168" s="51"/>
       <c r="AC168" s="11"/>
     </row>
     <row r="169" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6973,27 +6990,27 @@
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
-      <c r="H169" s="54"/>
-      <c r="I169" s="55"/>
-      <c r="J169" s="55"/>
-      <c r="K169" s="55"/>
-      <c r="L169" s="55"/>
-      <c r="M169" s="55"/>
-      <c r="N169" s="55"/>
-      <c r="O169" s="55"/>
-      <c r="P169" s="55"/>
-      <c r="Q169" s="55"/>
-      <c r="R169" s="55"/>
-      <c r="S169" s="55"/>
-      <c r="T169" s="55"/>
-      <c r="U169" s="55"/>
-      <c r="V169" s="55"/>
-      <c r="W169" s="55"/>
-      <c r="X169" s="55"/>
-      <c r="Y169" s="55"/>
-      <c r="Z169" s="55"/>
-      <c r="AA169" s="55"/>
-      <c r="AB169" s="56"/>
+      <c r="H169" s="52"/>
+      <c r="I169" s="53"/>
+      <c r="J169" s="53"/>
+      <c r="K169" s="53"/>
+      <c r="L169" s="53"/>
+      <c r="M169" s="53"/>
+      <c r="N169" s="53"/>
+      <c r="O169" s="53"/>
+      <c r="P169" s="53"/>
+      <c r="Q169" s="53"/>
+      <c r="R169" s="53"/>
+      <c r="S169" s="53"/>
+      <c r="T169" s="53"/>
+      <c r="U169" s="53"/>
+      <c r="V169" s="53"/>
+      <c r="W169" s="53"/>
+      <c r="X169" s="53"/>
+      <c r="Y169" s="53"/>
+      <c r="Z169" s="53"/>
+      <c r="AA169" s="53"/>
+      <c r="AB169" s="54"/>
       <c r="AC169" s="11"/>
     </row>
     <row r="170" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7035,27 +7052,27 @@
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
       <c r="G171" s="6"/>
-      <c r="H171" s="48"/>
-      <c r="I171" s="49"/>
-      <c r="J171" s="49"/>
-      <c r="K171" s="49"/>
-      <c r="L171" s="49"/>
-      <c r="M171" s="49"/>
-      <c r="N171" s="49"/>
-      <c r="O171" s="49"/>
-      <c r="P171" s="49"/>
-      <c r="Q171" s="49"/>
-      <c r="R171" s="49"/>
-      <c r="S171" s="49"/>
-      <c r="T171" s="49"/>
-      <c r="U171" s="49"/>
-      <c r="V171" s="49"/>
-      <c r="W171" s="49"/>
-      <c r="X171" s="49"/>
-      <c r="Y171" s="49"/>
-      <c r="Z171" s="49"/>
-      <c r="AA171" s="49"/>
-      <c r="AB171" s="50"/>
+      <c r="H171" s="46"/>
+      <c r="I171" s="47"/>
+      <c r="J171" s="47"/>
+      <c r="K171" s="47"/>
+      <c r="L171" s="47"/>
+      <c r="M171" s="47"/>
+      <c r="N171" s="47"/>
+      <c r="O171" s="47"/>
+      <c r="P171" s="47"/>
+      <c r="Q171" s="47"/>
+      <c r="R171" s="47"/>
+      <c r="S171" s="47"/>
+      <c r="T171" s="47"/>
+      <c r="U171" s="47"/>
+      <c r="V171" s="47"/>
+      <c r="W171" s="47"/>
+      <c r="X171" s="47"/>
+      <c r="Y171" s="47"/>
+      <c r="Z171" s="47"/>
+      <c r="AA171" s="47"/>
+      <c r="AB171" s="48"/>
       <c r="AC171" s="11"/>
     </row>
     <row r="172" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7065,27 +7082,27 @@
       <c r="E172" s="6"/>
       <c r="F172" s="6"/>
       <c r="G172" s="6"/>
-      <c r="H172" s="51"/>
-      <c r="I172" s="52"/>
-      <c r="J172" s="52"/>
-      <c r="K172" s="52"/>
-      <c r="L172" s="52"/>
-      <c r="M172" s="52"/>
-      <c r="N172" s="52"/>
-      <c r="O172" s="52"/>
-      <c r="P172" s="52"/>
-      <c r="Q172" s="52"/>
-      <c r="R172" s="52"/>
-      <c r="S172" s="52"/>
-      <c r="T172" s="52"/>
-      <c r="U172" s="52"/>
-      <c r="V172" s="52"/>
-      <c r="W172" s="52"/>
-      <c r="X172" s="52"/>
-      <c r="Y172" s="52"/>
-      <c r="Z172" s="52"/>
-      <c r="AA172" s="52"/>
-      <c r="AB172" s="53"/>
+      <c r="H172" s="49"/>
+      <c r="I172" s="50"/>
+      <c r="J172" s="50"/>
+      <c r="K172" s="50"/>
+      <c r="L172" s="50"/>
+      <c r="M172" s="50"/>
+      <c r="N172" s="50"/>
+      <c r="O172" s="50"/>
+      <c r="P172" s="50"/>
+      <c r="Q172" s="50"/>
+      <c r="R172" s="50"/>
+      <c r="S172" s="50"/>
+      <c r="T172" s="50"/>
+      <c r="U172" s="50"/>
+      <c r="V172" s="50"/>
+      <c r="W172" s="50"/>
+      <c r="X172" s="50"/>
+      <c r="Y172" s="50"/>
+      <c r="Z172" s="50"/>
+      <c r="AA172" s="50"/>
+      <c r="AB172" s="51"/>
       <c r="AC172" s="11"/>
     </row>
     <row r="173" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7095,27 +7112,27 @@
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6"/>
-      <c r="H173" s="51"/>
-      <c r="I173" s="52"/>
-      <c r="J173" s="52"/>
-      <c r="K173" s="52"/>
-      <c r="L173" s="52"/>
-      <c r="M173" s="52"/>
-      <c r="N173" s="52"/>
-      <c r="O173" s="52"/>
-      <c r="P173" s="52"/>
-      <c r="Q173" s="52"/>
-      <c r="R173" s="52"/>
-      <c r="S173" s="52"/>
-      <c r="T173" s="52"/>
-      <c r="U173" s="52"/>
-      <c r="V173" s="52"/>
-      <c r="W173" s="52"/>
-      <c r="X173" s="52"/>
-      <c r="Y173" s="52"/>
-      <c r="Z173" s="52"/>
-      <c r="AA173" s="52"/>
-      <c r="AB173" s="53"/>
+      <c r="H173" s="49"/>
+      <c r="I173" s="50"/>
+      <c r="J173" s="50"/>
+      <c r="K173" s="50"/>
+      <c r="L173" s="50"/>
+      <c r="M173" s="50"/>
+      <c r="N173" s="50"/>
+      <c r="O173" s="50"/>
+      <c r="P173" s="50"/>
+      <c r="Q173" s="50"/>
+      <c r="R173" s="50"/>
+      <c r="S173" s="50"/>
+      <c r="T173" s="50"/>
+      <c r="U173" s="50"/>
+      <c r="V173" s="50"/>
+      <c r="W173" s="50"/>
+      <c r="X173" s="50"/>
+      <c r="Y173" s="50"/>
+      <c r="Z173" s="50"/>
+      <c r="AA173" s="50"/>
+      <c r="AB173" s="51"/>
       <c r="AC173" s="11"/>
     </row>
     <row r="174" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7125,27 +7142,27 @@
       <c r="E174" s="6"/>
       <c r="F174" s="6"/>
       <c r="G174" s="6"/>
-      <c r="H174" s="51"/>
-      <c r="I174" s="52"/>
-      <c r="J174" s="52"/>
-      <c r="K174" s="52"/>
-      <c r="L174" s="52"/>
-      <c r="M174" s="52"/>
-      <c r="N174" s="52"/>
-      <c r="O174" s="52"/>
-      <c r="P174" s="52"/>
-      <c r="Q174" s="52"/>
-      <c r="R174" s="52"/>
-      <c r="S174" s="52"/>
-      <c r="T174" s="52"/>
-      <c r="U174" s="52"/>
-      <c r="V174" s="52"/>
-      <c r="W174" s="52"/>
-      <c r="X174" s="52"/>
-      <c r="Y174" s="52"/>
-      <c r="Z174" s="52"/>
-      <c r="AA174" s="52"/>
-      <c r="AB174" s="53"/>
+      <c r="H174" s="49"/>
+      <c r="I174" s="50"/>
+      <c r="J174" s="50"/>
+      <c r="K174" s="50"/>
+      <c r="L174" s="50"/>
+      <c r="M174" s="50"/>
+      <c r="N174" s="50"/>
+      <c r="O174" s="50"/>
+      <c r="P174" s="50"/>
+      <c r="Q174" s="50"/>
+      <c r="R174" s="50"/>
+      <c r="S174" s="50"/>
+      <c r="T174" s="50"/>
+      <c r="U174" s="50"/>
+      <c r="V174" s="50"/>
+      <c r="W174" s="50"/>
+      <c r="X174" s="50"/>
+      <c r="Y174" s="50"/>
+      <c r="Z174" s="50"/>
+      <c r="AA174" s="50"/>
+      <c r="AB174" s="51"/>
       <c r="AC174" s="11"/>
     </row>
     <row r="175" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7155,27 +7172,27 @@
       <c r="E175" s="6"/>
       <c r="F175" s="6"/>
       <c r="G175" s="6"/>
-      <c r="H175" s="51"/>
-      <c r="I175" s="52"/>
-      <c r="J175" s="52"/>
-      <c r="K175" s="52"/>
-      <c r="L175" s="52"/>
-      <c r="M175" s="52"/>
-      <c r="N175" s="52"/>
-      <c r="O175" s="52"/>
-      <c r="P175" s="52"/>
-      <c r="Q175" s="52"/>
-      <c r="R175" s="52"/>
-      <c r="S175" s="52"/>
-      <c r="T175" s="52"/>
-      <c r="U175" s="52"/>
-      <c r="V175" s="52"/>
-      <c r="W175" s="52"/>
-      <c r="X175" s="52"/>
-      <c r="Y175" s="52"/>
-      <c r="Z175" s="52"/>
-      <c r="AA175" s="52"/>
-      <c r="AB175" s="53"/>
+      <c r="H175" s="49"/>
+      <c r="I175" s="50"/>
+      <c r="J175" s="50"/>
+      <c r="K175" s="50"/>
+      <c r="L175" s="50"/>
+      <c r="M175" s="50"/>
+      <c r="N175" s="50"/>
+      <c r="O175" s="50"/>
+      <c r="P175" s="50"/>
+      <c r="Q175" s="50"/>
+      <c r="R175" s="50"/>
+      <c r="S175" s="50"/>
+      <c r="T175" s="50"/>
+      <c r="U175" s="50"/>
+      <c r="V175" s="50"/>
+      <c r="W175" s="50"/>
+      <c r="X175" s="50"/>
+      <c r="Y175" s="50"/>
+      <c r="Z175" s="50"/>
+      <c r="AA175" s="50"/>
+      <c r="AB175" s="51"/>
       <c r="AC175" s="11"/>
     </row>
     <row r="176" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7185,27 +7202,27 @@
       <c r="E176" s="6"/>
       <c r="F176" s="6"/>
       <c r="G176" s="6"/>
-      <c r="H176" s="51"/>
-      <c r="I176" s="52"/>
-      <c r="J176" s="52"/>
-      <c r="K176" s="52"/>
-      <c r="L176" s="52"/>
-      <c r="M176" s="52"/>
-      <c r="N176" s="52"/>
-      <c r="O176" s="52"/>
-      <c r="P176" s="52"/>
-      <c r="Q176" s="52"/>
-      <c r="R176" s="52"/>
-      <c r="S176" s="52"/>
-      <c r="T176" s="52"/>
-      <c r="U176" s="52"/>
-      <c r="V176" s="52"/>
-      <c r="W176" s="52"/>
-      <c r="X176" s="52"/>
-      <c r="Y176" s="52"/>
-      <c r="Z176" s="52"/>
-      <c r="AA176" s="52"/>
-      <c r="AB176" s="53"/>
+      <c r="H176" s="49"/>
+      <c r="I176" s="50"/>
+      <c r="J176" s="50"/>
+      <c r="K176" s="50"/>
+      <c r="L176" s="50"/>
+      <c r="M176" s="50"/>
+      <c r="N176" s="50"/>
+      <c r="O176" s="50"/>
+      <c r="P176" s="50"/>
+      <c r="Q176" s="50"/>
+      <c r="R176" s="50"/>
+      <c r="S176" s="50"/>
+      <c r="T176" s="50"/>
+      <c r="U176" s="50"/>
+      <c r="V176" s="50"/>
+      <c r="W176" s="50"/>
+      <c r="X176" s="50"/>
+      <c r="Y176" s="50"/>
+      <c r="Z176" s="50"/>
+      <c r="AA176" s="50"/>
+      <c r="AB176" s="51"/>
       <c r="AC176" s="11"/>
     </row>
     <row r="177" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7215,27 +7232,27 @@
       <c r="E177" s="6"/>
       <c r="F177" s="6"/>
       <c r="G177" s="6"/>
-      <c r="H177" s="54"/>
-      <c r="I177" s="55"/>
-      <c r="J177" s="55"/>
-      <c r="K177" s="55"/>
-      <c r="L177" s="55"/>
-      <c r="M177" s="55"/>
-      <c r="N177" s="55"/>
-      <c r="O177" s="55"/>
-      <c r="P177" s="55"/>
-      <c r="Q177" s="55"/>
-      <c r="R177" s="55"/>
-      <c r="S177" s="55"/>
-      <c r="T177" s="55"/>
-      <c r="U177" s="55"/>
-      <c r="V177" s="55"/>
-      <c r="W177" s="55"/>
-      <c r="X177" s="55"/>
-      <c r="Y177" s="55"/>
-      <c r="Z177" s="55"/>
-      <c r="AA177" s="55"/>
-      <c r="AB177" s="56"/>
+      <c r="H177" s="52"/>
+      <c r="I177" s="53"/>
+      <c r="J177" s="53"/>
+      <c r="K177" s="53"/>
+      <c r="L177" s="53"/>
+      <c r="M177" s="53"/>
+      <c r="N177" s="53"/>
+      <c r="O177" s="53"/>
+      <c r="P177" s="53"/>
+      <c r="Q177" s="53"/>
+      <c r="R177" s="53"/>
+      <c r="S177" s="53"/>
+      <c r="T177" s="53"/>
+      <c r="U177" s="53"/>
+      <c r="V177" s="53"/>
+      <c r="W177" s="53"/>
+      <c r="X177" s="53"/>
+      <c r="Y177" s="53"/>
+      <c r="Z177" s="53"/>
+      <c r="AA177" s="53"/>
+      <c r="AB177" s="54"/>
       <c r="AC177" s="11"/>
     </row>
     <row r="178" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7343,27 +7360,27 @@
         <v>2</v>
       </c>
       <c r="G182" s="6"/>
-      <c r="H182" s="48"/>
-      <c r="I182" s="49"/>
-      <c r="J182" s="49"/>
-      <c r="K182" s="49"/>
-      <c r="L182" s="49"/>
-      <c r="M182" s="49"/>
-      <c r="N182" s="49"/>
-      <c r="O182" s="49"/>
-      <c r="P182" s="49"/>
-      <c r="Q182" s="49"/>
-      <c r="R182" s="49"/>
-      <c r="S182" s="49"/>
-      <c r="T182" s="49"/>
-      <c r="U182" s="49"/>
-      <c r="V182" s="49"/>
-      <c r="W182" s="49"/>
-      <c r="X182" s="49"/>
-      <c r="Y182" s="49"/>
-      <c r="Z182" s="49"/>
-      <c r="AA182" s="49"/>
-      <c r="AB182" s="50"/>
+      <c r="H182" s="46"/>
+      <c r="I182" s="47"/>
+      <c r="J182" s="47"/>
+      <c r="K182" s="47"/>
+      <c r="L182" s="47"/>
+      <c r="M182" s="47"/>
+      <c r="N182" s="47"/>
+      <c r="O182" s="47"/>
+      <c r="P182" s="47"/>
+      <c r="Q182" s="47"/>
+      <c r="R182" s="47"/>
+      <c r="S182" s="47"/>
+      <c r="T182" s="47"/>
+      <c r="U182" s="47"/>
+      <c r="V182" s="47"/>
+      <c r="W182" s="47"/>
+      <c r="X182" s="47"/>
+      <c r="Y182" s="47"/>
+      <c r="Z182" s="47"/>
+      <c r="AA182" s="47"/>
+      <c r="AB182" s="48"/>
       <c r="AC182" s="11"/>
     </row>
     <row r="183" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7373,27 +7390,27 @@
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6"/>
-      <c r="H183" s="51"/>
-      <c r="I183" s="52"/>
-      <c r="J183" s="52"/>
-      <c r="K183" s="52"/>
-      <c r="L183" s="52"/>
-      <c r="M183" s="52"/>
-      <c r="N183" s="52"/>
-      <c r="O183" s="52"/>
-      <c r="P183" s="52"/>
-      <c r="Q183" s="52"/>
-      <c r="R183" s="52"/>
-      <c r="S183" s="52"/>
-      <c r="T183" s="52"/>
-      <c r="U183" s="52"/>
-      <c r="V183" s="52"/>
-      <c r="W183" s="52"/>
-      <c r="X183" s="52"/>
-      <c r="Y183" s="52"/>
-      <c r="Z183" s="52"/>
-      <c r="AA183" s="52"/>
-      <c r="AB183" s="53"/>
+      <c r="H183" s="49"/>
+      <c r="I183" s="50"/>
+      <c r="J183" s="50"/>
+      <c r="K183" s="50"/>
+      <c r="L183" s="50"/>
+      <c r="M183" s="50"/>
+      <c r="N183" s="50"/>
+      <c r="O183" s="50"/>
+      <c r="P183" s="50"/>
+      <c r="Q183" s="50"/>
+      <c r="R183" s="50"/>
+      <c r="S183" s="50"/>
+      <c r="T183" s="50"/>
+      <c r="U183" s="50"/>
+      <c r="V183" s="50"/>
+      <c r="W183" s="50"/>
+      <c r="X183" s="50"/>
+      <c r="Y183" s="50"/>
+      <c r="Z183" s="50"/>
+      <c r="AA183" s="50"/>
+      <c r="AB183" s="51"/>
       <c r="AC183" s="11"/>
     </row>
     <row r="184" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7403,27 +7420,27 @@
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
       <c r="G184" s="6"/>
-      <c r="H184" s="51"/>
-      <c r="I184" s="52"/>
-      <c r="J184" s="52"/>
-      <c r="K184" s="52"/>
-      <c r="L184" s="52"/>
-      <c r="M184" s="52"/>
-      <c r="N184" s="52"/>
-      <c r="O184" s="52"/>
-      <c r="P184" s="52"/>
-      <c r="Q184" s="52"/>
-      <c r="R184" s="52"/>
-      <c r="S184" s="52"/>
-      <c r="T184" s="52"/>
-      <c r="U184" s="52"/>
-      <c r="V184" s="52"/>
-      <c r="W184" s="52"/>
-      <c r="X184" s="52"/>
-      <c r="Y184" s="52"/>
-      <c r="Z184" s="52"/>
-      <c r="AA184" s="52"/>
-      <c r="AB184" s="53"/>
+      <c r="H184" s="49"/>
+      <c r="I184" s="50"/>
+      <c r="J184" s="50"/>
+      <c r="K184" s="50"/>
+      <c r="L184" s="50"/>
+      <c r="M184" s="50"/>
+      <c r="N184" s="50"/>
+      <c r="O184" s="50"/>
+      <c r="P184" s="50"/>
+      <c r="Q184" s="50"/>
+      <c r="R184" s="50"/>
+      <c r="S184" s="50"/>
+      <c r="T184" s="50"/>
+      <c r="U184" s="50"/>
+      <c r="V184" s="50"/>
+      <c r="W184" s="50"/>
+      <c r="X184" s="50"/>
+      <c r="Y184" s="50"/>
+      <c r="Z184" s="50"/>
+      <c r="AA184" s="50"/>
+      <c r="AB184" s="51"/>
       <c r="AC184" s="11"/>
     </row>
     <row r="185" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7433,27 +7450,27 @@
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
       <c r="G185" s="6"/>
-      <c r="H185" s="51"/>
-      <c r="I185" s="52"/>
-      <c r="J185" s="52"/>
-      <c r="K185" s="52"/>
-      <c r="L185" s="52"/>
-      <c r="M185" s="52"/>
-      <c r="N185" s="52"/>
-      <c r="O185" s="52"/>
-      <c r="P185" s="52"/>
-      <c r="Q185" s="52"/>
-      <c r="R185" s="52"/>
-      <c r="S185" s="52"/>
-      <c r="T185" s="52"/>
-      <c r="U185" s="52"/>
-      <c r="V185" s="52"/>
-      <c r="W185" s="52"/>
-      <c r="X185" s="52"/>
-      <c r="Y185" s="52"/>
-      <c r="Z185" s="52"/>
-      <c r="AA185" s="52"/>
-      <c r="AB185" s="53"/>
+      <c r="H185" s="49"/>
+      <c r="I185" s="50"/>
+      <c r="J185" s="50"/>
+      <c r="K185" s="50"/>
+      <c r="L185" s="50"/>
+      <c r="M185" s="50"/>
+      <c r="N185" s="50"/>
+      <c r="O185" s="50"/>
+      <c r="P185" s="50"/>
+      <c r="Q185" s="50"/>
+      <c r="R185" s="50"/>
+      <c r="S185" s="50"/>
+      <c r="T185" s="50"/>
+      <c r="U185" s="50"/>
+      <c r="V185" s="50"/>
+      <c r="W185" s="50"/>
+      <c r="X185" s="50"/>
+      <c r="Y185" s="50"/>
+      <c r="Z185" s="50"/>
+      <c r="AA185" s="50"/>
+      <c r="AB185" s="51"/>
       <c r="AC185" s="11"/>
     </row>
     <row r="186" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7463,27 +7480,27 @@
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
       <c r="G186" s="6"/>
-      <c r="H186" s="51"/>
-      <c r="I186" s="52"/>
-      <c r="J186" s="52"/>
-      <c r="K186" s="52"/>
-      <c r="L186" s="52"/>
-      <c r="M186" s="52"/>
-      <c r="N186" s="52"/>
-      <c r="O186" s="52"/>
-      <c r="P186" s="52"/>
-      <c r="Q186" s="52"/>
-      <c r="R186" s="52"/>
-      <c r="S186" s="52"/>
-      <c r="T186" s="52"/>
-      <c r="U186" s="52"/>
-      <c r="V186" s="52"/>
-      <c r="W186" s="52"/>
-      <c r="X186" s="52"/>
-      <c r="Y186" s="52"/>
-      <c r="Z186" s="52"/>
-      <c r="AA186" s="52"/>
-      <c r="AB186" s="53"/>
+      <c r="H186" s="49"/>
+      <c r="I186" s="50"/>
+      <c r="J186" s="50"/>
+      <c r="K186" s="50"/>
+      <c r="L186" s="50"/>
+      <c r="M186" s="50"/>
+      <c r="N186" s="50"/>
+      <c r="O186" s="50"/>
+      <c r="P186" s="50"/>
+      <c r="Q186" s="50"/>
+      <c r="R186" s="50"/>
+      <c r="S186" s="50"/>
+      <c r="T186" s="50"/>
+      <c r="U186" s="50"/>
+      <c r="V186" s="50"/>
+      <c r="W186" s="50"/>
+      <c r="X186" s="50"/>
+      <c r="Y186" s="50"/>
+      <c r="Z186" s="50"/>
+      <c r="AA186" s="50"/>
+      <c r="AB186" s="51"/>
       <c r="AC186" s="11"/>
     </row>
     <row r="187" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7493,27 +7510,27 @@
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
-      <c r="H187" s="51"/>
-      <c r="I187" s="52"/>
-      <c r="J187" s="52"/>
-      <c r="K187" s="52"/>
-      <c r="L187" s="52"/>
-      <c r="M187" s="52"/>
-      <c r="N187" s="52"/>
-      <c r="O187" s="52"/>
-      <c r="P187" s="52"/>
-      <c r="Q187" s="52"/>
-      <c r="R187" s="52"/>
-      <c r="S187" s="52"/>
-      <c r="T187" s="52"/>
-      <c r="U187" s="52"/>
-      <c r="V187" s="52"/>
-      <c r="W187" s="52"/>
-      <c r="X187" s="52"/>
-      <c r="Y187" s="52"/>
-      <c r="Z187" s="52"/>
-      <c r="AA187" s="52"/>
-      <c r="AB187" s="53"/>
+      <c r="H187" s="49"/>
+      <c r="I187" s="50"/>
+      <c r="J187" s="50"/>
+      <c r="K187" s="50"/>
+      <c r="L187" s="50"/>
+      <c r="M187" s="50"/>
+      <c r="N187" s="50"/>
+      <c r="O187" s="50"/>
+      <c r="P187" s="50"/>
+      <c r="Q187" s="50"/>
+      <c r="R187" s="50"/>
+      <c r="S187" s="50"/>
+      <c r="T187" s="50"/>
+      <c r="U187" s="50"/>
+      <c r="V187" s="50"/>
+      <c r="W187" s="50"/>
+      <c r="X187" s="50"/>
+      <c r="Y187" s="50"/>
+      <c r="Z187" s="50"/>
+      <c r="AA187" s="50"/>
+      <c r="AB187" s="51"/>
       <c r="AC187" s="11"/>
     </row>
     <row r="188" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7523,27 +7540,27 @@
       <c r="E188" s="6"/>
       <c r="F188" s="6"/>
       <c r="G188" s="6"/>
-      <c r="H188" s="54"/>
-      <c r="I188" s="55"/>
-      <c r="J188" s="55"/>
-      <c r="K188" s="55"/>
-      <c r="L188" s="55"/>
-      <c r="M188" s="55"/>
-      <c r="N188" s="55"/>
-      <c r="O188" s="55"/>
-      <c r="P188" s="55"/>
-      <c r="Q188" s="55"/>
-      <c r="R188" s="55"/>
-      <c r="S188" s="55"/>
-      <c r="T188" s="55"/>
-      <c r="U188" s="55"/>
-      <c r="V188" s="55"/>
-      <c r="W188" s="55"/>
-      <c r="X188" s="55"/>
-      <c r="Y188" s="55"/>
-      <c r="Z188" s="55"/>
-      <c r="AA188" s="55"/>
-      <c r="AB188" s="56"/>
+      <c r="H188" s="52"/>
+      <c r="I188" s="53"/>
+      <c r="J188" s="53"/>
+      <c r="K188" s="53"/>
+      <c r="L188" s="53"/>
+      <c r="M188" s="53"/>
+      <c r="N188" s="53"/>
+      <c r="O188" s="53"/>
+      <c r="P188" s="53"/>
+      <c r="Q188" s="53"/>
+      <c r="R188" s="53"/>
+      <c r="S188" s="53"/>
+      <c r="T188" s="53"/>
+      <c r="U188" s="53"/>
+      <c r="V188" s="53"/>
+      <c r="W188" s="53"/>
+      <c r="X188" s="53"/>
+      <c r="Y188" s="53"/>
+      <c r="Z188" s="53"/>
+      <c r="AA188" s="53"/>
+      <c r="AB188" s="54"/>
       <c r="AC188" s="11"/>
     </row>
     <row r="189" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7585,27 +7602,27 @@
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
       <c r="G190" s="6"/>
-      <c r="H190" s="48"/>
-      <c r="I190" s="49"/>
-      <c r="J190" s="49"/>
-      <c r="K190" s="49"/>
-      <c r="L190" s="49"/>
-      <c r="M190" s="49"/>
-      <c r="N190" s="49"/>
-      <c r="O190" s="49"/>
-      <c r="P190" s="49"/>
-      <c r="Q190" s="49"/>
-      <c r="R190" s="49"/>
-      <c r="S190" s="49"/>
-      <c r="T190" s="49"/>
-      <c r="U190" s="49"/>
-      <c r="V190" s="49"/>
-      <c r="W190" s="49"/>
-      <c r="X190" s="49"/>
-      <c r="Y190" s="49"/>
-      <c r="Z190" s="49"/>
-      <c r="AA190" s="49"/>
-      <c r="AB190" s="50"/>
+      <c r="H190" s="46"/>
+      <c r="I190" s="47"/>
+      <c r="J190" s="47"/>
+      <c r="K190" s="47"/>
+      <c r="L190" s="47"/>
+      <c r="M190" s="47"/>
+      <c r="N190" s="47"/>
+      <c r="O190" s="47"/>
+      <c r="P190" s="47"/>
+      <c r="Q190" s="47"/>
+      <c r="R190" s="47"/>
+      <c r="S190" s="47"/>
+      <c r="T190" s="47"/>
+      <c r="U190" s="47"/>
+      <c r="V190" s="47"/>
+      <c r="W190" s="47"/>
+      <c r="X190" s="47"/>
+      <c r="Y190" s="47"/>
+      <c r="Z190" s="47"/>
+      <c r="AA190" s="47"/>
+      <c r="AB190" s="48"/>
       <c r="AC190" s="11"/>
     </row>
     <row r="191" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7615,27 +7632,27 @@
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
       <c r="G191" s="6"/>
-      <c r="H191" s="51"/>
-      <c r="I191" s="52"/>
-      <c r="J191" s="52"/>
-      <c r="K191" s="52"/>
-      <c r="L191" s="52"/>
-      <c r="M191" s="52"/>
-      <c r="N191" s="52"/>
-      <c r="O191" s="52"/>
-      <c r="P191" s="52"/>
-      <c r="Q191" s="52"/>
-      <c r="R191" s="52"/>
-      <c r="S191" s="52"/>
-      <c r="T191" s="52"/>
-      <c r="U191" s="52"/>
-      <c r="V191" s="52"/>
-      <c r="W191" s="52"/>
-      <c r="X191" s="52"/>
-      <c r="Y191" s="52"/>
-      <c r="Z191" s="52"/>
-      <c r="AA191" s="52"/>
-      <c r="AB191" s="53"/>
+      <c r="H191" s="49"/>
+      <c r="I191" s="50"/>
+      <c r="J191" s="50"/>
+      <c r="K191" s="50"/>
+      <c r="L191" s="50"/>
+      <c r="M191" s="50"/>
+      <c r="N191" s="50"/>
+      <c r="O191" s="50"/>
+      <c r="P191" s="50"/>
+      <c r="Q191" s="50"/>
+      <c r="R191" s="50"/>
+      <c r="S191" s="50"/>
+      <c r="T191" s="50"/>
+      <c r="U191" s="50"/>
+      <c r="V191" s="50"/>
+      <c r="W191" s="50"/>
+      <c r="X191" s="50"/>
+      <c r="Y191" s="50"/>
+      <c r="Z191" s="50"/>
+      <c r="AA191" s="50"/>
+      <c r="AB191" s="51"/>
       <c r="AC191" s="11"/>
     </row>
     <row r="192" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7645,27 +7662,27 @@
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
       <c r="G192" s="6"/>
-      <c r="H192" s="51"/>
-      <c r="I192" s="52"/>
-      <c r="J192" s="52"/>
-      <c r="K192" s="52"/>
-      <c r="L192" s="52"/>
-      <c r="M192" s="52"/>
-      <c r="N192" s="52"/>
-      <c r="O192" s="52"/>
-      <c r="P192" s="52"/>
-      <c r="Q192" s="52"/>
-      <c r="R192" s="52"/>
-      <c r="S192" s="52"/>
-      <c r="T192" s="52"/>
-      <c r="U192" s="52"/>
-      <c r="V192" s="52"/>
-      <c r="W192" s="52"/>
-      <c r="X192" s="52"/>
-      <c r="Y192" s="52"/>
-      <c r="Z192" s="52"/>
-      <c r="AA192" s="52"/>
-      <c r="AB192" s="53"/>
+      <c r="H192" s="49"/>
+      <c r="I192" s="50"/>
+      <c r="J192" s="50"/>
+      <c r="K192" s="50"/>
+      <c r="L192" s="50"/>
+      <c r="M192" s="50"/>
+      <c r="N192" s="50"/>
+      <c r="O192" s="50"/>
+      <c r="P192" s="50"/>
+      <c r="Q192" s="50"/>
+      <c r="R192" s="50"/>
+      <c r="S192" s="50"/>
+      <c r="T192" s="50"/>
+      <c r="U192" s="50"/>
+      <c r="V192" s="50"/>
+      <c r="W192" s="50"/>
+      <c r="X192" s="50"/>
+      <c r="Y192" s="50"/>
+      <c r="Z192" s="50"/>
+      <c r="AA192" s="50"/>
+      <c r="AB192" s="51"/>
       <c r="AC192" s="11"/>
     </row>
     <row r="193" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7675,27 +7692,27 @@
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
       <c r="G193" s="6"/>
-      <c r="H193" s="51"/>
-      <c r="I193" s="52"/>
-      <c r="J193" s="52"/>
-      <c r="K193" s="52"/>
-      <c r="L193" s="52"/>
-      <c r="M193" s="52"/>
-      <c r="N193" s="52"/>
-      <c r="O193" s="52"/>
-      <c r="P193" s="52"/>
-      <c r="Q193" s="52"/>
-      <c r="R193" s="52"/>
-      <c r="S193" s="52"/>
-      <c r="T193" s="52"/>
-      <c r="U193" s="52"/>
-      <c r="V193" s="52"/>
-      <c r="W193" s="52"/>
-      <c r="X193" s="52"/>
-      <c r="Y193" s="52"/>
-      <c r="Z193" s="52"/>
-      <c r="AA193" s="52"/>
-      <c r="AB193" s="53"/>
+      <c r="H193" s="49"/>
+      <c r="I193" s="50"/>
+      <c r="J193" s="50"/>
+      <c r="K193" s="50"/>
+      <c r="L193" s="50"/>
+      <c r="M193" s="50"/>
+      <c r="N193" s="50"/>
+      <c r="O193" s="50"/>
+      <c r="P193" s="50"/>
+      <c r="Q193" s="50"/>
+      <c r="R193" s="50"/>
+      <c r="S193" s="50"/>
+      <c r="T193" s="50"/>
+      <c r="U193" s="50"/>
+      <c r="V193" s="50"/>
+      <c r="W193" s="50"/>
+      <c r="X193" s="50"/>
+      <c r="Y193" s="50"/>
+      <c r="Z193" s="50"/>
+      <c r="AA193" s="50"/>
+      <c r="AB193" s="51"/>
       <c r="AC193" s="11"/>
     </row>
     <row r="194" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7705,27 +7722,27 @@
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
-      <c r="H194" s="51"/>
-      <c r="I194" s="52"/>
-      <c r="J194" s="52"/>
-      <c r="K194" s="52"/>
-      <c r="L194" s="52"/>
-      <c r="M194" s="52"/>
-      <c r="N194" s="52"/>
-      <c r="O194" s="52"/>
-      <c r="P194" s="52"/>
-      <c r="Q194" s="52"/>
-      <c r="R194" s="52"/>
-      <c r="S194" s="52"/>
-      <c r="T194" s="52"/>
-      <c r="U194" s="52"/>
-      <c r="V194" s="52"/>
-      <c r="W194" s="52"/>
-      <c r="X194" s="52"/>
-      <c r="Y194" s="52"/>
-      <c r="Z194" s="52"/>
-      <c r="AA194" s="52"/>
-      <c r="AB194" s="53"/>
+      <c r="H194" s="49"/>
+      <c r="I194" s="50"/>
+      <c r="J194" s="50"/>
+      <c r="K194" s="50"/>
+      <c r="L194" s="50"/>
+      <c r="M194" s="50"/>
+      <c r="N194" s="50"/>
+      <c r="O194" s="50"/>
+      <c r="P194" s="50"/>
+      <c r="Q194" s="50"/>
+      <c r="R194" s="50"/>
+      <c r="S194" s="50"/>
+      <c r="T194" s="50"/>
+      <c r="U194" s="50"/>
+      <c r="V194" s="50"/>
+      <c r="W194" s="50"/>
+      <c r="X194" s="50"/>
+      <c r="Y194" s="50"/>
+      <c r="Z194" s="50"/>
+      <c r="AA194" s="50"/>
+      <c r="AB194" s="51"/>
       <c r="AC194" s="11"/>
     </row>
     <row r="195" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7735,27 +7752,27 @@
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
-      <c r="H195" s="51"/>
-      <c r="I195" s="52"/>
-      <c r="J195" s="52"/>
-      <c r="K195" s="52"/>
-      <c r="L195" s="52"/>
-      <c r="M195" s="52"/>
-      <c r="N195" s="52"/>
-      <c r="O195" s="52"/>
-      <c r="P195" s="52"/>
-      <c r="Q195" s="52"/>
-      <c r="R195" s="52"/>
-      <c r="S195" s="52"/>
-      <c r="T195" s="52"/>
-      <c r="U195" s="52"/>
-      <c r="V195" s="52"/>
-      <c r="W195" s="52"/>
-      <c r="X195" s="52"/>
-      <c r="Y195" s="52"/>
-      <c r="Z195" s="52"/>
-      <c r="AA195" s="52"/>
-      <c r="AB195" s="53"/>
+      <c r="H195" s="49"/>
+      <c r="I195" s="50"/>
+      <c r="J195" s="50"/>
+      <c r="K195" s="50"/>
+      <c r="L195" s="50"/>
+      <c r="M195" s="50"/>
+      <c r="N195" s="50"/>
+      <c r="O195" s="50"/>
+      <c r="P195" s="50"/>
+      <c r="Q195" s="50"/>
+      <c r="R195" s="50"/>
+      <c r="S195" s="50"/>
+      <c r="T195" s="50"/>
+      <c r="U195" s="50"/>
+      <c r="V195" s="50"/>
+      <c r="W195" s="50"/>
+      <c r="X195" s="50"/>
+      <c r="Y195" s="50"/>
+      <c r="Z195" s="50"/>
+      <c r="AA195" s="50"/>
+      <c r="AB195" s="51"/>
       <c r="AC195" s="11"/>
     </row>
     <row r="196" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7765,27 +7782,27 @@
       <c r="E196" s="6"/>
       <c r="F196" s="6"/>
       <c r="G196" s="6"/>
-      <c r="H196" s="54"/>
-      <c r="I196" s="55"/>
-      <c r="J196" s="55"/>
-      <c r="K196" s="55"/>
-      <c r="L196" s="55"/>
-      <c r="M196" s="55"/>
-      <c r="N196" s="55"/>
-      <c r="O196" s="55"/>
-      <c r="P196" s="55"/>
-      <c r="Q196" s="55"/>
-      <c r="R196" s="55"/>
-      <c r="S196" s="55"/>
-      <c r="T196" s="55"/>
-      <c r="U196" s="55"/>
-      <c r="V196" s="55"/>
-      <c r="W196" s="55"/>
-      <c r="X196" s="55"/>
-      <c r="Y196" s="55"/>
-      <c r="Z196" s="55"/>
-      <c r="AA196" s="55"/>
-      <c r="AB196" s="56"/>
+      <c r="H196" s="52"/>
+      <c r="I196" s="53"/>
+      <c r="J196" s="53"/>
+      <c r="K196" s="53"/>
+      <c r="L196" s="53"/>
+      <c r="M196" s="53"/>
+      <c r="N196" s="53"/>
+      <c r="O196" s="53"/>
+      <c r="P196" s="53"/>
+      <c r="Q196" s="53"/>
+      <c r="R196" s="53"/>
+      <c r="S196" s="53"/>
+      <c r="T196" s="53"/>
+      <c r="U196" s="53"/>
+      <c r="V196" s="53"/>
+      <c r="W196" s="53"/>
+      <c r="X196" s="53"/>
+      <c r="Y196" s="53"/>
+      <c r="Z196" s="53"/>
+      <c r="AA196" s="53"/>
+      <c r="AB196" s="54"/>
       <c r="AC196" s="11"/>
     </row>
     <row r="197" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7893,27 +7910,27 @@
         <v>2</v>
       </c>
       <c r="G201" s="6"/>
-      <c r="H201" s="48"/>
-      <c r="I201" s="49"/>
-      <c r="J201" s="49"/>
-      <c r="K201" s="49"/>
-      <c r="L201" s="49"/>
-      <c r="M201" s="49"/>
-      <c r="N201" s="49"/>
-      <c r="O201" s="49"/>
-      <c r="P201" s="49"/>
-      <c r="Q201" s="49"/>
-      <c r="R201" s="49"/>
-      <c r="S201" s="49"/>
-      <c r="T201" s="49"/>
-      <c r="U201" s="49"/>
-      <c r="V201" s="49"/>
-      <c r="W201" s="49"/>
-      <c r="X201" s="49"/>
-      <c r="Y201" s="49"/>
-      <c r="Z201" s="49"/>
-      <c r="AA201" s="49"/>
-      <c r="AB201" s="50"/>
+      <c r="H201" s="46"/>
+      <c r="I201" s="47"/>
+      <c r="J201" s="47"/>
+      <c r="K201" s="47"/>
+      <c r="L201" s="47"/>
+      <c r="M201" s="47"/>
+      <c r="N201" s="47"/>
+      <c r="O201" s="47"/>
+      <c r="P201" s="47"/>
+      <c r="Q201" s="47"/>
+      <c r="R201" s="47"/>
+      <c r="S201" s="47"/>
+      <c r="T201" s="47"/>
+      <c r="U201" s="47"/>
+      <c r="V201" s="47"/>
+      <c r="W201" s="47"/>
+      <c r="X201" s="47"/>
+      <c r="Y201" s="47"/>
+      <c r="Z201" s="47"/>
+      <c r="AA201" s="47"/>
+      <c r="AB201" s="48"/>
       <c r="AC201" s="11"/>
     </row>
     <row r="202" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7923,27 +7940,27 @@
       <c r="E202" s="6"/>
       <c r="F202" s="6"/>
       <c r="G202" s="6"/>
-      <c r="H202" s="51"/>
-      <c r="I202" s="52"/>
-      <c r="J202" s="52"/>
-      <c r="K202" s="52"/>
-      <c r="L202" s="52"/>
-      <c r="M202" s="52"/>
-      <c r="N202" s="52"/>
-      <c r="O202" s="52"/>
-      <c r="P202" s="52"/>
-      <c r="Q202" s="52"/>
-      <c r="R202" s="52"/>
-      <c r="S202" s="52"/>
-      <c r="T202" s="52"/>
-      <c r="U202" s="52"/>
-      <c r="V202" s="52"/>
-      <c r="W202" s="52"/>
-      <c r="X202" s="52"/>
-      <c r="Y202" s="52"/>
-      <c r="Z202" s="52"/>
-      <c r="AA202" s="52"/>
-      <c r="AB202" s="53"/>
+      <c r="H202" s="49"/>
+      <c r="I202" s="50"/>
+      <c r="J202" s="50"/>
+      <c r="K202" s="50"/>
+      <c r="L202" s="50"/>
+      <c r="M202" s="50"/>
+      <c r="N202" s="50"/>
+      <c r="O202" s="50"/>
+      <c r="P202" s="50"/>
+      <c r="Q202" s="50"/>
+      <c r="R202" s="50"/>
+      <c r="S202" s="50"/>
+      <c r="T202" s="50"/>
+      <c r="U202" s="50"/>
+      <c r="V202" s="50"/>
+      <c r="W202" s="50"/>
+      <c r="X202" s="50"/>
+      <c r="Y202" s="50"/>
+      <c r="Z202" s="50"/>
+      <c r="AA202" s="50"/>
+      <c r="AB202" s="51"/>
       <c r="AC202" s="11"/>
     </row>
     <row r="203" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7953,27 +7970,27 @@
       <c r="E203" s="6"/>
       <c r="F203" s="6"/>
       <c r="G203" s="6"/>
-      <c r="H203" s="51"/>
-      <c r="I203" s="52"/>
-      <c r="J203" s="52"/>
-      <c r="K203" s="52"/>
-      <c r="L203" s="52"/>
-      <c r="M203" s="52"/>
-      <c r="N203" s="52"/>
-      <c r="O203" s="52"/>
-      <c r="P203" s="52"/>
-      <c r="Q203" s="52"/>
-      <c r="R203" s="52"/>
-      <c r="S203" s="52"/>
-      <c r="T203" s="52"/>
-      <c r="U203" s="52"/>
-      <c r="V203" s="52"/>
-      <c r="W203" s="52"/>
-      <c r="X203" s="52"/>
-      <c r="Y203" s="52"/>
-      <c r="Z203" s="52"/>
-      <c r="AA203" s="52"/>
-      <c r="AB203" s="53"/>
+      <c r="H203" s="49"/>
+      <c r="I203" s="50"/>
+      <c r="J203" s="50"/>
+      <c r="K203" s="50"/>
+      <c r="L203" s="50"/>
+      <c r="M203" s="50"/>
+      <c r="N203" s="50"/>
+      <c r="O203" s="50"/>
+      <c r="P203" s="50"/>
+      <c r="Q203" s="50"/>
+      <c r="R203" s="50"/>
+      <c r="S203" s="50"/>
+      <c r="T203" s="50"/>
+      <c r="U203" s="50"/>
+      <c r="V203" s="50"/>
+      <c r="W203" s="50"/>
+      <c r="X203" s="50"/>
+      <c r="Y203" s="50"/>
+      <c r="Z203" s="50"/>
+      <c r="AA203" s="50"/>
+      <c r="AB203" s="51"/>
       <c r="AC203" s="11"/>
     </row>
     <row r="204" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7983,27 +8000,27 @@
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
       <c r="G204" s="6"/>
-      <c r="H204" s="51"/>
-      <c r="I204" s="52"/>
-      <c r="J204" s="52"/>
-      <c r="K204" s="52"/>
-      <c r="L204" s="52"/>
-      <c r="M204" s="52"/>
-      <c r="N204" s="52"/>
-      <c r="O204" s="52"/>
-      <c r="P204" s="52"/>
-      <c r="Q204" s="52"/>
-      <c r="R204" s="52"/>
-      <c r="S204" s="52"/>
-      <c r="T204" s="52"/>
-      <c r="U204" s="52"/>
-      <c r="V204" s="52"/>
-      <c r="W204" s="52"/>
-      <c r="X204" s="52"/>
-      <c r="Y204" s="52"/>
-      <c r="Z204" s="52"/>
-      <c r="AA204" s="52"/>
-      <c r="AB204" s="53"/>
+      <c r="H204" s="49"/>
+      <c r="I204" s="50"/>
+      <c r="J204" s="50"/>
+      <c r="K204" s="50"/>
+      <c r="L204" s="50"/>
+      <c r="M204" s="50"/>
+      <c r="N204" s="50"/>
+      <c r="O204" s="50"/>
+      <c r="P204" s="50"/>
+      <c r="Q204" s="50"/>
+      <c r="R204" s="50"/>
+      <c r="S204" s="50"/>
+      <c r="T204" s="50"/>
+      <c r="U204" s="50"/>
+      <c r="V204" s="50"/>
+      <c r="W204" s="50"/>
+      <c r="X204" s="50"/>
+      <c r="Y204" s="50"/>
+      <c r="Z204" s="50"/>
+      <c r="AA204" s="50"/>
+      <c r="AB204" s="51"/>
       <c r="AC204" s="11"/>
     </row>
     <row r="205" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8013,27 +8030,27 @@
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
       <c r="G205" s="6"/>
-      <c r="H205" s="51"/>
-      <c r="I205" s="52"/>
-      <c r="J205" s="52"/>
-      <c r="K205" s="52"/>
-      <c r="L205" s="52"/>
-      <c r="M205" s="52"/>
-      <c r="N205" s="52"/>
-      <c r="O205" s="52"/>
-      <c r="P205" s="52"/>
-      <c r="Q205" s="52"/>
-      <c r="R205" s="52"/>
-      <c r="S205" s="52"/>
-      <c r="T205" s="52"/>
-      <c r="U205" s="52"/>
-      <c r="V205" s="52"/>
-      <c r="W205" s="52"/>
-      <c r="X205" s="52"/>
-      <c r="Y205" s="52"/>
-      <c r="Z205" s="52"/>
-      <c r="AA205" s="52"/>
-      <c r="AB205" s="53"/>
+      <c r="H205" s="49"/>
+      <c r="I205" s="50"/>
+      <c r="J205" s="50"/>
+      <c r="K205" s="50"/>
+      <c r="L205" s="50"/>
+      <c r="M205" s="50"/>
+      <c r="N205" s="50"/>
+      <c r="O205" s="50"/>
+      <c r="P205" s="50"/>
+      <c r="Q205" s="50"/>
+      <c r="R205" s="50"/>
+      <c r="S205" s="50"/>
+      <c r="T205" s="50"/>
+      <c r="U205" s="50"/>
+      <c r="V205" s="50"/>
+      <c r="W205" s="50"/>
+      <c r="X205" s="50"/>
+      <c r="Y205" s="50"/>
+      <c r="Z205" s="50"/>
+      <c r="AA205" s="50"/>
+      <c r="AB205" s="51"/>
       <c r="AC205" s="11"/>
     </row>
     <row r="206" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8043,27 +8060,27 @@
       <c r="E206" s="6"/>
       <c r="F206" s="6"/>
       <c r="G206" s="6"/>
-      <c r="H206" s="51"/>
-      <c r="I206" s="52"/>
-      <c r="J206" s="52"/>
-      <c r="K206" s="52"/>
-      <c r="L206" s="52"/>
-      <c r="M206" s="52"/>
-      <c r="N206" s="52"/>
-      <c r="O206" s="52"/>
-      <c r="P206" s="52"/>
-      <c r="Q206" s="52"/>
-      <c r="R206" s="52"/>
-      <c r="S206" s="52"/>
-      <c r="T206" s="52"/>
-      <c r="U206" s="52"/>
-      <c r="V206" s="52"/>
-      <c r="W206" s="52"/>
-      <c r="X206" s="52"/>
-      <c r="Y206" s="52"/>
-      <c r="Z206" s="52"/>
-      <c r="AA206" s="52"/>
-      <c r="AB206" s="53"/>
+      <c r="H206" s="49"/>
+      <c r="I206" s="50"/>
+      <c r="J206" s="50"/>
+      <c r="K206" s="50"/>
+      <c r="L206" s="50"/>
+      <c r="M206" s="50"/>
+      <c r="N206" s="50"/>
+      <c r="O206" s="50"/>
+      <c r="P206" s="50"/>
+      <c r="Q206" s="50"/>
+      <c r="R206" s="50"/>
+      <c r="S206" s="50"/>
+      <c r="T206" s="50"/>
+      <c r="U206" s="50"/>
+      <c r="V206" s="50"/>
+      <c r="W206" s="50"/>
+      <c r="X206" s="50"/>
+      <c r="Y206" s="50"/>
+      <c r="Z206" s="50"/>
+      <c r="AA206" s="50"/>
+      <c r="AB206" s="51"/>
       <c r="AC206" s="11"/>
     </row>
     <row r="207" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8073,27 +8090,27 @@
       <c r="E207" s="6"/>
       <c r="F207" s="6"/>
       <c r="G207" s="6"/>
-      <c r="H207" s="54"/>
-      <c r="I207" s="55"/>
-      <c r="J207" s="55"/>
-      <c r="K207" s="55"/>
-      <c r="L207" s="55"/>
-      <c r="M207" s="55"/>
-      <c r="N207" s="55"/>
-      <c r="O207" s="55"/>
-      <c r="P207" s="55"/>
-      <c r="Q207" s="55"/>
-      <c r="R207" s="55"/>
-      <c r="S207" s="55"/>
-      <c r="T207" s="55"/>
-      <c r="U207" s="55"/>
-      <c r="V207" s="55"/>
-      <c r="W207" s="55"/>
-      <c r="X207" s="55"/>
-      <c r="Y207" s="55"/>
-      <c r="Z207" s="55"/>
-      <c r="AA207" s="55"/>
-      <c r="AB207" s="56"/>
+      <c r="H207" s="52"/>
+      <c r="I207" s="53"/>
+      <c r="J207" s="53"/>
+      <c r="K207" s="53"/>
+      <c r="L207" s="53"/>
+      <c r="M207" s="53"/>
+      <c r="N207" s="53"/>
+      <c r="O207" s="53"/>
+      <c r="P207" s="53"/>
+      <c r="Q207" s="53"/>
+      <c r="R207" s="53"/>
+      <c r="S207" s="53"/>
+      <c r="T207" s="53"/>
+      <c r="U207" s="53"/>
+      <c r="V207" s="53"/>
+      <c r="W207" s="53"/>
+      <c r="X207" s="53"/>
+      <c r="Y207" s="53"/>
+      <c r="Z207" s="53"/>
+      <c r="AA207" s="53"/>
+      <c r="AB207" s="54"/>
       <c r="AC207" s="11"/>
     </row>
     <row r="208" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8135,27 +8152,27 @@
       <c r="E209" s="6"/>
       <c r="F209" s="6"/>
       <c r="G209" s="6"/>
-      <c r="H209" s="48"/>
-      <c r="I209" s="49"/>
-      <c r="J209" s="49"/>
-      <c r="K209" s="49"/>
-      <c r="L209" s="49"/>
-      <c r="M209" s="49"/>
-      <c r="N209" s="49"/>
-      <c r="O209" s="49"/>
-      <c r="P209" s="49"/>
-      <c r="Q209" s="49"/>
-      <c r="R209" s="49"/>
-      <c r="S209" s="49"/>
-      <c r="T209" s="49"/>
-      <c r="U209" s="49"/>
-      <c r="V209" s="49"/>
-      <c r="W209" s="49"/>
-      <c r="X209" s="49"/>
-      <c r="Y209" s="49"/>
-      <c r="Z209" s="49"/>
-      <c r="AA209" s="49"/>
-      <c r="AB209" s="50"/>
+      <c r="H209" s="46"/>
+      <c r="I209" s="47"/>
+      <c r="J209" s="47"/>
+      <c r="K209" s="47"/>
+      <c r="L209" s="47"/>
+      <c r="M209" s="47"/>
+      <c r="N209" s="47"/>
+      <c r="O209" s="47"/>
+      <c r="P209" s="47"/>
+      <c r="Q209" s="47"/>
+      <c r="R209" s="47"/>
+      <c r="S209" s="47"/>
+      <c r="T209" s="47"/>
+      <c r="U209" s="47"/>
+      <c r="V209" s="47"/>
+      <c r="W209" s="47"/>
+      <c r="X209" s="47"/>
+      <c r="Y209" s="47"/>
+      <c r="Z209" s="47"/>
+      <c r="AA209" s="47"/>
+      <c r="AB209" s="48"/>
       <c r="AC209" s="11"/>
     </row>
     <row r="210" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8165,27 +8182,27 @@
       <c r="E210" s="6"/>
       <c r="F210" s="6"/>
       <c r="G210" s="6"/>
-      <c r="H210" s="51"/>
-      <c r="I210" s="52"/>
-      <c r="J210" s="52"/>
-      <c r="K210" s="52"/>
-      <c r="L210" s="52"/>
-      <c r="M210" s="52"/>
-      <c r="N210" s="52"/>
-      <c r="O210" s="52"/>
-      <c r="P210" s="52"/>
-      <c r="Q210" s="52"/>
-      <c r="R210" s="52"/>
-      <c r="S210" s="52"/>
-      <c r="T210" s="52"/>
-      <c r="U210" s="52"/>
-      <c r="V210" s="52"/>
-      <c r="W210" s="52"/>
-      <c r="X210" s="52"/>
-      <c r="Y210" s="52"/>
-      <c r="Z210" s="52"/>
-      <c r="AA210" s="52"/>
-      <c r="AB210" s="53"/>
+      <c r="H210" s="49"/>
+      <c r="I210" s="50"/>
+      <c r="J210" s="50"/>
+      <c r="K210" s="50"/>
+      <c r="L210" s="50"/>
+      <c r="M210" s="50"/>
+      <c r="N210" s="50"/>
+      <c r="O210" s="50"/>
+      <c r="P210" s="50"/>
+      <c r="Q210" s="50"/>
+      <c r="R210" s="50"/>
+      <c r="S210" s="50"/>
+      <c r="T210" s="50"/>
+      <c r="U210" s="50"/>
+      <c r="V210" s="50"/>
+      <c r="W210" s="50"/>
+      <c r="X210" s="50"/>
+      <c r="Y210" s="50"/>
+      <c r="Z210" s="50"/>
+      <c r="AA210" s="50"/>
+      <c r="AB210" s="51"/>
       <c r="AC210" s="11"/>
     </row>
     <row r="211" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8195,27 +8212,27 @@
       <c r="E211" s="6"/>
       <c r="F211" s="6"/>
       <c r="G211" s="6"/>
-      <c r="H211" s="51"/>
-      <c r="I211" s="52"/>
-      <c r="J211" s="52"/>
-      <c r="K211" s="52"/>
-      <c r="L211" s="52"/>
-      <c r="M211" s="52"/>
-      <c r="N211" s="52"/>
-      <c r="O211" s="52"/>
-      <c r="P211" s="52"/>
-      <c r="Q211" s="52"/>
-      <c r="R211" s="52"/>
-      <c r="S211" s="52"/>
-      <c r="T211" s="52"/>
-      <c r="U211" s="52"/>
-      <c r="V211" s="52"/>
-      <c r="W211" s="52"/>
-      <c r="X211" s="52"/>
-      <c r="Y211" s="52"/>
-      <c r="Z211" s="52"/>
-      <c r="AA211" s="52"/>
-      <c r="AB211" s="53"/>
+      <c r="H211" s="49"/>
+      <c r="I211" s="50"/>
+      <c r="J211" s="50"/>
+      <c r="K211" s="50"/>
+      <c r="L211" s="50"/>
+      <c r="M211" s="50"/>
+      <c r="N211" s="50"/>
+      <c r="O211" s="50"/>
+      <c r="P211" s="50"/>
+      <c r="Q211" s="50"/>
+      <c r="R211" s="50"/>
+      <c r="S211" s="50"/>
+      <c r="T211" s="50"/>
+      <c r="U211" s="50"/>
+      <c r="V211" s="50"/>
+      <c r="W211" s="50"/>
+      <c r="X211" s="50"/>
+      <c r="Y211" s="50"/>
+      <c r="Z211" s="50"/>
+      <c r="AA211" s="50"/>
+      <c r="AB211" s="51"/>
       <c r="AC211" s="11"/>
     </row>
     <row r="212" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8225,27 +8242,27 @@
       <c r="E212" s="6"/>
       <c r="F212" s="6"/>
       <c r="G212" s="6"/>
-      <c r="H212" s="51"/>
-      <c r="I212" s="52"/>
-      <c r="J212" s="52"/>
-      <c r="K212" s="52"/>
-      <c r="L212" s="52"/>
-      <c r="M212" s="52"/>
-      <c r="N212" s="52"/>
-      <c r="O212" s="52"/>
-      <c r="P212" s="52"/>
-      <c r="Q212" s="52"/>
-      <c r="R212" s="52"/>
-      <c r="S212" s="52"/>
-      <c r="T212" s="52"/>
-      <c r="U212" s="52"/>
-      <c r="V212" s="52"/>
-      <c r="W212" s="52"/>
-      <c r="X212" s="52"/>
-      <c r="Y212" s="52"/>
-      <c r="Z212" s="52"/>
-      <c r="AA212" s="52"/>
-      <c r="AB212" s="53"/>
+      <c r="H212" s="49"/>
+      <c r="I212" s="50"/>
+      <c r="J212" s="50"/>
+      <c r="K212" s="50"/>
+      <c r="L212" s="50"/>
+      <c r="M212" s="50"/>
+      <c r="N212" s="50"/>
+      <c r="O212" s="50"/>
+      <c r="P212" s="50"/>
+      <c r="Q212" s="50"/>
+      <c r="R212" s="50"/>
+      <c r="S212" s="50"/>
+      <c r="T212" s="50"/>
+      <c r="U212" s="50"/>
+      <c r="V212" s="50"/>
+      <c r="W212" s="50"/>
+      <c r="X212" s="50"/>
+      <c r="Y212" s="50"/>
+      <c r="Z212" s="50"/>
+      <c r="AA212" s="50"/>
+      <c r="AB212" s="51"/>
       <c r="AC212" s="11"/>
     </row>
     <row r="213" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8255,27 +8272,27 @@
       <c r="E213" s="6"/>
       <c r="F213" s="6"/>
       <c r="G213" s="6"/>
-      <c r="H213" s="51"/>
-      <c r="I213" s="52"/>
-      <c r="J213" s="52"/>
-      <c r="K213" s="52"/>
-      <c r="L213" s="52"/>
-      <c r="M213" s="52"/>
-      <c r="N213" s="52"/>
-      <c r="O213" s="52"/>
-      <c r="P213" s="52"/>
-      <c r="Q213" s="52"/>
-      <c r="R213" s="52"/>
-      <c r="S213" s="52"/>
-      <c r="T213" s="52"/>
-      <c r="U213" s="52"/>
-      <c r="V213" s="52"/>
-      <c r="W213" s="52"/>
-      <c r="X213" s="52"/>
-      <c r="Y213" s="52"/>
-      <c r="Z213" s="52"/>
-      <c r="AA213" s="52"/>
-      <c r="AB213" s="53"/>
+      <c r="H213" s="49"/>
+      <c r="I213" s="50"/>
+      <c r="J213" s="50"/>
+      <c r="K213" s="50"/>
+      <c r="L213" s="50"/>
+      <c r="M213" s="50"/>
+      <c r="N213" s="50"/>
+      <c r="O213" s="50"/>
+      <c r="P213" s="50"/>
+      <c r="Q213" s="50"/>
+      <c r="R213" s="50"/>
+      <c r="S213" s="50"/>
+      <c r="T213" s="50"/>
+      <c r="U213" s="50"/>
+      <c r="V213" s="50"/>
+      <c r="W213" s="50"/>
+      <c r="X213" s="50"/>
+      <c r="Y213" s="50"/>
+      <c r="Z213" s="50"/>
+      <c r="AA213" s="50"/>
+      <c r="AB213" s="51"/>
       <c r="AC213" s="11"/>
     </row>
     <row r="214" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8285,27 +8302,27 @@
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
-      <c r="H214" s="51"/>
-      <c r="I214" s="52"/>
-      <c r="J214" s="52"/>
-      <c r="K214" s="52"/>
-      <c r="L214" s="52"/>
-      <c r="M214" s="52"/>
-      <c r="N214" s="52"/>
-      <c r="O214" s="52"/>
-      <c r="P214" s="52"/>
-      <c r="Q214" s="52"/>
-      <c r="R214" s="52"/>
-      <c r="S214" s="52"/>
-      <c r="T214" s="52"/>
-      <c r="U214" s="52"/>
-      <c r="V214" s="52"/>
-      <c r="W214" s="52"/>
-      <c r="X214" s="52"/>
-      <c r="Y214" s="52"/>
-      <c r="Z214" s="52"/>
-      <c r="AA214" s="52"/>
-      <c r="AB214" s="53"/>
+      <c r="H214" s="49"/>
+      <c r="I214" s="50"/>
+      <c r="J214" s="50"/>
+      <c r="K214" s="50"/>
+      <c r="L214" s="50"/>
+      <c r="M214" s="50"/>
+      <c r="N214" s="50"/>
+      <c r="O214" s="50"/>
+      <c r="P214" s="50"/>
+      <c r="Q214" s="50"/>
+      <c r="R214" s="50"/>
+      <c r="S214" s="50"/>
+      <c r="T214" s="50"/>
+      <c r="U214" s="50"/>
+      <c r="V214" s="50"/>
+      <c r="W214" s="50"/>
+      <c r="X214" s="50"/>
+      <c r="Y214" s="50"/>
+      <c r="Z214" s="50"/>
+      <c r="AA214" s="50"/>
+      <c r="AB214" s="51"/>
       <c r="AC214" s="11"/>
     </row>
     <row r="215" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8315,27 +8332,27 @@
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
       <c r="G215" s="6"/>
-      <c r="H215" s="54"/>
-      <c r="I215" s="55"/>
-      <c r="J215" s="55"/>
-      <c r="K215" s="55"/>
-      <c r="L215" s="55"/>
-      <c r="M215" s="55"/>
-      <c r="N215" s="55"/>
-      <c r="O215" s="55"/>
-      <c r="P215" s="55"/>
-      <c r="Q215" s="55"/>
-      <c r="R215" s="55"/>
-      <c r="S215" s="55"/>
-      <c r="T215" s="55"/>
-      <c r="U215" s="55"/>
-      <c r="V215" s="55"/>
-      <c r="W215" s="55"/>
-      <c r="X215" s="55"/>
-      <c r="Y215" s="55"/>
-      <c r="Z215" s="55"/>
-      <c r="AA215" s="55"/>
-      <c r="AB215" s="56"/>
+      <c r="H215" s="52"/>
+      <c r="I215" s="53"/>
+      <c r="J215" s="53"/>
+      <c r="K215" s="53"/>
+      <c r="L215" s="53"/>
+      <c r="M215" s="53"/>
+      <c r="N215" s="53"/>
+      <c r="O215" s="53"/>
+      <c r="P215" s="53"/>
+      <c r="Q215" s="53"/>
+      <c r="R215" s="53"/>
+      <c r="S215" s="53"/>
+      <c r="T215" s="53"/>
+      <c r="U215" s="53"/>
+      <c r="V215" s="53"/>
+      <c r="W215" s="53"/>
+      <c r="X215" s="53"/>
+      <c r="Y215" s="53"/>
+      <c r="Z215" s="53"/>
+      <c r="AA215" s="53"/>
+      <c r="AB215" s="54"/>
       <c r="AC215" s="11"/>
     </row>
     <row r="216" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8370,6 +8387,43 @@
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B6:B23"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="H8:AB14"/>
+    <mergeCell ref="H16:AB22"/>
+    <mergeCell ref="B25:B42"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="H27:AB33"/>
+    <mergeCell ref="H35:AB41"/>
+    <mergeCell ref="B44:B61"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="H46:AB52"/>
+    <mergeCell ref="H54:AB60"/>
+    <mergeCell ref="B63:B83"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="H76:AB82"/>
+    <mergeCell ref="B85:B102"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="H87:AB93"/>
+    <mergeCell ref="H95:AB101"/>
+    <mergeCell ref="H65:AB74"/>
+    <mergeCell ref="B104:B121"/>
+    <mergeCell ref="D106:E106"/>
+    <mergeCell ref="H106:AB112"/>
+    <mergeCell ref="H114:AB120"/>
+    <mergeCell ref="B123:B140"/>
+    <mergeCell ref="D125:E125"/>
+    <mergeCell ref="H125:AB131"/>
+    <mergeCell ref="H133:AB139"/>
+    <mergeCell ref="B142:B159"/>
+    <mergeCell ref="D144:E144"/>
+    <mergeCell ref="H144:AB150"/>
+    <mergeCell ref="H152:AB158"/>
+    <mergeCell ref="B161:B178"/>
+    <mergeCell ref="D163:E163"/>
+    <mergeCell ref="H163:AB169"/>
+    <mergeCell ref="H171:AB177"/>
     <mergeCell ref="B180:B197"/>
     <mergeCell ref="D182:E182"/>
     <mergeCell ref="H182:AB188"/>
@@ -8378,48 +8432,12 @@
     <mergeCell ref="D201:E201"/>
     <mergeCell ref="H201:AB207"/>
     <mergeCell ref="H209:AB215"/>
-    <mergeCell ref="B142:B159"/>
-    <mergeCell ref="D144:E144"/>
-    <mergeCell ref="H144:AB150"/>
-    <mergeCell ref="H152:AB158"/>
-    <mergeCell ref="B161:B178"/>
-    <mergeCell ref="D163:E163"/>
-    <mergeCell ref="H163:AB169"/>
-    <mergeCell ref="H171:AB177"/>
-    <mergeCell ref="B104:B121"/>
-    <mergeCell ref="D106:E106"/>
-    <mergeCell ref="H106:AB112"/>
-    <mergeCell ref="H114:AB120"/>
-    <mergeCell ref="B123:B140"/>
-    <mergeCell ref="D125:E125"/>
-    <mergeCell ref="H125:AB131"/>
-    <mergeCell ref="H133:AB139"/>
-    <mergeCell ref="B63:B83"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="H76:AB82"/>
-    <mergeCell ref="B85:B102"/>
-    <mergeCell ref="D87:E87"/>
-    <mergeCell ref="H87:AB93"/>
-    <mergeCell ref="H95:AB101"/>
-    <mergeCell ref="H65:AB74"/>
-    <mergeCell ref="B25:B42"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="H27:AB33"/>
-    <mergeCell ref="H35:AB41"/>
-    <mergeCell ref="B44:B61"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="H46:AB52"/>
-    <mergeCell ref="H54:AB60"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B6:B23"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="H8:AB14"/>
-    <mergeCell ref="H16:AB22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H65" r:id="rId1" display="https://learn.microsoft.com/en-us/dotnet/maui/platform-integration/device/geolocation" xr:uid="{6A2F2CBC-218B-43EA-806A-9BF39365BDB2}"/>
     <hyperlink ref="H87" r:id="rId2" display="https://dummyjson.com/docs/posts_x000a_" xr:uid="{AFA4F006-3754-4C92-A758-50B6915FC379}"/>
     <hyperlink ref="H106" r:id="rId3" display="https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/refreshview_x000a_" xr:uid="{80E066CC-CE62-4304-89CB-2C900A3EBBE5}"/>
+    <hyperlink ref="H125" r:id="rId4" display="https://learn.microsoft.com/de-de/dotnet/communitytoolkit/maui/views/mediaelement" xr:uid="{A9CAE96C-CEA9-42B5-BE11-A814029EF10A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -8446,11 +8464,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>21</v>
       </c>
@@ -9292,27 +9310,27 @@
       <c r="E34" s="27"/>
       <c r="F34" s="28"/>
       <c r="G34" s="19"/>
-      <c r="H34" s="48"/>
-      <c r="I34" s="49"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
-      <c r="L34" s="49"/>
-      <c r="M34" s="49"/>
-      <c r="N34" s="49"/>
-      <c r="O34" s="49"/>
-      <c r="P34" s="49"/>
-      <c r="Q34" s="49"/>
-      <c r="R34" s="49"/>
-      <c r="S34" s="49"/>
-      <c r="T34" s="49"/>
-      <c r="U34" s="49"/>
-      <c r="V34" s="49"/>
-      <c r="W34" s="49"/>
-      <c r="X34" s="49"/>
-      <c r="Y34" s="49"/>
-      <c r="Z34" s="49"/>
-      <c r="AA34" s="49"/>
-      <c r="AB34" s="50"/>
+      <c r="H34" s="46"/>
+      <c r="I34" s="47"/>
+      <c r="J34" s="47"/>
+      <c r="K34" s="47"/>
+      <c r="L34" s="47"/>
+      <c r="M34" s="47"/>
+      <c r="N34" s="47"/>
+      <c r="O34" s="47"/>
+      <c r="P34" s="47"/>
+      <c r="Q34" s="47"/>
+      <c r="R34" s="47"/>
+      <c r="S34" s="47"/>
+      <c r="T34" s="47"/>
+      <c r="U34" s="47"/>
+      <c r="V34" s="47"/>
+      <c r="W34" s="47"/>
+      <c r="X34" s="47"/>
+      <c r="Y34" s="47"/>
+      <c r="Z34" s="47"/>
+      <c r="AA34" s="47"/>
+      <c r="AB34" s="48"/>
       <c r="AC34" s="16"/>
     </row>
     <row r="35" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9322,27 +9340,27 @@
       <c r="E35" s="19"/>
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
-      <c r="H35" s="51"/>
-      <c r="I35" s="52"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52"/>
-      <c r="M35" s="52"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="52"/>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="52"/>
-      <c r="R35" s="52"/>
-      <c r="S35" s="52"/>
-      <c r="T35" s="52"/>
-      <c r="U35" s="52"/>
-      <c r="V35" s="52"/>
-      <c r="W35" s="52"/>
-      <c r="X35" s="52"/>
-      <c r="Y35" s="52"/>
-      <c r="Z35" s="52"/>
-      <c r="AA35" s="52"/>
-      <c r="AB35" s="53"/>
+      <c r="H35" s="49"/>
+      <c r="I35" s="50"/>
+      <c r="J35" s="50"/>
+      <c r="K35" s="50"/>
+      <c r="L35" s="50"/>
+      <c r="M35" s="50"/>
+      <c r="N35" s="50"/>
+      <c r="O35" s="50"/>
+      <c r="P35" s="50"/>
+      <c r="Q35" s="50"/>
+      <c r="R35" s="50"/>
+      <c r="S35" s="50"/>
+      <c r="T35" s="50"/>
+      <c r="U35" s="50"/>
+      <c r="V35" s="50"/>
+      <c r="W35" s="50"/>
+      <c r="X35" s="50"/>
+      <c r="Y35" s="50"/>
+      <c r="Z35" s="50"/>
+      <c r="AA35" s="50"/>
+      <c r="AB35" s="51"/>
       <c r="AC35" s="16"/>
     </row>
     <row r="36" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9352,27 +9370,27 @@
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
-      <c r="H36" s="51"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="L36" s="52"/>
-      <c r="M36" s="52"/>
-      <c r="N36" s="52"/>
-      <c r="O36" s="52"/>
-      <c r="P36" s="52"/>
-      <c r="Q36" s="52"/>
-      <c r="R36" s="52"/>
-      <c r="S36" s="52"/>
-      <c r="T36" s="52"/>
-      <c r="U36" s="52"/>
-      <c r="V36" s="52"/>
-      <c r="W36" s="52"/>
-      <c r="X36" s="52"/>
-      <c r="Y36" s="52"/>
-      <c r="Z36" s="52"/>
-      <c r="AA36" s="52"/>
-      <c r="AB36" s="53"/>
+      <c r="H36" s="49"/>
+      <c r="I36" s="50"/>
+      <c r="J36" s="50"/>
+      <c r="K36" s="50"/>
+      <c r="L36" s="50"/>
+      <c r="M36" s="50"/>
+      <c r="N36" s="50"/>
+      <c r="O36" s="50"/>
+      <c r="P36" s="50"/>
+      <c r="Q36" s="50"/>
+      <c r="R36" s="50"/>
+      <c r="S36" s="50"/>
+      <c r="T36" s="50"/>
+      <c r="U36" s="50"/>
+      <c r="V36" s="50"/>
+      <c r="W36" s="50"/>
+      <c r="X36" s="50"/>
+      <c r="Y36" s="50"/>
+      <c r="Z36" s="50"/>
+      <c r="AA36" s="50"/>
+      <c r="AB36" s="51"/>
       <c r="AC36" s="16"/>
     </row>
     <row r="37" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9382,27 +9400,27 @@
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
-      <c r="H37" s="51"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="52"/>
-      <c r="N37" s="52"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="52"/>
-      <c r="S37" s="52"/>
-      <c r="T37" s="52"/>
-      <c r="U37" s="52"/>
-      <c r="V37" s="52"/>
-      <c r="W37" s="52"/>
-      <c r="X37" s="52"/>
-      <c r="Y37" s="52"/>
-      <c r="Z37" s="52"/>
-      <c r="AA37" s="52"/>
-      <c r="AB37" s="53"/>
+      <c r="H37" s="49"/>
+      <c r="I37" s="50"/>
+      <c r="J37" s="50"/>
+      <c r="K37" s="50"/>
+      <c r="L37" s="50"/>
+      <c r="M37" s="50"/>
+      <c r="N37" s="50"/>
+      <c r="O37" s="50"/>
+      <c r="P37" s="50"/>
+      <c r="Q37" s="50"/>
+      <c r="R37" s="50"/>
+      <c r="S37" s="50"/>
+      <c r="T37" s="50"/>
+      <c r="U37" s="50"/>
+      <c r="V37" s="50"/>
+      <c r="W37" s="50"/>
+      <c r="X37" s="50"/>
+      <c r="Y37" s="50"/>
+      <c r="Z37" s="50"/>
+      <c r="AA37" s="50"/>
+      <c r="AB37" s="51"/>
       <c r="AC37" s="16"/>
     </row>
     <row r="38" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9412,27 +9430,27 @@
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
-      <c r="H38" s="51"/>
-      <c r="I38" s="52"/>
-      <c r="J38" s="52"/>
-      <c r="K38" s="52"/>
-      <c r="L38" s="52"/>
-      <c r="M38" s="52"/>
-      <c r="N38" s="52"/>
-      <c r="O38" s="52"/>
-      <c r="P38" s="52"/>
-      <c r="Q38" s="52"/>
-      <c r="R38" s="52"/>
-      <c r="S38" s="52"/>
-      <c r="T38" s="52"/>
-      <c r="U38" s="52"/>
-      <c r="V38" s="52"/>
-      <c r="W38" s="52"/>
-      <c r="X38" s="52"/>
-      <c r="Y38" s="52"/>
-      <c r="Z38" s="52"/>
-      <c r="AA38" s="52"/>
-      <c r="AB38" s="53"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="50"/>
+      <c r="J38" s="50"/>
+      <c r="K38" s="50"/>
+      <c r="L38" s="50"/>
+      <c r="M38" s="50"/>
+      <c r="N38" s="50"/>
+      <c r="O38" s="50"/>
+      <c r="P38" s="50"/>
+      <c r="Q38" s="50"/>
+      <c r="R38" s="50"/>
+      <c r="S38" s="50"/>
+      <c r="T38" s="50"/>
+      <c r="U38" s="50"/>
+      <c r="V38" s="50"/>
+      <c r="W38" s="50"/>
+      <c r="X38" s="50"/>
+      <c r="Y38" s="50"/>
+      <c r="Z38" s="50"/>
+      <c r="AA38" s="50"/>
+      <c r="AB38" s="51"/>
       <c r="AC38" s="16"/>
     </row>
     <row r="39" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9442,27 +9460,27 @@
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="19"/>
-      <c r="H39" s="51"/>
-      <c r="I39" s="52"/>
-      <c r="J39" s="52"/>
-      <c r="K39" s="52"/>
-      <c r="L39" s="52"/>
-      <c r="M39" s="52"/>
-      <c r="N39" s="52"/>
-      <c r="O39" s="52"/>
-      <c r="P39" s="52"/>
-      <c r="Q39" s="52"/>
-      <c r="R39" s="52"/>
-      <c r="S39" s="52"/>
-      <c r="T39" s="52"/>
-      <c r="U39" s="52"/>
-      <c r="V39" s="52"/>
-      <c r="W39" s="52"/>
-      <c r="X39" s="52"/>
-      <c r="Y39" s="52"/>
-      <c r="Z39" s="52"/>
-      <c r="AA39" s="52"/>
-      <c r="AB39" s="53"/>
+      <c r="H39" s="49"/>
+      <c r="I39" s="50"/>
+      <c r="J39" s="50"/>
+      <c r="K39" s="50"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="50"/>
+      <c r="Q39" s="50"/>
+      <c r="R39" s="50"/>
+      <c r="S39" s="50"/>
+      <c r="T39" s="50"/>
+      <c r="U39" s="50"/>
+      <c r="V39" s="50"/>
+      <c r="W39" s="50"/>
+      <c r="X39" s="50"/>
+      <c r="Y39" s="50"/>
+      <c r="Z39" s="50"/>
+      <c r="AA39" s="50"/>
+      <c r="AB39" s="51"/>
       <c r="AC39" s="16"/>
     </row>
     <row r="40" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9472,27 +9490,27 @@
       <c r="E40" s="19"/>
       <c r="F40" s="19"/>
       <c r="G40" s="19"/>
-      <c r="H40" s="54"/>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
-      <c r="K40" s="55"/>
-      <c r="L40" s="55"/>
-      <c r="M40" s="55"/>
-      <c r="N40" s="55"/>
-      <c r="O40" s="55"/>
-      <c r="P40" s="55"/>
-      <c r="Q40" s="55"/>
-      <c r="R40" s="55"/>
-      <c r="S40" s="55"/>
-      <c r="T40" s="55"/>
-      <c r="U40" s="55"/>
-      <c r="V40" s="55"/>
-      <c r="W40" s="55"/>
-      <c r="X40" s="55"/>
-      <c r="Y40" s="55"/>
-      <c r="Z40" s="55"/>
-      <c r="AA40" s="55"/>
-      <c r="AB40" s="56"/>
+      <c r="H40" s="52"/>
+      <c r="I40" s="53"/>
+      <c r="J40" s="53"/>
+      <c r="K40" s="53"/>
+      <c r="L40" s="53"/>
+      <c r="M40" s="53"/>
+      <c r="N40" s="53"/>
+      <c r="O40" s="53"/>
+      <c r="P40" s="53"/>
+      <c r="Q40" s="53"/>
+      <c r="R40" s="53"/>
+      <c r="S40" s="53"/>
+      <c r="T40" s="53"/>
+      <c r="U40" s="53"/>
+      <c r="V40" s="53"/>
+      <c r="W40" s="53"/>
+      <c r="X40" s="53"/>
+      <c r="Y40" s="53"/>
+      <c r="Z40" s="53"/>
+      <c r="AA40" s="53"/>
+      <c r="AB40" s="54"/>
       <c r="AC40" s="16"/>
     </row>
     <row r="41" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9534,27 +9552,27 @@
       <c r="E42" s="19"/>
       <c r="F42" s="19"/>
       <c r="G42" s="19"/>
-      <c r="H42" s="48"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="49"/>
-      <c r="K42" s="49"/>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
-      <c r="N42" s="49"/>
-      <c r="O42" s="49"/>
-      <c r="P42" s="49"/>
-      <c r="Q42" s="49"/>
-      <c r="R42" s="49"/>
-      <c r="S42" s="49"/>
-      <c r="T42" s="49"/>
-      <c r="U42" s="49"/>
-      <c r="V42" s="49"/>
-      <c r="W42" s="49"/>
-      <c r="X42" s="49"/>
-      <c r="Y42" s="49"/>
-      <c r="Z42" s="49"/>
-      <c r="AA42" s="49"/>
-      <c r="AB42" s="50"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47"/>
+      <c r="K42" s="47"/>
+      <c r="L42" s="47"/>
+      <c r="M42" s="47"/>
+      <c r="N42" s="47"/>
+      <c r="O42" s="47"/>
+      <c r="P42" s="47"/>
+      <c r="Q42" s="47"/>
+      <c r="R42" s="47"/>
+      <c r="S42" s="47"/>
+      <c r="T42" s="47"/>
+      <c r="U42" s="47"/>
+      <c r="V42" s="47"/>
+      <c r="W42" s="47"/>
+      <c r="X42" s="47"/>
+      <c r="Y42" s="47"/>
+      <c r="Z42" s="47"/>
+      <c r="AA42" s="47"/>
+      <c r="AB42" s="48"/>
       <c r="AC42" s="16"/>
     </row>
     <row r="43" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9564,27 +9582,27 @@
       <c r="E43" s="19"/>
       <c r="F43" s="19"/>
       <c r="G43" s="19"/>
-      <c r="H43" s="51"/>
-      <c r="I43" s="52"/>
-      <c r="J43" s="52"/>
-      <c r="K43" s="52"/>
-      <c r="L43" s="52"/>
-      <c r="M43" s="52"/>
-      <c r="N43" s="52"/>
-      <c r="O43" s="52"/>
-      <c r="P43" s="52"/>
-      <c r="Q43" s="52"/>
-      <c r="R43" s="52"/>
-      <c r="S43" s="52"/>
-      <c r="T43" s="52"/>
-      <c r="U43" s="52"/>
-      <c r="V43" s="52"/>
-      <c r="W43" s="52"/>
-      <c r="X43" s="52"/>
-      <c r="Y43" s="52"/>
-      <c r="Z43" s="52"/>
-      <c r="AA43" s="52"/>
-      <c r="AB43" s="53"/>
+      <c r="H43" s="49"/>
+      <c r="I43" s="50"/>
+      <c r="J43" s="50"/>
+      <c r="K43" s="50"/>
+      <c r="L43" s="50"/>
+      <c r="M43" s="50"/>
+      <c r="N43" s="50"/>
+      <c r="O43" s="50"/>
+      <c r="P43" s="50"/>
+      <c r="Q43" s="50"/>
+      <c r="R43" s="50"/>
+      <c r="S43" s="50"/>
+      <c r="T43" s="50"/>
+      <c r="U43" s="50"/>
+      <c r="V43" s="50"/>
+      <c r="W43" s="50"/>
+      <c r="X43" s="50"/>
+      <c r="Y43" s="50"/>
+      <c r="Z43" s="50"/>
+      <c r="AA43" s="50"/>
+      <c r="AB43" s="51"/>
       <c r="AC43" s="16"/>
     </row>
     <row r="44" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9594,27 +9612,27 @@
       <c r="E44" s="19"/>
       <c r="F44" s="19"/>
       <c r="G44" s="19"/>
-      <c r="H44" s="51"/>
-      <c r="I44" s="52"/>
-      <c r="J44" s="52"/>
-      <c r="K44" s="52"/>
-      <c r="L44" s="52"/>
-      <c r="M44" s="52"/>
-      <c r="N44" s="52"/>
-      <c r="O44" s="52"/>
-      <c r="P44" s="52"/>
-      <c r="Q44" s="52"/>
-      <c r="R44" s="52"/>
-      <c r="S44" s="52"/>
-      <c r="T44" s="52"/>
-      <c r="U44" s="52"/>
-      <c r="V44" s="52"/>
-      <c r="W44" s="52"/>
-      <c r="X44" s="52"/>
-      <c r="Y44" s="52"/>
-      <c r="Z44" s="52"/>
-      <c r="AA44" s="52"/>
-      <c r="AB44" s="53"/>
+      <c r="H44" s="49"/>
+      <c r="I44" s="50"/>
+      <c r="J44" s="50"/>
+      <c r="K44" s="50"/>
+      <c r="L44" s="50"/>
+      <c r="M44" s="50"/>
+      <c r="N44" s="50"/>
+      <c r="O44" s="50"/>
+      <c r="P44" s="50"/>
+      <c r="Q44" s="50"/>
+      <c r="R44" s="50"/>
+      <c r="S44" s="50"/>
+      <c r="T44" s="50"/>
+      <c r="U44" s="50"/>
+      <c r="V44" s="50"/>
+      <c r="W44" s="50"/>
+      <c r="X44" s="50"/>
+      <c r="Y44" s="50"/>
+      <c r="Z44" s="50"/>
+      <c r="AA44" s="50"/>
+      <c r="AB44" s="51"/>
       <c r="AC44" s="16"/>
     </row>
     <row r="45" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9624,27 +9642,27 @@
       <c r="E45" s="19"/>
       <c r="F45" s="19"/>
       <c r="G45" s="19"/>
-      <c r="H45" s="51"/>
-      <c r="I45" s="52"/>
-      <c r="J45" s="52"/>
-      <c r="K45" s="52"/>
-      <c r="L45" s="52"/>
-      <c r="M45" s="52"/>
-      <c r="N45" s="52"/>
-      <c r="O45" s="52"/>
-      <c r="P45" s="52"/>
-      <c r="Q45" s="52"/>
-      <c r="R45" s="52"/>
-      <c r="S45" s="52"/>
-      <c r="T45" s="52"/>
-      <c r="U45" s="52"/>
-      <c r="V45" s="52"/>
-      <c r="W45" s="52"/>
-      <c r="X45" s="52"/>
-      <c r="Y45" s="52"/>
-      <c r="Z45" s="52"/>
-      <c r="AA45" s="52"/>
-      <c r="AB45" s="53"/>
+      <c r="H45" s="49"/>
+      <c r="I45" s="50"/>
+      <c r="J45" s="50"/>
+      <c r="K45" s="50"/>
+      <c r="L45" s="50"/>
+      <c r="M45" s="50"/>
+      <c r="N45" s="50"/>
+      <c r="O45" s="50"/>
+      <c r="P45" s="50"/>
+      <c r="Q45" s="50"/>
+      <c r="R45" s="50"/>
+      <c r="S45" s="50"/>
+      <c r="T45" s="50"/>
+      <c r="U45" s="50"/>
+      <c r="V45" s="50"/>
+      <c r="W45" s="50"/>
+      <c r="X45" s="50"/>
+      <c r="Y45" s="50"/>
+      <c r="Z45" s="50"/>
+      <c r="AA45" s="50"/>
+      <c r="AB45" s="51"/>
       <c r="AC45" s="16"/>
     </row>
     <row r="46" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9654,27 +9672,27 @@
       <c r="E46" s="19"/>
       <c r="F46" s="19"/>
       <c r="G46" s="19"/>
-      <c r="H46" s="51"/>
-      <c r="I46" s="52"/>
-      <c r="J46" s="52"/>
-      <c r="K46" s="52"/>
-      <c r="L46" s="52"/>
-      <c r="M46" s="52"/>
-      <c r="N46" s="52"/>
-      <c r="O46" s="52"/>
-      <c r="P46" s="52"/>
-      <c r="Q46" s="52"/>
-      <c r="R46" s="52"/>
-      <c r="S46" s="52"/>
-      <c r="T46" s="52"/>
-      <c r="U46" s="52"/>
-      <c r="V46" s="52"/>
-      <c r="W46" s="52"/>
-      <c r="X46" s="52"/>
-      <c r="Y46" s="52"/>
-      <c r="Z46" s="52"/>
-      <c r="AA46" s="52"/>
-      <c r="AB46" s="53"/>
+      <c r="H46" s="49"/>
+      <c r="I46" s="50"/>
+      <c r="J46" s="50"/>
+      <c r="K46" s="50"/>
+      <c r="L46" s="50"/>
+      <c r="M46" s="50"/>
+      <c r="N46" s="50"/>
+      <c r="O46" s="50"/>
+      <c r="P46" s="50"/>
+      <c r="Q46" s="50"/>
+      <c r="R46" s="50"/>
+      <c r="S46" s="50"/>
+      <c r="T46" s="50"/>
+      <c r="U46" s="50"/>
+      <c r="V46" s="50"/>
+      <c r="W46" s="50"/>
+      <c r="X46" s="50"/>
+      <c r="Y46" s="50"/>
+      <c r="Z46" s="50"/>
+      <c r="AA46" s="50"/>
+      <c r="AB46" s="51"/>
       <c r="AC46" s="16"/>
     </row>
     <row r="47" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9684,27 +9702,27 @@
       <c r="E47" s="19"/>
       <c r="F47" s="19"/>
       <c r="G47" s="19"/>
-      <c r="H47" s="51"/>
-      <c r="I47" s="52"/>
-      <c r="J47" s="52"/>
-      <c r="K47" s="52"/>
-      <c r="L47" s="52"/>
-      <c r="M47" s="52"/>
-      <c r="N47" s="52"/>
-      <c r="O47" s="52"/>
-      <c r="P47" s="52"/>
-      <c r="Q47" s="52"/>
-      <c r="R47" s="52"/>
-      <c r="S47" s="52"/>
-      <c r="T47" s="52"/>
-      <c r="U47" s="52"/>
-      <c r="V47" s="52"/>
-      <c r="W47" s="52"/>
-      <c r="X47" s="52"/>
-      <c r="Y47" s="52"/>
-      <c r="Z47" s="52"/>
-      <c r="AA47" s="52"/>
-      <c r="AB47" s="53"/>
+      <c r="H47" s="49"/>
+      <c r="I47" s="50"/>
+      <c r="J47" s="50"/>
+      <c r="K47" s="50"/>
+      <c r="L47" s="50"/>
+      <c r="M47" s="50"/>
+      <c r="N47" s="50"/>
+      <c r="O47" s="50"/>
+      <c r="P47" s="50"/>
+      <c r="Q47" s="50"/>
+      <c r="R47" s="50"/>
+      <c r="S47" s="50"/>
+      <c r="T47" s="50"/>
+      <c r="U47" s="50"/>
+      <c r="V47" s="50"/>
+      <c r="W47" s="50"/>
+      <c r="X47" s="50"/>
+      <c r="Y47" s="50"/>
+      <c r="Z47" s="50"/>
+      <c r="AA47" s="50"/>
+      <c r="AB47" s="51"/>
       <c r="AC47" s="16"/>
     </row>
     <row r="48" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9714,27 +9732,27 @@
       <c r="E48" s="19"/>
       <c r="F48" s="19"/>
       <c r="G48" s="19"/>
-      <c r="H48" s="54"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="55"/>
-      <c r="L48" s="55"/>
-      <c r="M48" s="55"/>
-      <c r="N48" s="55"/>
-      <c r="O48" s="55"/>
-      <c r="P48" s="55"/>
-      <c r="Q48" s="55"/>
-      <c r="R48" s="55"/>
-      <c r="S48" s="55"/>
-      <c r="T48" s="55"/>
-      <c r="U48" s="55"/>
-      <c r="V48" s="55"/>
-      <c r="W48" s="55"/>
-      <c r="X48" s="55"/>
-      <c r="Y48" s="55"/>
-      <c r="Z48" s="55"/>
-      <c r="AA48" s="55"/>
-      <c r="AB48" s="56"/>
+      <c r="H48" s="52"/>
+      <c r="I48" s="53"/>
+      <c r="J48" s="53"/>
+      <c r="K48" s="53"/>
+      <c r="L48" s="53"/>
+      <c r="M48" s="53"/>
+      <c r="N48" s="53"/>
+      <c r="O48" s="53"/>
+      <c r="P48" s="53"/>
+      <c r="Q48" s="53"/>
+      <c r="R48" s="53"/>
+      <c r="S48" s="53"/>
+      <c r="T48" s="53"/>
+      <c r="U48" s="53"/>
+      <c r="V48" s="53"/>
+      <c r="W48" s="53"/>
+      <c r="X48" s="53"/>
+      <c r="Y48" s="53"/>
+      <c r="Z48" s="53"/>
+      <c r="AA48" s="53"/>
+      <c r="AB48" s="54"/>
       <c r="AC48" s="16"/>
     </row>
     <row r="49" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9807,11 +9825,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>28</v>
       </c>
@@ -10616,11 +10634,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>33</v>
       </c>
@@ -11758,11 +11776,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>34</v>
       </c>
@@ -14509,6 +14527,19 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B6:B23"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="H8:AB14"/>
+    <mergeCell ref="H16:AB22"/>
+    <mergeCell ref="B26:B43"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="H28:AB34"/>
+    <mergeCell ref="H36:AB42"/>
+    <mergeCell ref="B46:B63"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="H48:AB54"/>
+    <mergeCell ref="H56:AB62"/>
     <mergeCell ref="B66:B83"/>
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="H68:AB74"/>
@@ -14517,19 +14548,6 @@
     <mergeCell ref="D88:F88"/>
     <mergeCell ref="H88:AB94"/>
     <mergeCell ref="H96:AB102"/>
-    <mergeCell ref="B26:B43"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="H28:AB34"/>
-    <mergeCell ref="H36:AB42"/>
-    <mergeCell ref="B46:B63"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="H48:AB54"/>
-    <mergeCell ref="H56:AB62"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B6:B23"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="H8:AB14"/>
-    <mergeCell ref="H16:AB22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -14556,11 +14574,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="56"/>
       <c r="I3" s="23" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
0.9 (5.1.1.8/5.1.1.9) Foto anzeigen/aufnehmen
</commit_message>
<xml_diff>
--- a/Projekttagebuch.xlsx
+++ b/Projekttagebuch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\projects\GW.Demo.Maui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DBF2A8D-30D6-4535-A3DB-09311CFBC2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B32E5BF-8CBF-4B81-BAA6-CAE5C42A590F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1DD67F99-F2FF-45C7-A69A-922EBC32F5C0}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="77">
   <si>
     <t>Framework:</t>
   </si>
@@ -300,6 +300,32 @@
   </si>
   <si>
     <t>MediaElement ist eher komfortabel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/image
+https://stackoverflow.com/questions/78133978/loading-images-from-a-folder-in-net-maui
+https://dev.to/serhii_korol_ab7776c50dba/working-with-files-in-net-maui-537n
+https://learn.microsoft.com/en-us/answers/questions/1024872/how-to-save-image-in-while-image-is-taken-from-cam
+https://learn.microsoft.com/en-us/dotnet/maui/platform-integration/storage/file-system-helpers
+</t>
+  </si>
+  <si>
+    <t>VM bereits vorbereitet für Erweiterung. Anzeige umgesetzt.</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://learn.microsoft.com/en-us/answers/questions/1024872/how-to-save-image-in-while-image-is-taken-from-cam
+https://learn.microsoft.com/en-us/dotnet/maui/platform-integration/device-media/picker
+https://learn.microsoft.com/en-us/dotnet/communitytoolkit/maui/views/camera-view
+</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>Konfiguration war tricky.</t>
   </si>
 </sst>
 </file>
@@ -631,6 +657,12 @@
     <xf numFmtId="49" fontId="1" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -657,12 +689,6 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2196,11 +2222,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>11</v>
       </c>
@@ -6254,33 +6280,37 @@
     <row r="144" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B144" s="44"/>
       <c r="C144" s="5"/>
-      <c r="D144" s="41"/>
+      <c r="D144" s="41" t="s">
+        <v>73</v>
+      </c>
       <c r="E144" s="42"/>
       <c r="F144" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G144" s="6"/>
-      <c r="H144" s="46"/>
-      <c r="I144" s="47"/>
-      <c r="J144" s="47"/>
-      <c r="K144" s="47"/>
-      <c r="L144" s="47"/>
-      <c r="M144" s="47"/>
-      <c r="N144" s="47"/>
-      <c r="O144" s="47"/>
-      <c r="P144" s="47"/>
-      <c r="Q144" s="47"/>
-      <c r="R144" s="47"/>
-      <c r="S144" s="47"/>
-      <c r="T144" s="47"/>
-      <c r="U144" s="47"/>
-      <c r="V144" s="47"/>
-      <c r="W144" s="47"/>
-      <c r="X144" s="47"/>
-      <c r="Y144" s="47"/>
-      <c r="Z144" s="47"/>
-      <c r="AA144" s="47"/>
-      <c r="AB144" s="48"/>
+      <c r="H144" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I144" s="33"/>
+      <c r="J144" s="33"/>
+      <c r="K144" s="33"/>
+      <c r="L144" s="33"/>
+      <c r="M144" s="33"/>
+      <c r="N144" s="33"/>
+      <c r="O144" s="33"/>
+      <c r="P144" s="33"/>
+      <c r="Q144" s="33"/>
+      <c r="R144" s="33"/>
+      <c r="S144" s="33"/>
+      <c r="T144" s="33"/>
+      <c r="U144" s="33"/>
+      <c r="V144" s="33"/>
+      <c r="W144" s="33"/>
+      <c r="X144" s="33"/>
+      <c r="Y144" s="33"/>
+      <c r="Z144" s="33"/>
+      <c r="AA144" s="33"/>
+      <c r="AB144" s="34"/>
       <c r="AC144" s="11"/>
     </row>
     <row r="145" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6290,27 +6320,27 @@
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
       <c r="G145" s="6"/>
-      <c r="H145" s="49"/>
-      <c r="I145" s="50"/>
-      <c r="J145" s="50"/>
-      <c r="K145" s="50"/>
-      <c r="L145" s="50"/>
-      <c r="M145" s="50"/>
-      <c r="N145" s="50"/>
-      <c r="O145" s="50"/>
-      <c r="P145" s="50"/>
-      <c r="Q145" s="50"/>
-      <c r="R145" s="50"/>
-      <c r="S145" s="50"/>
-      <c r="T145" s="50"/>
-      <c r="U145" s="50"/>
-      <c r="V145" s="50"/>
-      <c r="W145" s="50"/>
-      <c r="X145" s="50"/>
-      <c r="Y145" s="50"/>
-      <c r="Z145" s="50"/>
-      <c r="AA145" s="50"/>
-      <c r="AB145" s="51"/>
+      <c r="H145" s="35"/>
+      <c r="I145" s="36"/>
+      <c r="J145" s="36"/>
+      <c r="K145" s="36"/>
+      <c r="L145" s="36"/>
+      <c r="M145" s="36"/>
+      <c r="N145" s="36"/>
+      <c r="O145" s="36"/>
+      <c r="P145" s="36"/>
+      <c r="Q145" s="36"/>
+      <c r="R145" s="36"/>
+      <c r="S145" s="36"/>
+      <c r="T145" s="36"/>
+      <c r="U145" s="36"/>
+      <c r="V145" s="36"/>
+      <c r="W145" s="36"/>
+      <c r="X145" s="36"/>
+      <c r="Y145" s="36"/>
+      <c r="Z145" s="36"/>
+      <c r="AA145" s="36"/>
+      <c r="AB145" s="37"/>
       <c r="AC145" s="11"/>
     </row>
     <row r="146" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6320,27 +6350,27 @@
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
       <c r="G146" s="6"/>
-      <c r="H146" s="49"/>
-      <c r="I146" s="50"/>
-      <c r="J146" s="50"/>
-      <c r="K146" s="50"/>
-      <c r="L146" s="50"/>
-      <c r="M146" s="50"/>
-      <c r="N146" s="50"/>
-      <c r="O146" s="50"/>
-      <c r="P146" s="50"/>
-      <c r="Q146" s="50"/>
-      <c r="R146" s="50"/>
-      <c r="S146" s="50"/>
-      <c r="T146" s="50"/>
-      <c r="U146" s="50"/>
-      <c r="V146" s="50"/>
-      <c r="W146" s="50"/>
-      <c r="X146" s="50"/>
-      <c r="Y146" s="50"/>
-      <c r="Z146" s="50"/>
-      <c r="AA146" s="50"/>
-      <c r="AB146" s="51"/>
+      <c r="H146" s="35"/>
+      <c r="I146" s="36"/>
+      <c r="J146" s="36"/>
+      <c r="K146" s="36"/>
+      <c r="L146" s="36"/>
+      <c r="M146" s="36"/>
+      <c r="N146" s="36"/>
+      <c r="O146" s="36"/>
+      <c r="P146" s="36"/>
+      <c r="Q146" s="36"/>
+      <c r="R146" s="36"/>
+      <c r="S146" s="36"/>
+      <c r="T146" s="36"/>
+      <c r="U146" s="36"/>
+      <c r="V146" s="36"/>
+      <c r="W146" s="36"/>
+      <c r="X146" s="36"/>
+      <c r="Y146" s="36"/>
+      <c r="Z146" s="36"/>
+      <c r="AA146" s="36"/>
+      <c r="AB146" s="37"/>
       <c r="AC146" s="11"/>
     </row>
     <row r="147" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6350,27 +6380,27 @@
       <c r="E147" s="6"/>
       <c r="F147" s="6"/>
       <c r="G147" s="6"/>
-      <c r="H147" s="49"/>
-      <c r="I147" s="50"/>
-      <c r="J147" s="50"/>
-      <c r="K147" s="50"/>
-      <c r="L147" s="50"/>
-      <c r="M147" s="50"/>
-      <c r="N147" s="50"/>
-      <c r="O147" s="50"/>
-      <c r="P147" s="50"/>
-      <c r="Q147" s="50"/>
-      <c r="R147" s="50"/>
-      <c r="S147" s="50"/>
-      <c r="T147" s="50"/>
-      <c r="U147" s="50"/>
-      <c r="V147" s="50"/>
-      <c r="W147" s="50"/>
-      <c r="X147" s="50"/>
-      <c r="Y147" s="50"/>
-      <c r="Z147" s="50"/>
-      <c r="AA147" s="50"/>
-      <c r="AB147" s="51"/>
+      <c r="H147" s="35"/>
+      <c r="I147" s="36"/>
+      <c r="J147" s="36"/>
+      <c r="K147" s="36"/>
+      <c r="L147" s="36"/>
+      <c r="M147" s="36"/>
+      <c r="N147" s="36"/>
+      <c r="O147" s="36"/>
+      <c r="P147" s="36"/>
+      <c r="Q147" s="36"/>
+      <c r="R147" s="36"/>
+      <c r="S147" s="36"/>
+      <c r="T147" s="36"/>
+      <c r="U147" s="36"/>
+      <c r="V147" s="36"/>
+      <c r="W147" s="36"/>
+      <c r="X147" s="36"/>
+      <c r="Y147" s="36"/>
+      <c r="Z147" s="36"/>
+      <c r="AA147" s="36"/>
+      <c r="AB147" s="37"/>
       <c r="AC147" s="11"/>
     </row>
     <row r="148" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6380,27 +6410,27 @@
       <c r="E148" s="6"/>
       <c r="F148" s="6"/>
       <c r="G148" s="6"/>
-      <c r="H148" s="49"/>
-      <c r="I148" s="50"/>
-      <c r="J148" s="50"/>
-      <c r="K148" s="50"/>
-      <c r="L148" s="50"/>
-      <c r="M148" s="50"/>
-      <c r="N148" s="50"/>
-      <c r="O148" s="50"/>
-      <c r="P148" s="50"/>
-      <c r="Q148" s="50"/>
-      <c r="R148" s="50"/>
-      <c r="S148" s="50"/>
-      <c r="T148" s="50"/>
-      <c r="U148" s="50"/>
-      <c r="V148" s="50"/>
-      <c r="W148" s="50"/>
-      <c r="X148" s="50"/>
-      <c r="Y148" s="50"/>
-      <c r="Z148" s="50"/>
-      <c r="AA148" s="50"/>
-      <c r="AB148" s="51"/>
+      <c r="H148" s="35"/>
+      <c r="I148" s="36"/>
+      <c r="J148" s="36"/>
+      <c r="K148" s="36"/>
+      <c r="L148" s="36"/>
+      <c r="M148" s="36"/>
+      <c r="N148" s="36"/>
+      <c r="O148" s="36"/>
+      <c r="P148" s="36"/>
+      <c r="Q148" s="36"/>
+      <c r="R148" s="36"/>
+      <c r="S148" s="36"/>
+      <c r="T148" s="36"/>
+      <c r="U148" s="36"/>
+      <c r="V148" s="36"/>
+      <c r="W148" s="36"/>
+      <c r="X148" s="36"/>
+      <c r="Y148" s="36"/>
+      <c r="Z148" s="36"/>
+      <c r="AA148" s="36"/>
+      <c r="AB148" s="37"/>
       <c r="AC148" s="11"/>
     </row>
     <row r="149" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6410,27 +6440,27 @@
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
       <c r="G149" s="6"/>
-      <c r="H149" s="49"/>
-      <c r="I149" s="50"/>
-      <c r="J149" s="50"/>
-      <c r="K149" s="50"/>
-      <c r="L149" s="50"/>
-      <c r="M149" s="50"/>
-      <c r="N149" s="50"/>
-      <c r="O149" s="50"/>
-      <c r="P149" s="50"/>
-      <c r="Q149" s="50"/>
-      <c r="R149" s="50"/>
-      <c r="S149" s="50"/>
-      <c r="T149" s="50"/>
-      <c r="U149" s="50"/>
-      <c r="V149" s="50"/>
-      <c r="W149" s="50"/>
-      <c r="X149" s="50"/>
-      <c r="Y149" s="50"/>
-      <c r="Z149" s="50"/>
-      <c r="AA149" s="50"/>
-      <c r="AB149" s="51"/>
+      <c r="H149" s="35"/>
+      <c r="I149" s="36"/>
+      <c r="J149" s="36"/>
+      <c r="K149" s="36"/>
+      <c r="L149" s="36"/>
+      <c r="M149" s="36"/>
+      <c r="N149" s="36"/>
+      <c r="O149" s="36"/>
+      <c r="P149" s="36"/>
+      <c r="Q149" s="36"/>
+      <c r="R149" s="36"/>
+      <c r="S149" s="36"/>
+      <c r="T149" s="36"/>
+      <c r="U149" s="36"/>
+      <c r="V149" s="36"/>
+      <c r="W149" s="36"/>
+      <c r="X149" s="36"/>
+      <c r="Y149" s="36"/>
+      <c r="Z149" s="36"/>
+      <c r="AA149" s="36"/>
+      <c r="AB149" s="37"/>
       <c r="AC149" s="11"/>
     </row>
     <row r="150" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6440,27 +6470,27 @@
       <c r="E150" s="6"/>
       <c r="F150" s="6"/>
       <c r="G150" s="6"/>
-      <c r="H150" s="52"/>
-      <c r="I150" s="53"/>
-      <c r="J150" s="53"/>
-      <c r="K150" s="53"/>
-      <c r="L150" s="53"/>
-      <c r="M150" s="53"/>
-      <c r="N150" s="53"/>
-      <c r="O150" s="53"/>
-      <c r="P150" s="53"/>
-      <c r="Q150" s="53"/>
-      <c r="R150" s="53"/>
-      <c r="S150" s="53"/>
-      <c r="T150" s="53"/>
-      <c r="U150" s="53"/>
-      <c r="V150" s="53"/>
-      <c r="W150" s="53"/>
-      <c r="X150" s="53"/>
-      <c r="Y150" s="53"/>
-      <c r="Z150" s="53"/>
-      <c r="AA150" s="53"/>
-      <c r="AB150" s="54"/>
+      <c r="H150" s="38"/>
+      <c r="I150" s="39"/>
+      <c r="J150" s="39"/>
+      <c r="K150" s="39"/>
+      <c r="L150" s="39"/>
+      <c r="M150" s="39"/>
+      <c r="N150" s="39"/>
+      <c r="O150" s="39"/>
+      <c r="P150" s="39"/>
+      <c r="Q150" s="39"/>
+      <c r="R150" s="39"/>
+      <c r="S150" s="39"/>
+      <c r="T150" s="39"/>
+      <c r="U150" s="39"/>
+      <c r="V150" s="39"/>
+      <c r="W150" s="39"/>
+      <c r="X150" s="39"/>
+      <c r="Y150" s="39"/>
+      <c r="Z150" s="39"/>
+      <c r="AA150" s="39"/>
+      <c r="AB150" s="40"/>
       <c r="AC150" s="11"/>
     </row>
     <row r="151" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6502,27 +6532,29 @@
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6"/>
-      <c r="H152" s="46"/>
-      <c r="I152" s="47"/>
-      <c r="J152" s="47"/>
-      <c r="K152" s="47"/>
-      <c r="L152" s="47"/>
-      <c r="M152" s="47"/>
-      <c r="N152" s="47"/>
-      <c r="O152" s="47"/>
-      <c r="P152" s="47"/>
-      <c r="Q152" s="47"/>
-      <c r="R152" s="47"/>
-      <c r="S152" s="47"/>
-      <c r="T152" s="47"/>
-      <c r="U152" s="47"/>
-      <c r="V152" s="47"/>
-      <c r="W152" s="47"/>
-      <c r="X152" s="47"/>
-      <c r="Y152" s="47"/>
-      <c r="Z152" s="47"/>
-      <c r="AA152" s="47"/>
-      <c r="AB152" s="48"/>
+      <c r="H152" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I152" s="33"/>
+      <c r="J152" s="33"/>
+      <c r="K152" s="33"/>
+      <c r="L152" s="33"/>
+      <c r="M152" s="33"/>
+      <c r="N152" s="33"/>
+      <c r="O152" s="33"/>
+      <c r="P152" s="33"/>
+      <c r="Q152" s="33"/>
+      <c r="R152" s="33"/>
+      <c r="S152" s="33"/>
+      <c r="T152" s="33"/>
+      <c r="U152" s="33"/>
+      <c r="V152" s="33"/>
+      <c r="W152" s="33"/>
+      <c r="X152" s="33"/>
+      <c r="Y152" s="33"/>
+      <c r="Z152" s="33"/>
+      <c r="AA152" s="33"/>
+      <c r="AB152" s="34"/>
       <c r="AC152" s="11"/>
     </row>
     <row r="153" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6532,27 +6564,27 @@
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
       <c r="G153" s="6"/>
-      <c r="H153" s="49"/>
-      <c r="I153" s="50"/>
-      <c r="J153" s="50"/>
-      <c r="K153" s="50"/>
-      <c r="L153" s="50"/>
-      <c r="M153" s="50"/>
-      <c r="N153" s="50"/>
-      <c r="O153" s="50"/>
-      <c r="P153" s="50"/>
-      <c r="Q153" s="50"/>
-      <c r="R153" s="50"/>
-      <c r="S153" s="50"/>
-      <c r="T153" s="50"/>
-      <c r="U153" s="50"/>
-      <c r="V153" s="50"/>
-      <c r="W153" s="50"/>
-      <c r="X153" s="50"/>
-      <c r="Y153" s="50"/>
-      <c r="Z153" s="50"/>
-      <c r="AA153" s="50"/>
-      <c r="AB153" s="51"/>
+      <c r="H153" s="35"/>
+      <c r="I153" s="36"/>
+      <c r="J153" s="36"/>
+      <c r="K153" s="36"/>
+      <c r="L153" s="36"/>
+      <c r="M153" s="36"/>
+      <c r="N153" s="36"/>
+      <c r="O153" s="36"/>
+      <c r="P153" s="36"/>
+      <c r="Q153" s="36"/>
+      <c r="R153" s="36"/>
+      <c r="S153" s="36"/>
+      <c r="T153" s="36"/>
+      <c r="U153" s="36"/>
+      <c r="V153" s="36"/>
+      <c r="W153" s="36"/>
+      <c r="X153" s="36"/>
+      <c r="Y153" s="36"/>
+      <c r="Z153" s="36"/>
+      <c r="AA153" s="36"/>
+      <c r="AB153" s="37"/>
       <c r="AC153" s="11"/>
     </row>
     <row r="154" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6562,27 +6594,27 @@
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
       <c r="G154" s="6"/>
-      <c r="H154" s="49"/>
-      <c r="I154" s="50"/>
-      <c r="J154" s="50"/>
-      <c r="K154" s="50"/>
-      <c r="L154" s="50"/>
-      <c r="M154" s="50"/>
-      <c r="N154" s="50"/>
-      <c r="O154" s="50"/>
-      <c r="P154" s="50"/>
-      <c r="Q154" s="50"/>
-      <c r="R154" s="50"/>
-      <c r="S154" s="50"/>
-      <c r="T154" s="50"/>
-      <c r="U154" s="50"/>
-      <c r="V154" s="50"/>
-      <c r="W154" s="50"/>
-      <c r="X154" s="50"/>
-      <c r="Y154" s="50"/>
-      <c r="Z154" s="50"/>
-      <c r="AA154" s="50"/>
-      <c r="AB154" s="51"/>
+      <c r="H154" s="35"/>
+      <c r="I154" s="36"/>
+      <c r="J154" s="36"/>
+      <c r="K154" s="36"/>
+      <c r="L154" s="36"/>
+      <c r="M154" s="36"/>
+      <c r="N154" s="36"/>
+      <c r="O154" s="36"/>
+      <c r="P154" s="36"/>
+      <c r="Q154" s="36"/>
+      <c r="R154" s="36"/>
+      <c r="S154" s="36"/>
+      <c r="T154" s="36"/>
+      <c r="U154" s="36"/>
+      <c r="V154" s="36"/>
+      <c r="W154" s="36"/>
+      <c r="X154" s="36"/>
+      <c r="Y154" s="36"/>
+      <c r="Z154" s="36"/>
+      <c r="AA154" s="36"/>
+      <c r="AB154" s="37"/>
       <c r="AC154" s="11"/>
     </row>
     <row r="155" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6592,27 +6624,27 @@
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
       <c r="G155" s="6"/>
-      <c r="H155" s="49"/>
-      <c r="I155" s="50"/>
-      <c r="J155" s="50"/>
-      <c r="K155" s="50"/>
-      <c r="L155" s="50"/>
-      <c r="M155" s="50"/>
-      <c r="N155" s="50"/>
-      <c r="O155" s="50"/>
-      <c r="P155" s="50"/>
-      <c r="Q155" s="50"/>
-      <c r="R155" s="50"/>
-      <c r="S155" s="50"/>
-      <c r="T155" s="50"/>
-      <c r="U155" s="50"/>
-      <c r="V155" s="50"/>
-      <c r="W155" s="50"/>
-      <c r="X155" s="50"/>
-      <c r="Y155" s="50"/>
-      <c r="Z155" s="50"/>
-      <c r="AA155" s="50"/>
-      <c r="AB155" s="51"/>
+      <c r="H155" s="35"/>
+      <c r="I155" s="36"/>
+      <c r="J155" s="36"/>
+      <c r="K155" s="36"/>
+      <c r="L155" s="36"/>
+      <c r="M155" s="36"/>
+      <c r="N155" s="36"/>
+      <c r="O155" s="36"/>
+      <c r="P155" s="36"/>
+      <c r="Q155" s="36"/>
+      <c r="R155" s="36"/>
+      <c r="S155" s="36"/>
+      <c r="T155" s="36"/>
+      <c r="U155" s="36"/>
+      <c r="V155" s="36"/>
+      <c r="W155" s="36"/>
+      <c r="X155" s="36"/>
+      <c r="Y155" s="36"/>
+      <c r="Z155" s="36"/>
+      <c r="AA155" s="36"/>
+      <c r="AB155" s="37"/>
       <c r="AC155" s="11"/>
     </row>
     <row r="156" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6622,27 +6654,27 @@
       <c r="E156" s="6"/>
       <c r="F156" s="6"/>
       <c r="G156" s="6"/>
-      <c r="H156" s="49"/>
-      <c r="I156" s="50"/>
-      <c r="J156" s="50"/>
-      <c r="K156" s="50"/>
-      <c r="L156" s="50"/>
-      <c r="M156" s="50"/>
-      <c r="N156" s="50"/>
-      <c r="O156" s="50"/>
-      <c r="P156" s="50"/>
-      <c r="Q156" s="50"/>
-      <c r="R156" s="50"/>
-      <c r="S156" s="50"/>
-      <c r="T156" s="50"/>
-      <c r="U156" s="50"/>
-      <c r="V156" s="50"/>
-      <c r="W156" s="50"/>
-      <c r="X156" s="50"/>
-      <c r="Y156" s="50"/>
-      <c r="Z156" s="50"/>
-      <c r="AA156" s="50"/>
-      <c r="AB156" s="51"/>
+      <c r="H156" s="35"/>
+      <c r="I156" s="36"/>
+      <c r="J156" s="36"/>
+      <c r="K156" s="36"/>
+      <c r="L156" s="36"/>
+      <c r="M156" s="36"/>
+      <c r="N156" s="36"/>
+      <c r="O156" s="36"/>
+      <c r="P156" s="36"/>
+      <c r="Q156" s="36"/>
+      <c r="R156" s="36"/>
+      <c r="S156" s="36"/>
+      <c r="T156" s="36"/>
+      <c r="U156" s="36"/>
+      <c r="V156" s="36"/>
+      <c r="W156" s="36"/>
+      <c r="X156" s="36"/>
+      <c r="Y156" s="36"/>
+      <c r="Z156" s="36"/>
+      <c r="AA156" s="36"/>
+      <c r="AB156" s="37"/>
       <c r="AC156" s="11"/>
     </row>
     <row r="157" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6652,27 +6684,27 @@
       <c r="E157" s="6"/>
       <c r="F157" s="6"/>
       <c r="G157" s="6"/>
-      <c r="H157" s="49"/>
-      <c r="I157" s="50"/>
-      <c r="J157" s="50"/>
-      <c r="K157" s="50"/>
-      <c r="L157" s="50"/>
-      <c r="M157" s="50"/>
-      <c r="N157" s="50"/>
-      <c r="O157" s="50"/>
-      <c r="P157" s="50"/>
-      <c r="Q157" s="50"/>
-      <c r="R157" s="50"/>
-      <c r="S157" s="50"/>
-      <c r="T157" s="50"/>
-      <c r="U157" s="50"/>
-      <c r="V157" s="50"/>
-      <c r="W157" s="50"/>
-      <c r="X157" s="50"/>
-      <c r="Y157" s="50"/>
-      <c r="Z157" s="50"/>
-      <c r="AA157" s="50"/>
-      <c r="AB157" s="51"/>
+      <c r="H157" s="35"/>
+      <c r="I157" s="36"/>
+      <c r="J157" s="36"/>
+      <c r="K157" s="36"/>
+      <c r="L157" s="36"/>
+      <c r="M157" s="36"/>
+      <c r="N157" s="36"/>
+      <c r="O157" s="36"/>
+      <c r="P157" s="36"/>
+      <c r="Q157" s="36"/>
+      <c r="R157" s="36"/>
+      <c r="S157" s="36"/>
+      <c r="T157" s="36"/>
+      <c r="U157" s="36"/>
+      <c r="V157" s="36"/>
+      <c r="W157" s="36"/>
+      <c r="X157" s="36"/>
+      <c r="Y157" s="36"/>
+      <c r="Z157" s="36"/>
+      <c r="AA157" s="36"/>
+      <c r="AB157" s="37"/>
       <c r="AC157" s="11"/>
     </row>
     <row r="158" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6682,27 +6714,27 @@
       <c r="E158" s="6"/>
       <c r="F158" s="6"/>
       <c r="G158" s="6"/>
-      <c r="H158" s="52"/>
-      <c r="I158" s="53"/>
-      <c r="J158" s="53"/>
-      <c r="K158" s="53"/>
-      <c r="L158" s="53"/>
-      <c r="M158" s="53"/>
-      <c r="N158" s="53"/>
-      <c r="O158" s="53"/>
-      <c r="P158" s="53"/>
-      <c r="Q158" s="53"/>
-      <c r="R158" s="53"/>
-      <c r="S158" s="53"/>
-      <c r="T158" s="53"/>
-      <c r="U158" s="53"/>
-      <c r="V158" s="53"/>
-      <c r="W158" s="53"/>
-      <c r="X158" s="53"/>
-      <c r="Y158" s="53"/>
-      <c r="Z158" s="53"/>
-      <c r="AA158" s="53"/>
-      <c r="AB158" s="54"/>
+      <c r="H158" s="38"/>
+      <c r="I158" s="39"/>
+      <c r="J158" s="39"/>
+      <c r="K158" s="39"/>
+      <c r="L158" s="39"/>
+      <c r="M158" s="39"/>
+      <c r="N158" s="39"/>
+      <c r="O158" s="39"/>
+      <c r="P158" s="39"/>
+      <c r="Q158" s="39"/>
+      <c r="R158" s="39"/>
+      <c r="S158" s="39"/>
+      <c r="T158" s="39"/>
+      <c r="U158" s="39"/>
+      <c r="V158" s="39"/>
+      <c r="W158" s="39"/>
+      <c r="X158" s="39"/>
+      <c r="Y158" s="39"/>
+      <c r="Z158" s="39"/>
+      <c r="AA158" s="39"/>
+      <c r="AB158" s="40"/>
       <c r="AC158" s="11"/>
     </row>
     <row r="159" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6804,33 +6836,37 @@
     <row r="163" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B163" s="44"/>
       <c r="C163" s="5"/>
-      <c r="D163" s="41"/>
+      <c r="D163" s="41" t="s">
+        <v>75</v>
+      </c>
       <c r="E163" s="42"/>
       <c r="F163" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G163" s="6"/>
-      <c r="H163" s="46"/>
-      <c r="I163" s="47"/>
-      <c r="J163" s="47"/>
-      <c r="K163" s="47"/>
-      <c r="L163" s="47"/>
-      <c r="M163" s="47"/>
-      <c r="N163" s="47"/>
-      <c r="O163" s="47"/>
-      <c r="P163" s="47"/>
-      <c r="Q163" s="47"/>
-      <c r="R163" s="47"/>
-      <c r="S163" s="47"/>
-      <c r="T163" s="47"/>
-      <c r="U163" s="47"/>
-      <c r="V163" s="47"/>
-      <c r="W163" s="47"/>
-      <c r="X163" s="47"/>
-      <c r="Y163" s="47"/>
-      <c r="Z163" s="47"/>
-      <c r="AA163" s="47"/>
-      <c r="AB163" s="48"/>
+      <c r="H163" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="I163" s="33"/>
+      <c r="J163" s="33"/>
+      <c r="K163" s="33"/>
+      <c r="L163" s="33"/>
+      <c r="M163" s="33"/>
+      <c r="N163" s="33"/>
+      <c r="O163" s="33"/>
+      <c r="P163" s="33"/>
+      <c r="Q163" s="33"/>
+      <c r="R163" s="33"/>
+      <c r="S163" s="33"/>
+      <c r="T163" s="33"/>
+      <c r="U163" s="33"/>
+      <c r="V163" s="33"/>
+      <c r="W163" s="33"/>
+      <c r="X163" s="33"/>
+      <c r="Y163" s="33"/>
+      <c r="Z163" s="33"/>
+      <c r="AA163" s="33"/>
+      <c r="AB163" s="34"/>
       <c r="AC163" s="11"/>
     </row>
     <row r="164" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6840,27 +6876,27 @@
       <c r="E164" s="6"/>
       <c r="F164" s="6"/>
       <c r="G164" s="6"/>
-      <c r="H164" s="49"/>
-      <c r="I164" s="50"/>
-      <c r="J164" s="50"/>
-      <c r="K164" s="50"/>
-      <c r="L164" s="50"/>
-      <c r="M164" s="50"/>
-      <c r="N164" s="50"/>
-      <c r="O164" s="50"/>
-      <c r="P164" s="50"/>
-      <c r="Q164" s="50"/>
-      <c r="R164" s="50"/>
-      <c r="S164" s="50"/>
-      <c r="T164" s="50"/>
-      <c r="U164" s="50"/>
-      <c r="V164" s="50"/>
-      <c r="W164" s="50"/>
-      <c r="X164" s="50"/>
-      <c r="Y164" s="50"/>
-      <c r="Z164" s="50"/>
-      <c r="AA164" s="50"/>
-      <c r="AB164" s="51"/>
+      <c r="H164" s="35"/>
+      <c r="I164" s="36"/>
+      <c r="J164" s="36"/>
+      <c r="K164" s="36"/>
+      <c r="L164" s="36"/>
+      <c r="M164" s="36"/>
+      <c r="N164" s="36"/>
+      <c r="O164" s="36"/>
+      <c r="P164" s="36"/>
+      <c r="Q164" s="36"/>
+      <c r="R164" s="36"/>
+      <c r="S164" s="36"/>
+      <c r="T164" s="36"/>
+      <c r="U164" s="36"/>
+      <c r="V164" s="36"/>
+      <c r="W164" s="36"/>
+      <c r="X164" s="36"/>
+      <c r="Y164" s="36"/>
+      <c r="Z164" s="36"/>
+      <c r="AA164" s="36"/>
+      <c r="AB164" s="37"/>
       <c r="AC164" s="11"/>
     </row>
     <row r="165" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6870,27 +6906,27 @@
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
       <c r="G165" s="6"/>
-      <c r="H165" s="49"/>
-      <c r="I165" s="50"/>
-      <c r="J165" s="50"/>
-      <c r="K165" s="50"/>
-      <c r="L165" s="50"/>
-      <c r="M165" s="50"/>
-      <c r="N165" s="50"/>
-      <c r="O165" s="50"/>
-      <c r="P165" s="50"/>
-      <c r="Q165" s="50"/>
-      <c r="R165" s="50"/>
-      <c r="S165" s="50"/>
-      <c r="T165" s="50"/>
-      <c r="U165" s="50"/>
-      <c r="V165" s="50"/>
-      <c r="W165" s="50"/>
-      <c r="X165" s="50"/>
-      <c r="Y165" s="50"/>
-      <c r="Z165" s="50"/>
-      <c r="AA165" s="50"/>
-      <c r="AB165" s="51"/>
+      <c r="H165" s="35"/>
+      <c r="I165" s="36"/>
+      <c r="J165" s="36"/>
+      <c r="K165" s="36"/>
+      <c r="L165" s="36"/>
+      <c r="M165" s="36"/>
+      <c r="N165" s="36"/>
+      <c r="O165" s="36"/>
+      <c r="P165" s="36"/>
+      <c r="Q165" s="36"/>
+      <c r="R165" s="36"/>
+      <c r="S165" s="36"/>
+      <c r="T165" s="36"/>
+      <c r="U165" s="36"/>
+      <c r="V165" s="36"/>
+      <c r="W165" s="36"/>
+      <c r="X165" s="36"/>
+      <c r="Y165" s="36"/>
+      <c r="Z165" s="36"/>
+      <c r="AA165" s="36"/>
+      <c r="AB165" s="37"/>
       <c r="AC165" s="11"/>
     </row>
     <row r="166" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6900,27 +6936,27 @@
       <c r="E166" s="6"/>
       <c r="F166" s="6"/>
       <c r="G166" s="6"/>
-      <c r="H166" s="49"/>
-      <c r="I166" s="50"/>
-      <c r="J166" s="50"/>
-      <c r="K166" s="50"/>
-      <c r="L166" s="50"/>
-      <c r="M166" s="50"/>
-      <c r="N166" s="50"/>
-      <c r="O166" s="50"/>
-      <c r="P166" s="50"/>
-      <c r="Q166" s="50"/>
-      <c r="R166" s="50"/>
-      <c r="S166" s="50"/>
-      <c r="T166" s="50"/>
-      <c r="U166" s="50"/>
-      <c r="V166" s="50"/>
-      <c r="W166" s="50"/>
-      <c r="X166" s="50"/>
-      <c r="Y166" s="50"/>
-      <c r="Z166" s="50"/>
-      <c r="AA166" s="50"/>
-      <c r="AB166" s="51"/>
+      <c r="H166" s="35"/>
+      <c r="I166" s="36"/>
+      <c r="J166" s="36"/>
+      <c r="K166" s="36"/>
+      <c r="L166" s="36"/>
+      <c r="M166" s="36"/>
+      <c r="N166" s="36"/>
+      <c r="O166" s="36"/>
+      <c r="P166" s="36"/>
+      <c r="Q166" s="36"/>
+      <c r="R166" s="36"/>
+      <c r="S166" s="36"/>
+      <c r="T166" s="36"/>
+      <c r="U166" s="36"/>
+      <c r="V166" s="36"/>
+      <c r="W166" s="36"/>
+      <c r="X166" s="36"/>
+      <c r="Y166" s="36"/>
+      <c r="Z166" s="36"/>
+      <c r="AA166" s="36"/>
+      <c r="AB166" s="37"/>
       <c r="AC166" s="11"/>
     </row>
     <row r="167" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6930,27 +6966,27 @@
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
       <c r="G167" s="6"/>
-      <c r="H167" s="49"/>
-      <c r="I167" s="50"/>
-      <c r="J167" s="50"/>
-      <c r="K167" s="50"/>
-      <c r="L167" s="50"/>
-      <c r="M167" s="50"/>
-      <c r="N167" s="50"/>
-      <c r="O167" s="50"/>
-      <c r="P167" s="50"/>
-      <c r="Q167" s="50"/>
-      <c r="R167" s="50"/>
-      <c r="S167" s="50"/>
-      <c r="T167" s="50"/>
-      <c r="U167" s="50"/>
-      <c r="V167" s="50"/>
-      <c r="W167" s="50"/>
-      <c r="X167" s="50"/>
-      <c r="Y167" s="50"/>
-      <c r="Z167" s="50"/>
-      <c r="AA167" s="50"/>
-      <c r="AB167" s="51"/>
+      <c r="H167" s="35"/>
+      <c r="I167" s="36"/>
+      <c r="J167" s="36"/>
+      <c r="K167" s="36"/>
+      <c r="L167" s="36"/>
+      <c r="M167" s="36"/>
+      <c r="N167" s="36"/>
+      <c r="O167" s="36"/>
+      <c r="P167" s="36"/>
+      <c r="Q167" s="36"/>
+      <c r="R167" s="36"/>
+      <c r="S167" s="36"/>
+      <c r="T167" s="36"/>
+      <c r="U167" s="36"/>
+      <c r="V167" s="36"/>
+      <c r="W167" s="36"/>
+      <c r="X167" s="36"/>
+      <c r="Y167" s="36"/>
+      <c r="Z167" s="36"/>
+      <c r="AA167" s="36"/>
+      <c r="AB167" s="37"/>
       <c r="AC167" s="11"/>
     </row>
     <row r="168" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6960,27 +6996,27 @@
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
       <c r="G168" s="6"/>
-      <c r="H168" s="49"/>
-      <c r="I168" s="50"/>
-      <c r="J168" s="50"/>
-      <c r="K168" s="50"/>
-      <c r="L168" s="50"/>
-      <c r="M168" s="50"/>
-      <c r="N168" s="50"/>
-      <c r="O168" s="50"/>
-      <c r="P168" s="50"/>
-      <c r="Q168" s="50"/>
-      <c r="R168" s="50"/>
-      <c r="S168" s="50"/>
-      <c r="T168" s="50"/>
-      <c r="U168" s="50"/>
-      <c r="V168" s="50"/>
-      <c r="W168" s="50"/>
-      <c r="X168" s="50"/>
-      <c r="Y168" s="50"/>
-      <c r="Z168" s="50"/>
-      <c r="AA168" s="50"/>
-      <c r="AB168" s="51"/>
+      <c r="H168" s="35"/>
+      <c r="I168" s="36"/>
+      <c r="J168" s="36"/>
+      <c r="K168" s="36"/>
+      <c r="L168" s="36"/>
+      <c r="M168" s="36"/>
+      <c r="N168" s="36"/>
+      <c r="O168" s="36"/>
+      <c r="P168" s="36"/>
+      <c r="Q168" s="36"/>
+      <c r="R168" s="36"/>
+      <c r="S168" s="36"/>
+      <c r="T168" s="36"/>
+      <c r="U168" s="36"/>
+      <c r="V168" s="36"/>
+      <c r="W168" s="36"/>
+      <c r="X168" s="36"/>
+      <c r="Y168" s="36"/>
+      <c r="Z168" s="36"/>
+      <c r="AA168" s="36"/>
+      <c r="AB168" s="37"/>
       <c r="AC168" s="11"/>
     </row>
     <row r="169" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6990,27 +7026,27 @@
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
-      <c r="H169" s="52"/>
-      <c r="I169" s="53"/>
-      <c r="J169" s="53"/>
-      <c r="K169" s="53"/>
-      <c r="L169" s="53"/>
-      <c r="M169" s="53"/>
-      <c r="N169" s="53"/>
-      <c r="O169" s="53"/>
-      <c r="P169" s="53"/>
-      <c r="Q169" s="53"/>
-      <c r="R169" s="53"/>
-      <c r="S169" s="53"/>
-      <c r="T169" s="53"/>
-      <c r="U169" s="53"/>
-      <c r="V169" s="53"/>
-      <c r="W169" s="53"/>
-      <c r="X169" s="53"/>
-      <c r="Y169" s="53"/>
-      <c r="Z169" s="53"/>
-      <c r="AA169" s="53"/>
-      <c r="AB169" s="54"/>
+      <c r="H169" s="38"/>
+      <c r="I169" s="39"/>
+      <c r="J169" s="39"/>
+      <c r="K169" s="39"/>
+      <c r="L169" s="39"/>
+      <c r="M169" s="39"/>
+      <c r="N169" s="39"/>
+      <c r="O169" s="39"/>
+      <c r="P169" s="39"/>
+      <c r="Q169" s="39"/>
+      <c r="R169" s="39"/>
+      <c r="S169" s="39"/>
+      <c r="T169" s="39"/>
+      <c r="U169" s="39"/>
+      <c r="V169" s="39"/>
+      <c r="W169" s="39"/>
+      <c r="X169" s="39"/>
+      <c r="Y169" s="39"/>
+      <c r="Z169" s="39"/>
+      <c r="AA169" s="39"/>
+      <c r="AB169" s="40"/>
       <c r="AC169" s="11"/>
     </row>
     <row r="170" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7052,27 +7088,29 @@
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
       <c r="G171" s="6"/>
-      <c r="H171" s="46"/>
-      <c r="I171" s="47"/>
-      <c r="J171" s="47"/>
-      <c r="K171" s="47"/>
-      <c r="L171" s="47"/>
-      <c r="M171" s="47"/>
-      <c r="N171" s="47"/>
-      <c r="O171" s="47"/>
-      <c r="P171" s="47"/>
-      <c r="Q171" s="47"/>
-      <c r="R171" s="47"/>
-      <c r="S171" s="47"/>
-      <c r="T171" s="47"/>
-      <c r="U171" s="47"/>
-      <c r="V171" s="47"/>
-      <c r="W171" s="47"/>
-      <c r="X171" s="47"/>
-      <c r="Y171" s="47"/>
-      <c r="Z171" s="47"/>
-      <c r="AA171" s="47"/>
-      <c r="AB171" s="48"/>
+      <c r="H171" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="I171" s="33"/>
+      <c r="J171" s="33"/>
+      <c r="K171" s="33"/>
+      <c r="L171" s="33"/>
+      <c r="M171" s="33"/>
+      <c r="N171" s="33"/>
+      <c r="O171" s="33"/>
+      <c r="P171" s="33"/>
+      <c r="Q171" s="33"/>
+      <c r="R171" s="33"/>
+      <c r="S171" s="33"/>
+      <c r="T171" s="33"/>
+      <c r="U171" s="33"/>
+      <c r="V171" s="33"/>
+      <c r="W171" s="33"/>
+      <c r="X171" s="33"/>
+      <c r="Y171" s="33"/>
+      <c r="Z171" s="33"/>
+      <c r="AA171" s="33"/>
+      <c r="AB171" s="34"/>
       <c r="AC171" s="11"/>
     </row>
     <row r="172" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7082,27 +7120,27 @@
       <c r="E172" s="6"/>
       <c r="F172" s="6"/>
       <c r="G172" s="6"/>
-      <c r="H172" s="49"/>
-      <c r="I172" s="50"/>
-      <c r="J172" s="50"/>
-      <c r="K172" s="50"/>
-      <c r="L172" s="50"/>
-      <c r="M172" s="50"/>
-      <c r="N172" s="50"/>
-      <c r="O172" s="50"/>
-      <c r="P172" s="50"/>
-      <c r="Q172" s="50"/>
-      <c r="R172" s="50"/>
-      <c r="S172" s="50"/>
-      <c r="T172" s="50"/>
-      <c r="U172" s="50"/>
-      <c r="V172" s="50"/>
-      <c r="W172" s="50"/>
-      <c r="X172" s="50"/>
-      <c r="Y172" s="50"/>
-      <c r="Z172" s="50"/>
-      <c r="AA172" s="50"/>
-      <c r="AB172" s="51"/>
+      <c r="H172" s="35"/>
+      <c r="I172" s="36"/>
+      <c r="J172" s="36"/>
+      <c r="K172" s="36"/>
+      <c r="L172" s="36"/>
+      <c r="M172" s="36"/>
+      <c r="N172" s="36"/>
+      <c r="O172" s="36"/>
+      <c r="P172" s="36"/>
+      <c r="Q172" s="36"/>
+      <c r="R172" s="36"/>
+      <c r="S172" s="36"/>
+      <c r="T172" s="36"/>
+      <c r="U172" s="36"/>
+      <c r="V172" s="36"/>
+      <c r="W172" s="36"/>
+      <c r="X172" s="36"/>
+      <c r="Y172" s="36"/>
+      <c r="Z172" s="36"/>
+      <c r="AA172" s="36"/>
+      <c r="AB172" s="37"/>
       <c r="AC172" s="11"/>
     </row>
     <row r="173" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7112,27 +7150,27 @@
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6"/>
-      <c r="H173" s="49"/>
-      <c r="I173" s="50"/>
-      <c r="J173" s="50"/>
-      <c r="K173" s="50"/>
-      <c r="L173" s="50"/>
-      <c r="M173" s="50"/>
-      <c r="N173" s="50"/>
-      <c r="O173" s="50"/>
-      <c r="P173" s="50"/>
-      <c r="Q173" s="50"/>
-      <c r="R173" s="50"/>
-      <c r="S173" s="50"/>
-      <c r="T173" s="50"/>
-      <c r="U173" s="50"/>
-      <c r="V173" s="50"/>
-      <c r="W173" s="50"/>
-      <c r="X173" s="50"/>
-      <c r="Y173" s="50"/>
-      <c r="Z173" s="50"/>
-      <c r="AA173" s="50"/>
-      <c r="AB173" s="51"/>
+      <c r="H173" s="35"/>
+      <c r="I173" s="36"/>
+      <c r="J173" s="36"/>
+      <c r="K173" s="36"/>
+      <c r="L173" s="36"/>
+      <c r="M173" s="36"/>
+      <c r="N173" s="36"/>
+      <c r="O173" s="36"/>
+      <c r="P173" s="36"/>
+      <c r="Q173" s="36"/>
+      <c r="R173" s="36"/>
+      <c r="S173" s="36"/>
+      <c r="T173" s="36"/>
+      <c r="U173" s="36"/>
+      <c r="V173" s="36"/>
+      <c r="W173" s="36"/>
+      <c r="X173" s="36"/>
+      <c r="Y173" s="36"/>
+      <c r="Z173" s="36"/>
+      <c r="AA173" s="36"/>
+      <c r="AB173" s="37"/>
       <c r="AC173" s="11"/>
     </row>
     <row r="174" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7142,27 +7180,27 @@
       <c r="E174" s="6"/>
       <c r="F174" s="6"/>
       <c r="G174" s="6"/>
-      <c r="H174" s="49"/>
-      <c r="I174" s="50"/>
-      <c r="J174" s="50"/>
-      <c r="K174" s="50"/>
-      <c r="L174" s="50"/>
-      <c r="M174" s="50"/>
-      <c r="N174" s="50"/>
-      <c r="O174" s="50"/>
-      <c r="P174" s="50"/>
-      <c r="Q174" s="50"/>
-      <c r="R174" s="50"/>
-      <c r="S174" s="50"/>
-      <c r="T174" s="50"/>
-      <c r="U174" s="50"/>
-      <c r="V174" s="50"/>
-      <c r="W174" s="50"/>
-      <c r="X174" s="50"/>
-      <c r="Y174" s="50"/>
-      <c r="Z174" s="50"/>
-      <c r="AA174" s="50"/>
-      <c r="AB174" s="51"/>
+      <c r="H174" s="35"/>
+      <c r="I174" s="36"/>
+      <c r="J174" s="36"/>
+      <c r="K174" s="36"/>
+      <c r="L174" s="36"/>
+      <c r="M174" s="36"/>
+      <c r="N174" s="36"/>
+      <c r="O174" s="36"/>
+      <c r="P174" s="36"/>
+      <c r="Q174" s="36"/>
+      <c r="R174" s="36"/>
+      <c r="S174" s="36"/>
+      <c r="T174" s="36"/>
+      <c r="U174" s="36"/>
+      <c r="V174" s="36"/>
+      <c r="W174" s="36"/>
+      <c r="X174" s="36"/>
+      <c r="Y174" s="36"/>
+      <c r="Z174" s="36"/>
+      <c r="AA174" s="36"/>
+      <c r="AB174" s="37"/>
       <c r="AC174" s="11"/>
     </row>
     <row r="175" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7172,27 +7210,27 @@
       <c r="E175" s="6"/>
       <c r="F175" s="6"/>
       <c r="G175" s="6"/>
-      <c r="H175" s="49"/>
-      <c r="I175" s="50"/>
-      <c r="J175" s="50"/>
-      <c r="K175" s="50"/>
-      <c r="L175" s="50"/>
-      <c r="M175" s="50"/>
-      <c r="N175" s="50"/>
-      <c r="O175" s="50"/>
-      <c r="P175" s="50"/>
-      <c r="Q175" s="50"/>
-      <c r="R175" s="50"/>
-      <c r="S175" s="50"/>
-      <c r="T175" s="50"/>
-      <c r="U175" s="50"/>
-      <c r="V175" s="50"/>
-      <c r="W175" s="50"/>
-      <c r="X175" s="50"/>
-      <c r="Y175" s="50"/>
-      <c r="Z175" s="50"/>
-      <c r="AA175" s="50"/>
-      <c r="AB175" s="51"/>
+      <c r="H175" s="35"/>
+      <c r="I175" s="36"/>
+      <c r="J175" s="36"/>
+      <c r="K175" s="36"/>
+      <c r="L175" s="36"/>
+      <c r="M175" s="36"/>
+      <c r="N175" s="36"/>
+      <c r="O175" s="36"/>
+      <c r="P175" s="36"/>
+      <c r="Q175" s="36"/>
+      <c r="R175" s="36"/>
+      <c r="S175" s="36"/>
+      <c r="T175" s="36"/>
+      <c r="U175" s="36"/>
+      <c r="V175" s="36"/>
+      <c r="W175" s="36"/>
+      <c r="X175" s="36"/>
+      <c r="Y175" s="36"/>
+      <c r="Z175" s="36"/>
+      <c r="AA175" s="36"/>
+      <c r="AB175" s="37"/>
       <c r="AC175" s="11"/>
     </row>
     <row r="176" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7202,27 +7240,27 @@
       <c r="E176" s="6"/>
       <c r="F176" s="6"/>
       <c r="G176" s="6"/>
-      <c r="H176" s="49"/>
-      <c r="I176" s="50"/>
-      <c r="J176" s="50"/>
-      <c r="K176" s="50"/>
-      <c r="L176" s="50"/>
-      <c r="M176" s="50"/>
-      <c r="N176" s="50"/>
-      <c r="O176" s="50"/>
-      <c r="P176" s="50"/>
-      <c r="Q176" s="50"/>
-      <c r="R176" s="50"/>
-      <c r="S176" s="50"/>
-      <c r="T176" s="50"/>
-      <c r="U176" s="50"/>
-      <c r="V176" s="50"/>
-      <c r="W176" s="50"/>
-      <c r="X176" s="50"/>
-      <c r="Y176" s="50"/>
-      <c r="Z176" s="50"/>
-      <c r="AA176" s="50"/>
-      <c r="AB176" s="51"/>
+      <c r="H176" s="35"/>
+      <c r="I176" s="36"/>
+      <c r="J176" s="36"/>
+      <c r="K176" s="36"/>
+      <c r="L176" s="36"/>
+      <c r="M176" s="36"/>
+      <c r="N176" s="36"/>
+      <c r="O176" s="36"/>
+      <c r="P176" s="36"/>
+      <c r="Q176" s="36"/>
+      <c r="R176" s="36"/>
+      <c r="S176" s="36"/>
+      <c r="T176" s="36"/>
+      <c r="U176" s="36"/>
+      <c r="V176" s="36"/>
+      <c r="W176" s="36"/>
+      <c r="X176" s="36"/>
+      <c r="Y176" s="36"/>
+      <c r="Z176" s="36"/>
+      <c r="AA176" s="36"/>
+      <c r="AB176" s="37"/>
       <c r="AC176" s="11"/>
     </row>
     <row r="177" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7232,27 +7270,27 @@
       <c r="E177" s="6"/>
       <c r="F177" s="6"/>
       <c r="G177" s="6"/>
-      <c r="H177" s="52"/>
-      <c r="I177" s="53"/>
-      <c r="J177" s="53"/>
-      <c r="K177" s="53"/>
-      <c r="L177" s="53"/>
-      <c r="M177" s="53"/>
-      <c r="N177" s="53"/>
-      <c r="O177" s="53"/>
-      <c r="P177" s="53"/>
-      <c r="Q177" s="53"/>
-      <c r="R177" s="53"/>
-      <c r="S177" s="53"/>
-      <c r="T177" s="53"/>
-      <c r="U177" s="53"/>
-      <c r="V177" s="53"/>
-      <c r="W177" s="53"/>
-      <c r="X177" s="53"/>
-      <c r="Y177" s="53"/>
-      <c r="Z177" s="53"/>
-      <c r="AA177" s="53"/>
-      <c r="AB177" s="54"/>
+      <c r="H177" s="38"/>
+      <c r="I177" s="39"/>
+      <c r="J177" s="39"/>
+      <c r="K177" s="39"/>
+      <c r="L177" s="39"/>
+      <c r="M177" s="39"/>
+      <c r="N177" s="39"/>
+      <c r="O177" s="39"/>
+      <c r="P177" s="39"/>
+      <c r="Q177" s="39"/>
+      <c r="R177" s="39"/>
+      <c r="S177" s="39"/>
+      <c r="T177" s="39"/>
+      <c r="U177" s="39"/>
+      <c r="V177" s="39"/>
+      <c r="W177" s="39"/>
+      <c r="X177" s="39"/>
+      <c r="Y177" s="39"/>
+      <c r="Z177" s="39"/>
+      <c r="AA177" s="39"/>
+      <c r="AB177" s="40"/>
       <c r="AC177" s="11"/>
     </row>
     <row r="178" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7360,27 +7398,27 @@
         <v>2</v>
       </c>
       <c r="G182" s="6"/>
-      <c r="H182" s="46"/>
-      <c r="I182" s="47"/>
-      <c r="J182" s="47"/>
-      <c r="K182" s="47"/>
-      <c r="L182" s="47"/>
-      <c r="M182" s="47"/>
-      <c r="N182" s="47"/>
-      <c r="O182" s="47"/>
-      <c r="P182" s="47"/>
-      <c r="Q182" s="47"/>
-      <c r="R182" s="47"/>
-      <c r="S182" s="47"/>
-      <c r="T182" s="47"/>
-      <c r="U182" s="47"/>
-      <c r="V182" s="47"/>
-      <c r="W182" s="47"/>
-      <c r="X182" s="47"/>
-      <c r="Y182" s="47"/>
-      <c r="Z182" s="47"/>
-      <c r="AA182" s="47"/>
-      <c r="AB182" s="48"/>
+      <c r="H182" s="48"/>
+      <c r="I182" s="49"/>
+      <c r="J182" s="49"/>
+      <c r="K182" s="49"/>
+      <c r="L182" s="49"/>
+      <c r="M182" s="49"/>
+      <c r="N182" s="49"/>
+      <c r="O182" s="49"/>
+      <c r="P182" s="49"/>
+      <c r="Q182" s="49"/>
+      <c r="R182" s="49"/>
+      <c r="S182" s="49"/>
+      <c r="T182" s="49"/>
+      <c r="U182" s="49"/>
+      <c r="V182" s="49"/>
+      <c r="W182" s="49"/>
+      <c r="X182" s="49"/>
+      <c r="Y182" s="49"/>
+      <c r="Z182" s="49"/>
+      <c r="AA182" s="49"/>
+      <c r="AB182" s="50"/>
       <c r="AC182" s="11"/>
     </row>
     <row r="183" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7390,27 +7428,27 @@
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6"/>
-      <c r="H183" s="49"/>
-      <c r="I183" s="50"/>
-      <c r="J183" s="50"/>
-      <c r="K183" s="50"/>
-      <c r="L183" s="50"/>
-      <c r="M183" s="50"/>
-      <c r="N183" s="50"/>
-      <c r="O183" s="50"/>
-      <c r="P183" s="50"/>
-      <c r="Q183" s="50"/>
-      <c r="R183" s="50"/>
-      <c r="S183" s="50"/>
-      <c r="T183" s="50"/>
-      <c r="U183" s="50"/>
-      <c r="V183" s="50"/>
-      <c r="W183" s="50"/>
-      <c r="X183" s="50"/>
-      <c r="Y183" s="50"/>
-      <c r="Z183" s="50"/>
-      <c r="AA183" s="50"/>
-      <c r="AB183" s="51"/>
+      <c r="H183" s="51"/>
+      <c r="I183" s="52"/>
+      <c r="J183" s="52"/>
+      <c r="K183" s="52"/>
+      <c r="L183" s="52"/>
+      <c r="M183" s="52"/>
+      <c r="N183" s="52"/>
+      <c r="O183" s="52"/>
+      <c r="P183" s="52"/>
+      <c r="Q183" s="52"/>
+      <c r="R183" s="52"/>
+      <c r="S183" s="52"/>
+      <c r="T183" s="52"/>
+      <c r="U183" s="52"/>
+      <c r="V183" s="52"/>
+      <c r="W183" s="52"/>
+      <c r="X183" s="52"/>
+      <c r="Y183" s="52"/>
+      <c r="Z183" s="52"/>
+      <c r="AA183" s="52"/>
+      <c r="AB183" s="53"/>
       <c r="AC183" s="11"/>
     </row>
     <row r="184" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7420,27 +7458,27 @@
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
       <c r="G184" s="6"/>
-      <c r="H184" s="49"/>
-      <c r="I184" s="50"/>
-      <c r="J184" s="50"/>
-      <c r="K184" s="50"/>
-      <c r="L184" s="50"/>
-      <c r="M184" s="50"/>
-      <c r="N184" s="50"/>
-      <c r="O184" s="50"/>
-      <c r="P184" s="50"/>
-      <c r="Q184" s="50"/>
-      <c r="R184" s="50"/>
-      <c r="S184" s="50"/>
-      <c r="T184" s="50"/>
-      <c r="U184" s="50"/>
-      <c r="V184" s="50"/>
-      <c r="W184" s="50"/>
-      <c r="X184" s="50"/>
-      <c r="Y184" s="50"/>
-      <c r="Z184" s="50"/>
-      <c r="AA184" s="50"/>
-      <c r="AB184" s="51"/>
+      <c r="H184" s="51"/>
+      <c r="I184" s="52"/>
+      <c r="J184" s="52"/>
+      <c r="K184" s="52"/>
+      <c r="L184" s="52"/>
+      <c r="M184" s="52"/>
+      <c r="N184" s="52"/>
+      <c r="O184" s="52"/>
+      <c r="P184" s="52"/>
+      <c r="Q184" s="52"/>
+      <c r="R184" s="52"/>
+      <c r="S184" s="52"/>
+      <c r="T184" s="52"/>
+      <c r="U184" s="52"/>
+      <c r="V184" s="52"/>
+      <c r="W184" s="52"/>
+      <c r="X184" s="52"/>
+      <c r="Y184" s="52"/>
+      <c r="Z184" s="52"/>
+      <c r="AA184" s="52"/>
+      <c r="AB184" s="53"/>
       <c r="AC184" s="11"/>
     </row>
     <row r="185" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7450,27 +7488,27 @@
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
       <c r="G185" s="6"/>
-      <c r="H185" s="49"/>
-      <c r="I185" s="50"/>
-      <c r="J185" s="50"/>
-      <c r="K185" s="50"/>
-      <c r="L185" s="50"/>
-      <c r="M185" s="50"/>
-      <c r="N185" s="50"/>
-      <c r="O185" s="50"/>
-      <c r="P185" s="50"/>
-      <c r="Q185" s="50"/>
-      <c r="R185" s="50"/>
-      <c r="S185" s="50"/>
-      <c r="T185" s="50"/>
-      <c r="U185" s="50"/>
-      <c r="V185" s="50"/>
-      <c r="W185" s="50"/>
-      <c r="X185" s="50"/>
-      <c r="Y185" s="50"/>
-      <c r="Z185" s="50"/>
-      <c r="AA185" s="50"/>
-      <c r="AB185" s="51"/>
+      <c r="H185" s="51"/>
+      <c r="I185" s="52"/>
+      <c r="J185" s="52"/>
+      <c r="K185" s="52"/>
+      <c r="L185" s="52"/>
+      <c r="M185" s="52"/>
+      <c r="N185" s="52"/>
+      <c r="O185" s="52"/>
+      <c r="P185" s="52"/>
+      <c r="Q185" s="52"/>
+      <c r="R185" s="52"/>
+      <c r="S185" s="52"/>
+      <c r="T185" s="52"/>
+      <c r="U185" s="52"/>
+      <c r="V185" s="52"/>
+      <c r="W185" s="52"/>
+      <c r="X185" s="52"/>
+      <c r="Y185" s="52"/>
+      <c r="Z185" s="52"/>
+      <c r="AA185" s="52"/>
+      <c r="AB185" s="53"/>
       <c r="AC185" s="11"/>
     </row>
     <row r="186" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7480,27 +7518,27 @@
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
       <c r="G186" s="6"/>
-      <c r="H186" s="49"/>
-      <c r="I186" s="50"/>
-      <c r="J186" s="50"/>
-      <c r="K186" s="50"/>
-      <c r="L186" s="50"/>
-      <c r="M186" s="50"/>
-      <c r="N186" s="50"/>
-      <c r="O186" s="50"/>
-      <c r="P186" s="50"/>
-      <c r="Q186" s="50"/>
-      <c r="R186" s="50"/>
-      <c r="S186" s="50"/>
-      <c r="T186" s="50"/>
-      <c r="U186" s="50"/>
-      <c r="V186" s="50"/>
-      <c r="W186" s="50"/>
-      <c r="X186" s="50"/>
-      <c r="Y186" s="50"/>
-      <c r="Z186" s="50"/>
-      <c r="AA186" s="50"/>
-      <c r="AB186" s="51"/>
+      <c r="H186" s="51"/>
+      <c r="I186" s="52"/>
+      <c r="J186" s="52"/>
+      <c r="K186" s="52"/>
+      <c r="L186" s="52"/>
+      <c r="M186" s="52"/>
+      <c r="N186" s="52"/>
+      <c r="O186" s="52"/>
+      <c r="P186" s="52"/>
+      <c r="Q186" s="52"/>
+      <c r="R186" s="52"/>
+      <c r="S186" s="52"/>
+      <c r="T186" s="52"/>
+      <c r="U186" s="52"/>
+      <c r="V186" s="52"/>
+      <c r="W186" s="52"/>
+      <c r="X186" s="52"/>
+      <c r="Y186" s="52"/>
+      <c r="Z186" s="52"/>
+      <c r="AA186" s="52"/>
+      <c r="AB186" s="53"/>
       <c r="AC186" s="11"/>
     </row>
     <row r="187" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7510,27 +7548,27 @@
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
-      <c r="H187" s="49"/>
-      <c r="I187" s="50"/>
-      <c r="J187" s="50"/>
-      <c r="K187" s="50"/>
-      <c r="L187" s="50"/>
-      <c r="M187" s="50"/>
-      <c r="N187" s="50"/>
-      <c r="O187" s="50"/>
-      <c r="P187" s="50"/>
-      <c r="Q187" s="50"/>
-      <c r="R187" s="50"/>
-      <c r="S187" s="50"/>
-      <c r="T187" s="50"/>
-      <c r="U187" s="50"/>
-      <c r="V187" s="50"/>
-      <c r="W187" s="50"/>
-      <c r="X187" s="50"/>
-      <c r="Y187" s="50"/>
-      <c r="Z187" s="50"/>
-      <c r="AA187" s="50"/>
-      <c r="AB187" s="51"/>
+      <c r="H187" s="51"/>
+      <c r="I187" s="52"/>
+      <c r="J187" s="52"/>
+      <c r="K187" s="52"/>
+      <c r="L187" s="52"/>
+      <c r="M187" s="52"/>
+      <c r="N187" s="52"/>
+      <c r="O187" s="52"/>
+      <c r="P187" s="52"/>
+      <c r="Q187" s="52"/>
+      <c r="R187" s="52"/>
+      <c r="S187" s="52"/>
+      <c r="T187" s="52"/>
+      <c r="U187" s="52"/>
+      <c r="V187" s="52"/>
+      <c r="W187" s="52"/>
+      <c r="X187" s="52"/>
+      <c r="Y187" s="52"/>
+      <c r="Z187" s="52"/>
+      <c r="AA187" s="52"/>
+      <c r="AB187" s="53"/>
       <c r="AC187" s="11"/>
     </row>
     <row r="188" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7540,27 +7578,27 @@
       <c r="E188" s="6"/>
       <c r="F188" s="6"/>
       <c r="G188" s="6"/>
-      <c r="H188" s="52"/>
-      <c r="I188" s="53"/>
-      <c r="J188" s="53"/>
-      <c r="K188" s="53"/>
-      <c r="L188" s="53"/>
-      <c r="M188" s="53"/>
-      <c r="N188" s="53"/>
-      <c r="O188" s="53"/>
-      <c r="P188" s="53"/>
-      <c r="Q188" s="53"/>
-      <c r="R188" s="53"/>
-      <c r="S188" s="53"/>
-      <c r="T188" s="53"/>
-      <c r="U188" s="53"/>
-      <c r="V188" s="53"/>
-      <c r="W188" s="53"/>
-      <c r="X188" s="53"/>
-      <c r="Y188" s="53"/>
-      <c r="Z188" s="53"/>
-      <c r="AA188" s="53"/>
-      <c r="AB188" s="54"/>
+      <c r="H188" s="54"/>
+      <c r="I188" s="55"/>
+      <c r="J188" s="55"/>
+      <c r="K188" s="55"/>
+      <c r="L188" s="55"/>
+      <c r="M188" s="55"/>
+      <c r="N188" s="55"/>
+      <c r="O188" s="55"/>
+      <c r="P188" s="55"/>
+      <c r="Q188" s="55"/>
+      <c r="R188" s="55"/>
+      <c r="S188" s="55"/>
+      <c r="T188" s="55"/>
+      <c r="U188" s="55"/>
+      <c r="V188" s="55"/>
+      <c r="W188" s="55"/>
+      <c r="X188" s="55"/>
+      <c r="Y188" s="55"/>
+      <c r="Z188" s="55"/>
+      <c r="AA188" s="55"/>
+      <c r="AB188" s="56"/>
       <c r="AC188" s="11"/>
     </row>
     <row r="189" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7602,27 +7640,27 @@
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
       <c r="G190" s="6"/>
-      <c r="H190" s="46"/>
-      <c r="I190" s="47"/>
-      <c r="J190" s="47"/>
-      <c r="K190" s="47"/>
-      <c r="L190" s="47"/>
-      <c r="M190" s="47"/>
-      <c r="N190" s="47"/>
-      <c r="O190" s="47"/>
-      <c r="P190" s="47"/>
-      <c r="Q190" s="47"/>
-      <c r="R190" s="47"/>
-      <c r="S190" s="47"/>
-      <c r="T190" s="47"/>
-      <c r="U190" s="47"/>
-      <c r="V190" s="47"/>
-      <c r="W190" s="47"/>
-      <c r="X190" s="47"/>
-      <c r="Y190" s="47"/>
-      <c r="Z190" s="47"/>
-      <c r="AA190" s="47"/>
-      <c r="AB190" s="48"/>
+      <c r="H190" s="48"/>
+      <c r="I190" s="49"/>
+      <c r="J190" s="49"/>
+      <c r="K190" s="49"/>
+      <c r="L190" s="49"/>
+      <c r="M190" s="49"/>
+      <c r="N190" s="49"/>
+      <c r="O190" s="49"/>
+      <c r="P190" s="49"/>
+      <c r="Q190" s="49"/>
+      <c r="R190" s="49"/>
+      <c r="S190" s="49"/>
+      <c r="T190" s="49"/>
+      <c r="U190" s="49"/>
+      <c r="V190" s="49"/>
+      <c r="W190" s="49"/>
+      <c r="X190" s="49"/>
+      <c r="Y190" s="49"/>
+      <c r="Z190" s="49"/>
+      <c r="AA190" s="49"/>
+      <c r="AB190" s="50"/>
       <c r="AC190" s="11"/>
     </row>
     <row r="191" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7632,27 +7670,27 @@
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
       <c r="G191" s="6"/>
-      <c r="H191" s="49"/>
-      <c r="I191" s="50"/>
-      <c r="J191" s="50"/>
-      <c r="K191" s="50"/>
-      <c r="L191" s="50"/>
-      <c r="M191" s="50"/>
-      <c r="N191" s="50"/>
-      <c r="O191" s="50"/>
-      <c r="P191" s="50"/>
-      <c r="Q191" s="50"/>
-      <c r="R191" s="50"/>
-      <c r="S191" s="50"/>
-      <c r="T191" s="50"/>
-      <c r="U191" s="50"/>
-      <c r="V191" s="50"/>
-      <c r="W191" s="50"/>
-      <c r="X191" s="50"/>
-      <c r="Y191" s="50"/>
-      <c r="Z191" s="50"/>
-      <c r="AA191" s="50"/>
-      <c r="AB191" s="51"/>
+      <c r="H191" s="51"/>
+      <c r="I191" s="52"/>
+      <c r="J191" s="52"/>
+      <c r="K191" s="52"/>
+      <c r="L191" s="52"/>
+      <c r="M191" s="52"/>
+      <c r="N191" s="52"/>
+      <c r="O191" s="52"/>
+      <c r="P191" s="52"/>
+      <c r="Q191" s="52"/>
+      <c r="R191" s="52"/>
+      <c r="S191" s="52"/>
+      <c r="T191" s="52"/>
+      <c r="U191" s="52"/>
+      <c r="V191" s="52"/>
+      <c r="W191" s="52"/>
+      <c r="X191" s="52"/>
+      <c r="Y191" s="52"/>
+      <c r="Z191" s="52"/>
+      <c r="AA191" s="52"/>
+      <c r="AB191" s="53"/>
       <c r="AC191" s="11"/>
     </row>
     <row r="192" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7662,27 +7700,27 @@
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
       <c r="G192" s="6"/>
-      <c r="H192" s="49"/>
-      <c r="I192" s="50"/>
-      <c r="J192" s="50"/>
-      <c r="K192" s="50"/>
-      <c r="L192" s="50"/>
-      <c r="M192" s="50"/>
-      <c r="N192" s="50"/>
-      <c r="O192" s="50"/>
-      <c r="P192" s="50"/>
-      <c r="Q192" s="50"/>
-      <c r="R192" s="50"/>
-      <c r="S192" s="50"/>
-      <c r="T192" s="50"/>
-      <c r="U192" s="50"/>
-      <c r="V192" s="50"/>
-      <c r="W192" s="50"/>
-      <c r="X192" s="50"/>
-      <c r="Y192" s="50"/>
-      <c r="Z192" s="50"/>
-      <c r="AA192" s="50"/>
-      <c r="AB192" s="51"/>
+      <c r="H192" s="51"/>
+      <c r="I192" s="52"/>
+      <c r="J192" s="52"/>
+      <c r="K192" s="52"/>
+      <c r="L192" s="52"/>
+      <c r="M192" s="52"/>
+      <c r="N192" s="52"/>
+      <c r="O192" s="52"/>
+      <c r="P192" s="52"/>
+      <c r="Q192" s="52"/>
+      <c r="R192" s="52"/>
+      <c r="S192" s="52"/>
+      <c r="T192" s="52"/>
+      <c r="U192" s="52"/>
+      <c r="V192" s="52"/>
+      <c r="W192" s="52"/>
+      <c r="X192" s="52"/>
+      <c r="Y192" s="52"/>
+      <c r="Z192" s="52"/>
+      <c r="AA192" s="52"/>
+      <c r="AB192" s="53"/>
       <c r="AC192" s="11"/>
     </row>
     <row r="193" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7692,27 +7730,27 @@
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
       <c r="G193" s="6"/>
-      <c r="H193" s="49"/>
-      <c r="I193" s="50"/>
-      <c r="J193" s="50"/>
-      <c r="K193" s="50"/>
-      <c r="L193" s="50"/>
-      <c r="M193" s="50"/>
-      <c r="N193" s="50"/>
-      <c r="O193" s="50"/>
-      <c r="P193" s="50"/>
-      <c r="Q193" s="50"/>
-      <c r="R193" s="50"/>
-      <c r="S193" s="50"/>
-      <c r="T193" s="50"/>
-      <c r="U193" s="50"/>
-      <c r="V193" s="50"/>
-      <c r="W193" s="50"/>
-      <c r="X193" s="50"/>
-      <c r="Y193" s="50"/>
-      <c r="Z193" s="50"/>
-      <c r="AA193" s="50"/>
-      <c r="AB193" s="51"/>
+      <c r="H193" s="51"/>
+      <c r="I193" s="52"/>
+      <c r="J193" s="52"/>
+      <c r="K193" s="52"/>
+      <c r="L193" s="52"/>
+      <c r="M193" s="52"/>
+      <c r="N193" s="52"/>
+      <c r="O193" s="52"/>
+      <c r="P193" s="52"/>
+      <c r="Q193" s="52"/>
+      <c r="R193" s="52"/>
+      <c r="S193" s="52"/>
+      <c r="T193" s="52"/>
+      <c r="U193" s="52"/>
+      <c r="V193" s="52"/>
+      <c r="W193" s="52"/>
+      <c r="X193" s="52"/>
+      <c r="Y193" s="52"/>
+      <c r="Z193" s="52"/>
+      <c r="AA193" s="52"/>
+      <c r="AB193" s="53"/>
       <c r="AC193" s="11"/>
     </row>
     <row r="194" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7722,27 +7760,27 @@
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
-      <c r="H194" s="49"/>
-      <c r="I194" s="50"/>
-      <c r="J194" s="50"/>
-      <c r="K194" s="50"/>
-      <c r="L194" s="50"/>
-      <c r="M194" s="50"/>
-      <c r="N194" s="50"/>
-      <c r="O194" s="50"/>
-      <c r="P194" s="50"/>
-      <c r="Q194" s="50"/>
-      <c r="R194" s="50"/>
-      <c r="S194" s="50"/>
-      <c r="T194" s="50"/>
-      <c r="U194" s="50"/>
-      <c r="V194" s="50"/>
-      <c r="W194" s="50"/>
-      <c r="X194" s="50"/>
-      <c r="Y194" s="50"/>
-      <c r="Z194" s="50"/>
-      <c r="AA194" s="50"/>
-      <c r="AB194" s="51"/>
+      <c r="H194" s="51"/>
+      <c r="I194" s="52"/>
+      <c r="J194" s="52"/>
+      <c r="K194" s="52"/>
+      <c r="L194" s="52"/>
+      <c r="M194" s="52"/>
+      <c r="N194" s="52"/>
+      <c r="O194" s="52"/>
+      <c r="P194" s="52"/>
+      <c r="Q194" s="52"/>
+      <c r="R194" s="52"/>
+      <c r="S194" s="52"/>
+      <c r="T194" s="52"/>
+      <c r="U194" s="52"/>
+      <c r="V194" s="52"/>
+      <c r="W194" s="52"/>
+      <c r="X194" s="52"/>
+      <c r="Y194" s="52"/>
+      <c r="Z194" s="52"/>
+      <c r="AA194" s="52"/>
+      <c r="AB194" s="53"/>
       <c r="AC194" s="11"/>
     </row>
     <row r="195" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7752,27 +7790,27 @@
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
-      <c r="H195" s="49"/>
-      <c r="I195" s="50"/>
-      <c r="J195" s="50"/>
-      <c r="K195" s="50"/>
-      <c r="L195" s="50"/>
-      <c r="M195" s="50"/>
-      <c r="N195" s="50"/>
-      <c r="O195" s="50"/>
-      <c r="P195" s="50"/>
-      <c r="Q195" s="50"/>
-      <c r="R195" s="50"/>
-      <c r="S195" s="50"/>
-      <c r="T195" s="50"/>
-      <c r="U195" s="50"/>
-      <c r="V195" s="50"/>
-      <c r="W195" s="50"/>
-      <c r="X195" s="50"/>
-      <c r="Y195" s="50"/>
-      <c r="Z195" s="50"/>
-      <c r="AA195" s="50"/>
-      <c r="AB195" s="51"/>
+      <c r="H195" s="51"/>
+      <c r="I195" s="52"/>
+      <c r="J195" s="52"/>
+      <c r="K195" s="52"/>
+      <c r="L195" s="52"/>
+      <c r="M195" s="52"/>
+      <c r="N195" s="52"/>
+      <c r="O195" s="52"/>
+      <c r="P195" s="52"/>
+      <c r="Q195" s="52"/>
+      <c r="R195" s="52"/>
+      <c r="S195" s="52"/>
+      <c r="T195" s="52"/>
+      <c r="U195" s="52"/>
+      <c r="V195" s="52"/>
+      <c r="W195" s="52"/>
+      <c r="X195" s="52"/>
+      <c r="Y195" s="52"/>
+      <c r="Z195" s="52"/>
+      <c r="AA195" s="52"/>
+      <c r="AB195" s="53"/>
       <c r="AC195" s="11"/>
     </row>
     <row r="196" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7782,27 +7820,27 @@
       <c r="E196" s="6"/>
       <c r="F196" s="6"/>
       <c r="G196" s="6"/>
-      <c r="H196" s="52"/>
-      <c r="I196" s="53"/>
-      <c r="J196" s="53"/>
-      <c r="K196" s="53"/>
-      <c r="L196" s="53"/>
-      <c r="M196" s="53"/>
-      <c r="N196" s="53"/>
-      <c r="O196" s="53"/>
-      <c r="P196" s="53"/>
-      <c r="Q196" s="53"/>
-      <c r="R196" s="53"/>
-      <c r="S196" s="53"/>
-      <c r="T196" s="53"/>
-      <c r="U196" s="53"/>
-      <c r="V196" s="53"/>
-      <c r="W196" s="53"/>
-      <c r="X196" s="53"/>
-      <c r="Y196" s="53"/>
-      <c r="Z196" s="53"/>
-      <c r="AA196" s="53"/>
-      <c r="AB196" s="54"/>
+      <c r="H196" s="54"/>
+      <c r="I196" s="55"/>
+      <c r="J196" s="55"/>
+      <c r="K196" s="55"/>
+      <c r="L196" s="55"/>
+      <c r="M196" s="55"/>
+      <c r="N196" s="55"/>
+      <c r="O196" s="55"/>
+      <c r="P196" s="55"/>
+      <c r="Q196" s="55"/>
+      <c r="R196" s="55"/>
+      <c r="S196" s="55"/>
+      <c r="T196" s="55"/>
+      <c r="U196" s="55"/>
+      <c r="V196" s="55"/>
+      <c r="W196" s="55"/>
+      <c r="X196" s="55"/>
+      <c r="Y196" s="55"/>
+      <c r="Z196" s="55"/>
+      <c r="AA196" s="55"/>
+      <c r="AB196" s="56"/>
       <c r="AC196" s="11"/>
     </row>
     <row r="197" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7910,27 +7948,27 @@
         <v>2</v>
       </c>
       <c r="G201" s="6"/>
-      <c r="H201" s="46"/>
-      <c r="I201" s="47"/>
-      <c r="J201" s="47"/>
-      <c r="K201" s="47"/>
-      <c r="L201" s="47"/>
-      <c r="M201" s="47"/>
-      <c r="N201" s="47"/>
-      <c r="O201" s="47"/>
-      <c r="P201" s="47"/>
-      <c r="Q201" s="47"/>
-      <c r="R201" s="47"/>
-      <c r="S201" s="47"/>
-      <c r="T201" s="47"/>
-      <c r="U201" s="47"/>
-      <c r="V201" s="47"/>
-      <c r="W201" s="47"/>
-      <c r="X201" s="47"/>
-      <c r="Y201" s="47"/>
-      <c r="Z201" s="47"/>
-      <c r="AA201" s="47"/>
-      <c r="AB201" s="48"/>
+      <c r="H201" s="48"/>
+      <c r="I201" s="49"/>
+      <c r="J201" s="49"/>
+      <c r="K201" s="49"/>
+      <c r="L201" s="49"/>
+      <c r="M201" s="49"/>
+      <c r="N201" s="49"/>
+      <c r="O201" s="49"/>
+      <c r="P201" s="49"/>
+      <c r="Q201" s="49"/>
+      <c r="R201" s="49"/>
+      <c r="S201" s="49"/>
+      <c r="T201" s="49"/>
+      <c r="U201" s="49"/>
+      <c r="V201" s="49"/>
+      <c r="W201" s="49"/>
+      <c r="X201" s="49"/>
+      <c r="Y201" s="49"/>
+      <c r="Z201" s="49"/>
+      <c r="AA201" s="49"/>
+      <c r="AB201" s="50"/>
       <c r="AC201" s="11"/>
     </row>
     <row r="202" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7940,27 +7978,27 @@
       <c r="E202" s="6"/>
       <c r="F202" s="6"/>
       <c r="G202" s="6"/>
-      <c r="H202" s="49"/>
-      <c r="I202" s="50"/>
-      <c r="J202" s="50"/>
-      <c r="K202" s="50"/>
-      <c r="L202" s="50"/>
-      <c r="M202" s="50"/>
-      <c r="N202" s="50"/>
-      <c r="O202" s="50"/>
-      <c r="P202" s="50"/>
-      <c r="Q202" s="50"/>
-      <c r="R202" s="50"/>
-      <c r="S202" s="50"/>
-      <c r="T202" s="50"/>
-      <c r="U202" s="50"/>
-      <c r="V202" s="50"/>
-      <c r="W202" s="50"/>
-      <c r="X202" s="50"/>
-      <c r="Y202" s="50"/>
-      <c r="Z202" s="50"/>
-      <c r="AA202" s="50"/>
-      <c r="AB202" s="51"/>
+      <c r="H202" s="51"/>
+      <c r="I202" s="52"/>
+      <c r="J202" s="52"/>
+      <c r="K202" s="52"/>
+      <c r="L202" s="52"/>
+      <c r="M202" s="52"/>
+      <c r="N202" s="52"/>
+      <c r="O202" s="52"/>
+      <c r="P202" s="52"/>
+      <c r="Q202" s="52"/>
+      <c r="R202" s="52"/>
+      <c r="S202" s="52"/>
+      <c r="T202" s="52"/>
+      <c r="U202" s="52"/>
+      <c r="V202" s="52"/>
+      <c r="W202" s="52"/>
+      <c r="X202" s="52"/>
+      <c r="Y202" s="52"/>
+      <c r="Z202" s="52"/>
+      <c r="AA202" s="52"/>
+      <c r="AB202" s="53"/>
       <c r="AC202" s="11"/>
     </row>
     <row r="203" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -7970,27 +8008,27 @@
       <c r="E203" s="6"/>
       <c r="F203" s="6"/>
       <c r="G203" s="6"/>
-      <c r="H203" s="49"/>
-      <c r="I203" s="50"/>
-      <c r="J203" s="50"/>
-      <c r="K203" s="50"/>
-      <c r="L203" s="50"/>
-      <c r="M203" s="50"/>
-      <c r="N203" s="50"/>
-      <c r="O203" s="50"/>
-      <c r="P203" s="50"/>
-      <c r="Q203" s="50"/>
-      <c r="R203" s="50"/>
-      <c r="S203" s="50"/>
-      <c r="T203" s="50"/>
-      <c r="U203" s="50"/>
-      <c r="V203" s="50"/>
-      <c r="W203" s="50"/>
-      <c r="X203" s="50"/>
-      <c r="Y203" s="50"/>
-      <c r="Z203" s="50"/>
-      <c r="AA203" s="50"/>
-      <c r="AB203" s="51"/>
+      <c r="H203" s="51"/>
+      <c r="I203" s="52"/>
+      <c r="J203" s="52"/>
+      <c r="K203" s="52"/>
+      <c r="L203" s="52"/>
+      <c r="M203" s="52"/>
+      <c r="N203" s="52"/>
+      <c r="O203" s="52"/>
+      <c r="P203" s="52"/>
+      <c r="Q203" s="52"/>
+      <c r="R203" s="52"/>
+      <c r="S203" s="52"/>
+      <c r="T203" s="52"/>
+      <c r="U203" s="52"/>
+      <c r="V203" s="52"/>
+      <c r="W203" s="52"/>
+      <c r="X203" s="52"/>
+      <c r="Y203" s="52"/>
+      <c r="Z203" s="52"/>
+      <c r="AA203" s="52"/>
+      <c r="AB203" s="53"/>
       <c r="AC203" s="11"/>
     </row>
     <row r="204" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8000,27 +8038,27 @@
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
       <c r="G204" s="6"/>
-      <c r="H204" s="49"/>
-      <c r="I204" s="50"/>
-      <c r="J204" s="50"/>
-      <c r="K204" s="50"/>
-      <c r="L204" s="50"/>
-      <c r="M204" s="50"/>
-      <c r="N204" s="50"/>
-      <c r="O204" s="50"/>
-      <c r="P204" s="50"/>
-      <c r="Q204" s="50"/>
-      <c r="R204" s="50"/>
-      <c r="S204" s="50"/>
-      <c r="T204" s="50"/>
-      <c r="U204" s="50"/>
-      <c r="V204" s="50"/>
-      <c r="W204" s="50"/>
-      <c r="X204" s="50"/>
-      <c r="Y204" s="50"/>
-      <c r="Z204" s="50"/>
-      <c r="AA204" s="50"/>
-      <c r="AB204" s="51"/>
+      <c r="H204" s="51"/>
+      <c r="I204" s="52"/>
+      <c r="J204" s="52"/>
+      <c r="K204" s="52"/>
+      <c r="L204" s="52"/>
+      <c r="M204" s="52"/>
+      <c r="N204" s="52"/>
+      <c r="O204" s="52"/>
+      <c r="P204" s="52"/>
+      <c r="Q204" s="52"/>
+      <c r="R204" s="52"/>
+      <c r="S204" s="52"/>
+      <c r="T204" s="52"/>
+      <c r="U204" s="52"/>
+      <c r="V204" s="52"/>
+      <c r="W204" s="52"/>
+      <c r="X204" s="52"/>
+      <c r="Y204" s="52"/>
+      <c r="Z204" s="52"/>
+      <c r="AA204" s="52"/>
+      <c r="AB204" s="53"/>
       <c r="AC204" s="11"/>
     </row>
     <row r="205" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8030,27 +8068,27 @@
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
       <c r="G205" s="6"/>
-      <c r="H205" s="49"/>
-      <c r="I205" s="50"/>
-      <c r="J205" s="50"/>
-      <c r="K205" s="50"/>
-      <c r="L205" s="50"/>
-      <c r="M205" s="50"/>
-      <c r="N205" s="50"/>
-      <c r="O205" s="50"/>
-      <c r="P205" s="50"/>
-      <c r="Q205" s="50"/>
-      <c r="R205" s="50"/>
-      <c r="S205" s="50"/>
-      <c r="T205" s="50"/>
-      <c r="U205" s="50"/>
-      <c r="V205" s="50"/>
-      <c r="W205" s="50"/>
-      <c r="X205" s="50"/>
-      <c r="Y205" s="50"/>
-      <c r="Z205" s="50"/>
-      <c r="AA205" s="50"/>
-      <c r="AB205" s="51"/>
+      <c r="H205" s="51"/>
+      <c r="I205" s="52"/>
+      <c r="J205" s="52"/>
+      <c r="K205" s="52"/>
+      <c r="L205" s="52"/>
+      <c r="M205" s="52"/>
+      <c r="N205" s="52"/>
+      <c r="O205" s="52"/>
+      <c r="P205" s="52"/>
+      <c r="Q205" s="52"/>
+      <c r="R205" s="52"/>
+      <c r="S205" s="52"/>
+      <c r="T205" s="52"/>
+      <c r="U205" s="52"/>
+      <c r="V205" s="52"/>
+      <c r="W205" s="52"/>
+      <c r="X205" s="52"/>
+      <c r="Y205" s="52"/>
+      <c r="Z205" s="52"/>
+      <c r="AA205" s="52"/>
+      <c r="AB205" s="53"/>
       <c r="AC205" s="11"/>
     </row>
     <row r="206" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8060,27 +8098,27 @@
       <c r="E206" s="6"/>
       <c r="F206" s="6"/>
       <c r="G206" s="6"/>
-      <c r="H206" s="49"/>
-      <c r="I206" s="50"/>
-      <c r="J206" s="50"/>
-      <c r="K206" s="50"/>
-      <c r="L206" s="50"/>
-      <c r="M206" s="50"/>
-      <c r="N206" s="50"/>
-      <c r="O206" s="50"/>
-      <c r="P206" s="50"/>
-      <c r="Q206" s="50"/>
-      <c r="R206" s="50"/>
-      <c r="S206" s="50"/>
-      <c r="T206" s="50"/>
-      <c r="U206" s="50"/>
-      <c r="V206" s="50"/>
-      <c r="W206" s="50"/>
-      <c r="X206" s="50"/>
-      <c r="Y206" s="50"/>
-      <c r="Z206" s="50"/>
-      <c r="AA206" s="50"/>
-      <c r="AB206" s="51"/>
+      <c r="H206" s="51"/>
+      <c r="I206" s="52"/>
+      <c r="J206" s="52"/>
+      <c r="K206" s="52"/>
+      <c r="L206" s="52"/>
+      <c r="M206" s="52"/>
+      <c r="N206" s="52"/>
+      <c r="O206" s="52"/>
+      <c r="P206" s="52"/>
+      <c r="Q206" s="52"/>
+      <c r="R206" s="52"/>
+      <c r="S206" s="52"/>
+      <c r="T206" s="52"/>
+      <c r="U206" s="52"/>
+      <c r="V206" s="52"/>
+      <c r="W206" s="52"/>
+      <c r="X206" s="52"/>
+      <c r="Y206" s="52"/>
+      <c r="Z206" s="52"/>
+      <c r="AA206" s="52"/>
+      <c r="AB206" s="53"/>
       <c r="AC206" s="11"/>
     </row>
     <row r="207" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8090,27 +8128,27 @@
       <c r="E207" s="6"/>
       <c r="F207" s="6"/>
       <c r="G207" s="6"/>
-      <c r="H207" s="52"/>
-      <c r="I207" s="53"/>
-      <c r="J207" s="53"/>
-      <c r="K207" s="53"/>
-      <c r="L207" s="53"/>
-      <c r="M207" s="53"/>
-      <c r="N207" s="53"/>
-      <c r="O207" s="53"/>
-      <c r="P207" s="53"/>
-      <c r="Q207" s="53"/>
-      <c r="R207" s="53"/>
-      <c r="S207" s="53"/>
-      <c r="T207" s="53"/>
-      <c r="U207" s="53"/>
-      <c r="V207" s="53"/>
-      <c r="W207" s="53"/>
-      <c r="X207" s="53"/>
-      <c r="Y207" s="53"/>
-      <c r="Z207" s="53"/>
-      <c r="AA207" s="53"/>
-      <c r="AB207" s="54"/>
+      <c r="H207" s="54"/>
+      <c r="I207" s="55"/>
+      <c r="J207" s="55"/>
+      <c r="K207" s="55"/>
+      <c r="L207" s="55"/>
+      <c r="M207" s="55"/>
+      <c r="N207" s="55"/>
+      <c r="O207" s="55"/>
+      <c r="P207" s="55"/>
+      <c r="Q207" s="55"/>
+      <c r="R207" s="55"/>
+      <c r="S207" s="55"/>
+      <c r="T207" s="55"/>
+      <c r="U207" s="55"/>
+      <c r="V207" s="55"/>
+      <c r="W207" s="55"/>
+      <c r="X207" s="55"/>
+      <c r="Y207" s="55"/>
+      <c r="Z207" s="55"/>
+      <c r="AA207" s="55"/>
+      <c r="AB207" s="56"/>
       <c r="AC207" s="11"/>
     </row>
     <row r="208" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8152,27 +8190,27 @@
       <c r="E209" s="6"/>
       <c r="F209" s="6"/>
       <c r="G209" s="6"/>
-      <c r="H209" s="46"/>
-      <c r="I209" s="47"/>
-      <c r="J209" s="47"/>
-      <c r="K209" s="47"/>
-      <c r="L209" s="47"/>
-      <c r="M209" s="47"/>
-      <c r="N209" s="47"/>
-      <c r="O209" s="47"/>
-      <c r="P209" s="47"/>
-      <c r="Q209" s="47"/>
-      <c r="R209" s="47"/>
-      <c r="S209" s="47"/>
-      <c r="T209" s="47"/>
-      <c r="U209" s="47"/>
-      <c r="V209" s="47"/>
-      <c r="W209" s="47"/>
-      <c r="X209" s="47"/>
-      <c r="Y209" s="47"/>
-      <c r="Z209" s="47"/>
-      <c r="AA209" s="47"/>
-      <c r="AB209" s="48"/>
+      <c r="H209" s="48"/>
+      <c r="I209" s="49"/>
+      <c r="J209" s="49"/>
+      <c r="K209" s="49"/>
+      <c r="L209" s="49"/>
+      <c r="M209" s="49"/>
+      <c r="N209" s="49"/>
+      <c r="O209" s="49"/>
+      <c r="P209" s="49"/>
+      <c r="Q209" s="49"/>
+      <c r="R209" s="49"/>
+      <c r="S209" s="49"/>
+      <c r="T209" s="49"/>
+      <c r="U209" s="49"/>
+      <c r="V209" s="49"/>
+      <c r="W209" s="49"/>
+      <c r="X209" s="49"/>
+      <c r="Y209" s="49"/>
+      <c r="Z209" s="49"/>
+      <c r="AA209" s="49"/>
+      <c r="AB209" s="50"/>
       <c r="AC209" s="11"/>
     </row>
     <row r="210" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8182,27 +8220,27 @@
       <c r="E210" s="6"/>
       <c r="F210" s="6"/>
       <c r="G210" s="6"/>
-      <c r="H210" s="49"/>
-      <c r="I210" s="50"/>
-      <c r="J210" s="50"/>
-      <c r="K210" s="50"/>
-      <c r="L210" s="50"/>
-      <c r="M210" s="50"/>
-      <c r="N210" s="50"/>
-      <c r="O210" s="50"/>
-      <c r="P210" s="50"/>
-      <c r="Q210" s="50"/>
-      <c r="R210" s="50"/>
-      <c r="S210" s="50"/>
-      <c r="T210" s="50"/>
-      <c r="U210" s="50"/>
-      <c r="V210" s="50"/>
-      <c r="W210" s="50"/>
-      <c r="X210" s="50"/>
-      <c r="Y210" s="50"/>
-      <c r="Z210" s="50"/>
-      <c r="AA210" s="50"/>
-      <c r="AB210" s="51"/>
+      <c r="H210" s="51"/>
+      <c r="I210" s="52"/>
+      <c r="J210" s="52"/>
+      <c r="K210" s="52"/>
+      <c r="L210" s="52"/>
+      <c r="M210" s="52"/>
+      <c r="N210" s="52"/>
+      <c r="O210" s="52"/>
+      <c r="P210" s="52"/>
+      <c r="Q210" s="52"/>
+      <c r="R210" s="52"/>
+      <c r="S210" s="52"/>
+      <c r="T210" s="52"/>
+      <c r="U210" s="52"/>
+      <c r="V210" s="52"/>
+      <c r="W210" s="52"/>
+      <c r="X210" s="52"/>
+      <c r="Y210" s="52"/>
+      <c r="Z210" s="52"/>
+      <c r="AA210" s="52"/>
+      <c r="AB210" s="53"/>
       <c r="AC210" s="11"/>
     </row>
     <row r="211" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8212,27 +8250,27 @@
       <c r="E211" s="6"/>
       <c r="F211" s="6"/>
       <c r="G211" s="6"/>
-      <c r="H211" s="49"/>
-      <c r="I211" s="50"/>
-      <c r="J211" s="50"/>
-      <c r="K211" s="50"/>
-      <c r="L211" s="50"/>
-      <c r="M211" s="50"/>
-      <c r="N211" s="50"/>
-      <c r="O211" s="50"/>
-      <c r="P211" s="50"/>
-      <c r="Q211" s="50"/>
-      <c r="R211" s="50"/>
-      <c r="S211" s="50"/>
-      <c r="T211" s="50"/>
-      <c r="U211" s="50"/>
-      <c r="V211" s="50"/>
-      <c r="W211" s="50"/>
-      <c r="X211" s="50"/>
-      <c r="Y211" s="50"/>
-      <c r="Z211" s="50"/>
-      <c r="AA211" s="50"/>
-      <c r="AB211" s="51"/>
+      <c r="H211" s="51"/>
+      <c r="I211" s="52"/>
+      <c r="J211" s="52"/>
+      <c r="K211" s="52"/>
+      <c r="L211" s="52"/>
+      <c r="M211" s="52"/>
+      <c r="N211" s="52"/>
+      <c r="O211" s="52"/>
+      <c r="P211" s="52"/>
+      <c r="Q211" s="52"/>
+      <c r="R211" s="52"/>
+      <c r="S211" s="52"/>
+      <c r="T211" s="52"/>
+      <c r="U211" s="52"/>
+      <c r="V211" s="52"/>
+      <c r="W211" s="52"/>
+      <c r="X211" s="52"/>
+      <c r="Y211" s="52"/>
+      <c r="Z211" s="52"/>
+      <c r="AA211" s="52"/>
+      <c r="AB211" s="53"/>
       <c r="AC211" s="11"/>
     </row>
     <row r="212" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8242,27 +8280,27 @@
       <c r="E212" s="6"/>
       <c r="F212" s="6"/>
       <c r="G212" s="6"/>
-      <c r="H212" s="49"/>
-      <c r="I212" s="50"/>
-      <c r="J212" s="50"/>
-      <c r="K212" s="50"/>
-      <c r="L212" s="50"/>
-      <c r="M212" s="50"/>
-      <c r="N212" s="50"/>
-      <c r="O212" s="50"/>
-      <c r="P212" s="50"/>
-      <c r="Q212" s="50"/>
-      <c r="R212" s="50"/>
-      <c r="S212" s="50"/>
-      <c r="T212" s="50"/>
-      <c r="U212" s="50"/>
-      <c r="V212" s="50"/>
-      <c r="W212" s="50"/>
-      <c r="X212" s="50"/>
-      <c r="Y212" s="50"/>
-      <c r="Z212" s="50"/>
-      <c r="AA212" s="50"/>
-      <c r="AB212" s="51"/>
+      <c r="H212" s="51"/>
+      <c r="I212" s="52"/>
+      <c r="J212" s="52"/>
+      <c r="K212" s="52"/>
+      <c r="L212" s="52"/>
+      <c r="M212" s="52"/>
+      <c r="N212" s="52"/>
+      <c r="O212" s="52"/>
+      <c r="P212" s="52"/>
+      <c r="Q212" s="52"/>
+      <c r="R212" s="52"/>
+      <c r="S212" s="52"/>
+      <c r="T212" s="52"/>
+      <c r="U212" s="52"/>
+      <c r="V212" s="52"/>
+      <c r="W212" s="52"/>
+      <c r="X212" s="52"/>
+      <c r="Y212" s="52"/>
+      <c r="Z212" s="52"/>
+      <c r="AA212" s="52"/>
+      <c r="AB212" s="53"/>
       <c r="AC212" s="11"/>
     </row>
     <row r="213" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8272,27 +8310,27 @@
       <c r="E213" s="6"/>
       <c r="F213" s="6"/>
       <c r="G213" s="6"/>
-      <c r="H213" s="49"/>
-      <c r="I213" s="50"/>
-      <c r="J213" s="50"/>
-      <c r="K213" s="50"/>
-      <c r="L213" s="50"/>
-      <c r="M213" s="50"/>
-      <c r="N213" s="50"/>
-      <c r="O213" s="50"/>
-      <c r="P213" s="50"/>
-      <c r="Q213" s="50"/>
-      <c r="R213" s="50"/>
-      <c r="S213" s="50"/>
-      <c r="T213" s="50"/>
-      <c r="U213" s="50"/>
-      <c r="V213" s="50"/>
-      <c r="W213" s="50"/>
-      <c r="X213" s="50"/>
-      <c r="Y213" s="50"/>
-      <c r="Z213" s="50"/>
-      <c r="AA213" s="50"/>
-      <c r="AB213" s="51"/>
+      <c r="H213" s="51"/>
+      <c r="I213" s="52"/>
+      <c r="J213" s="52"/>
+      <c r="K213" s="52"/>
+      <c r="L213" s="52"/>
+      <c r="M213" s="52"/>
+      <c r="N213" s="52"/>
+      <c r="O213" s="52"/>
+      <c r="P213" s="52"/>
+      <c r="Q213" s="52"/>
+      <c r="R213" s="52"/>
+      <c r="S213" s="52"/>
+      <c r="T213" s="52"/>
+      <c r="U213" s="52"/>
+      <c r="V213" s="52"/>
+      <c r="W213" s="52"/>
+      <c r="X213" s="52"/>
+      <c r="Y213" s="52"/>
+      <c r="Z213" s="52"/>
+      <c r="AA213" s="52"/>
+      <c r="AB213" s="53"/>
       <c r="AC213" s="11"/>
     </row>
     <row r="214" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8302,27 +8340,27 @@
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
-      <c r="H214" s="49"/>
-      <c r="I214" s="50"/>
-      <c r="J214" s="50"/>
-      <c r="K214" s="50"/>
-      <c r="L214" s="50"/>
-      <c r="M214" s="50"/>
-      <c r="N214" s="50"/>
-      <c r="O214" s="50"/>
-      <c r="P214" s="50"/>
-      <c r="Q214" s="50"/>
-      <c r="R214" s="50"/>
-      <c r="S214" s="50"/>
-      <c r="T214" s="50"/>
-      <c r="U214" s="50"/>
-      <c r="V214" s="50"/>
-      <c r="W214" s="50"/>
-      <c r="X214" s="50"/>
-      <c r="Y214" s="50"/>
-      <c r="Z214" s="50"/>
-      <c r="AA214" s="50"/>
-      <c r="AB214" s="51"/>
+      <c r="H214" s="51"/>
+      <c r="I214" s="52"/>
+      <c r="J214" s="52"/>
+      <c r="K214" s="52"/>
+      <c r="L214" s="52"/>
+      <c r="M214" s="52"/>
+      <c r="N214" s="52"/>
+      <c r="O214" s="52"/>
+      <c r="P214" s="52"/>
+      <c r="Q214" s="52"/>
+      <c r="R214" s="52"/>
+      <c r="S214" s="52"/>
+      <c r="T214" s="52"/>
+      <c r="U214" s="52"/>
+      <c r="V214" s="52"/>
+      <c r="W214" s="52"/>
+      <c r="X214" s="52"/>
+      <c r="Y214" s="52"/>
+      <c r="Z214" s="52"/>
+      <c r="AA214" s="52"/>
+      <c r="AB214" s="53"/>
       <c r="AC214" s="11"/>
     </row>
     <row r="215" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8332,27 +8370,27 @@
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
       <c r="G215" s="6"/>
-      <c r="H215" s="52"/>
-      <c r="I215" s="53"/>
-      <c r="J215" s="53"/>
-      <c r="K215" s="53"/>
-      <c r="L215" s="53"/>
-      <c r="M215" s="53"/>
-      <c r="N215" s="53"/>
-      <c r="O215" s="53"/>
-      <c r="P215" s="53"/>
-      <c r="Q215" s="53"/>
-      <c r="R215" s="53"/>
-      <c r="S215" s="53"/>
-      <c r="T215" s="53"/>
-      <c r="U215" s="53"/>
-      <c r="V215" s="53"/>
-      <c r="W215" s="53"/>
-      <c r="X215" s="53"/>
-      <c r="Y215" s="53"/>
-      <c r="Z215" s="53"/>
-      <c r="AA215" s="53"/>
-      <c r="AB215" s="54"/>
+      <c r="H215" s="54"/>
+      <c r="I215" s="55"/>
+      <c r="J215" s="55"/>
+      <c r="K215" s="55"/>
+      <c r="L215" s="55"/>
+      <c r="M215" s="55"/>
+      <c r="N215" s="55"/>
+      <c r="O215" s="55"/>
+      <c r="P215" s="55"/>
+      <c r="Q215" s="55"/>
+      <c r="R215" s="55"/>
+      <c r="S215" s="55"/>
+      <c r="T215" s="55"/>
+      <c r="U215" s="55"/>
+      <c r="V215" s="55"/>
+      <c r="W215" s="55"/>
+      <c r="X215" s="55"/>
+      <c r="Y215" s="55"/>
+      <c r="Z215" s="55"/>
+      <c r="AA215" s="55"/>
+      <c r="AB215" s="56"/>
       <c r="AC215" s="11"/>
     </row>
     <row r="216" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -8387,11 +8425,38 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B6:B23"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="H8:AB14"/>
-    <mergeCell ref="H16:AB22"/>
+    <mergeCell ref="B180:B197"/>
+    <mergeCell ref="D182:E182"/>
+    <mergeCell ref="H182:AB188"/>
+    <mergeCell ref="H190:AB196"/>
+    <mergeCell ref="B199:B216"/>
+    <mergeCell ref="D201:E201"/>
+    <mergeCell ref="H201:AB207"/>
+    <mergeCell ref="H209:AB215"/>
+    <mergeCell ref="B142:B159"/>
+    <mergeCell ref="D144:E144"/>
+    <mergeCell ref="H144:AB150"/>
+    <mergeCell ref="H152:AB158"/>
+    <mergeCell ref="B161:B178"/>
+    <mergeCell ref="D163:E163"/>
+    <mergeCell ref="H163:AB169"/>
+    <mergeCell ref="H171:AB177"/>
+    <mergeCell ref="B104:B121"/>
+    <mergeCell ref="D106:E106"/>
+    <mergeCell ref="H106:AB112"/>
+    <mergeCell ref="H114:AB120"/>
+    <mergeCell ref="B123:B140"/>
+    <mergeCell ref="D125:E125"/>
+    <mergeCell ref="H125:AB131"/>
+    <mergeCell ref="H133:AB139"/>
+    <mergeCell ref="B63:B83"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="H76:AB82"/>
+    <mergeCell ref="B85:B102"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="H87:AB93"/>
+    <mergeCell ref="H95:AB101"/>
+    <mergeCell ref="H65:AB74"/>
     <mergeCell ref="B25:B42"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="H27:AB33"/>
@@ -8400,44 +8465,19 @@
     <mergeCell ref="D46:E46"/>
     <mergeCell ref="H46:AB52"/>
     <mergeCell ref="H54:AB60"/>
-    <mergeCell ref="B63:B83"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="H76:AB82"/>
-    <mergeCell ref="B85:B102"/>
-    <mergeCell ref="D87:E87"/>
-    <mergeCell ref="H87:AB93"/>
-    <mergeCell ref="H95:AB101"/>
-    <mergeCell ref="H65:AB74"/>
-    <mergeCell ref="B104:B121"/>
-    <mergeCell ref="D106:E106"/>
-    <mergeCell ref="H106:AB112"/>
-    <mergeCell ref="H114:AB120"/>
-    <mergeCell ref="B123:B140"/>
-    <mergeCell ref="D125:E125"/>
-    <mergeCell ref="H125:AB131"/>
-    <mergeCell ref="H133:AB139"/>
-    <mergeCell ref="B142:B159"/>
-    <mergeCell ref="D144:E144"/>
-    <mergeCell ref="H144:AB150"/>
-    <mergeCell ref="H152:AB158"/>
-    <mergeCell ref="B161:B178"/>
-    <mergeCell ref="D163:E163"/>
-    <mergeCell ref="H163:AB169"/>
-    <mergeCell ref="H171:AB177"/>
-    <mergeCell ref="B180:B197"/>
-    <mergeCell ref="D182:E182"/>
-    <mergeCell ref="H182:AB188"/>
-    <mergeCell ref="H190:AB196"/>
-    <mergeCell ref="B199:B216"/>
-    <mergeCell ref="D201:E201"/>
-    <mergeCell ref="H201:AB207"/>
-    <mergeCell ref="H209:AB215"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B6:B23"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="H8:AB14"/>
+    <mergeCell ref="H16:AB22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H65" r:id="rId1" display="https://learn.microsoft.com/en-us/dotnet/maui/platform-integration/device/geolocation" xr:uid="{6A2F2CBC-218B-43EA-806A-9BF39365BDB2}"/>
     <hyperlink ref="H87" r:id="rId2" display="https://dummyjson.com/docs/posts_x000a_" xr:uid="{AFA4F006-3754-4C92-A758-50B6915FC379}"/>
     <hyperlink ref="H106" r:id="rId3" display="https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/refreshview_x000a_" xr:uid="{80E066CC-CE62-4304-89CB-2C900A3EBBE5}"/>
     <hyperlink ref="H125" r:id="rId4" display="https://learn.microsoft.com/de-de/dotnet/communitytoolkit/maui/views/mediaelement" xr:uid="{A9CAE96C-CEA9-42B5-BE11-A814029EF10A}"/>
+    <hyperlink ref="H144" r:id="rId5" display="https://learn.microsoft.com/en-us/dotnet/maui/user-interface/controls/image_x000a_" xr:uid="{78B087E0-3533-42B3-9793-DB52FF358744}"/>
+    <hyperlink ref="H163" r:id="rId6" display="https://learn.microsoft.com/en-us/answers/questions/1024872/how-to-save-image-in-while-image-is-taken-from-cam_x000a_" xr:uid="{81FCBD1E-C0B4-4911-AA37-73831C593508}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -8464,11 +8504,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>21</v>
       </c>
@@ -9310,27 +9350,27 @@
       <c r="E34" s="27"/>
       <c r="F34" s="28"/>
       <c r="G34" s="19"/>
-      <c r="H34" s="46"/>
-      <c r="I34" s="47"/>
-      <c r="J34" s="47"/>
-      <c r="K34" s="47"/>
-      <c r="L34" s="47"/>
-      <c r="M34" s="47"/>
-      <c r="N34" s="47"/>
-      <c r="O34" s="47"/>
-      <c r="P34" s="47"/>
-      <c r="Q34" s="47"/>
-      <c r="R34" s="47"/>
-      <c r="S34" s="47"/>
-      <c r="T34" s="47"/>
-      <c r="U34" s="47"/>
-      <c r="V34" s="47"/>
-      <c r="W34" s="47"/>
-      <c r="X34" s="47"/>
-      <c r="Y34" s="47"/>
-      <c r="Z34" s="47"/>
-      <c r="AA34" s="47"/>
-      <c r="AB34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="49"/>
+      <c r="J34" s="49"/>
+      <c r="K34" s="49"/>
+      <c r="L34" s="49"/>
+      <c r="M34" s="49"/>
+      <c r="N34" s="49"/>
+      <c r="O34" s="49"/>
+      <c r="P34" s="49"/>
+      <c r="Q34" s="49"/>
+      <c r="R34" s="49"/>
+      <c r="S34" s="49"/>
+      <c r="T34" s="49"/>
+      <c r="U34" s="49"/>
+      <c r="V34" s="49"/>
+      <c r="W34" s="49"/>
+      <c r="X34" s="49"/>
+      <c r="Y34" s="49"/>
+      <c r="Z34" s="49"/>
+      <c r="AA34" s="49"/>
+      <c r="AB34" s="50"/>
       <c r="AC34" s="16"/>
     </row>
     <row r="35" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9340,27 +9380,27 @@
       <c r="E35" s="19"/>
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="50"/>
-      <c r="K35" s="50"/>
-      <c r="L35" s="50"/>
-      <c r="M35" s="50"/>
-      <c r="N35" s="50"/>
-      <c r="O35" s="50"/>
-      <c r="P35" s="50"/>
-      <c r="Q35" s="50"/>
-      <c r="R35" s="50"/>
-      <c r="S35" s="50"/>
-      <c r="T35" s="50"/>
-      <c r="U35" s="50"/>
-      <c r="V35" s="50"/>
-      <c r="W35" s="50"/>
-      <c r="X35" s="50"/>
-      <c r="Y35" s="50"/>
-      <c r="Z35" s="50"/>
-      <c r="AA35" s="50"/>
-      <c r="AB35" s="51"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="52"/>
+      <c r="J35" s="52"/>
+      <c r="K35" s="52"/>
+      <c r="L35" s="52"/>
+      <c r="M35" s="52"/>
+      <c r="N35" s="52"/>
+      <c r="O35" s="52"/>
+      <c r="P35" s="52"/>
+      <c r="Q35" s="52"/>
+      <c r="R35" s="52"/>
+      <c r="S35" s="52"/>
+      <c r="T35" s="52"/>
+      <c r="U35" s="52"/>
+      <c r="V35" s="52"/>
+      <c r="W35" s="52"/>
+      <c r="X35" s="52"/>
+      <c r="Y35" s="52"/>
+      <c r="Z35" s="52"/>
+      <c r="AA35" s="52"/>
+      <c r="AB35" s="53"/>
       <c r="AC35" s="16"/>
     </row>
     <row r="36" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9370,27 +9410,27 @@
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="50"/>
-      <c r="K36" s="50"/>
-      <c r="L36" s="50"/>
-      <c r="M36" s="50"/>
-      <c r="N36" s="50"/>
-      <c r="O36" s="50"/>
-      <c r="P36" s="50"/>
-      <c r="Q36" s="50"/>
-      <c r="R36" s="50"/>
-      <c r="S36" s="50"/>
-      <c r="T36" s="50"/>
-      <c r="U36" s="50"/>
-      <c r="V36" s="50"/>
-      <c r="W36" s="50"/>
-      <c r="X36" s="50"/>
-      <c r="Y36" s="50"/>
-      <c r="Z36" s="50"/>
-      <c r="AA36" s="50"/>
-      <c r="AB36" s="51"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="52"/>
+      <c r="J36" s="52"/>
+      <c r="K36" s="52"/>
+      <c r="L36" s="52"/>
+      <c r="M36" s="52"/>
+      <c r="N36" s="52"/>
+      <c r="O36" s="52"/>
+      <c r="P36" s="52"/>
+      <c r="Q36" s="52"/>
+      <c r="R36" s="52"/>
+      <c r="S36" s="52"/>
+      <c r="T36" s="52"/>
+      <c r="U36" s="52"/>
+      <c r="V36" s="52"/>
+      <c r="W36" s="52"/>
+      <c r="X36" s="52"/>
+      <c r="Y36" s="52"/>
+      <c r="Z36" s="52"/>
+      <c r="AA36" s="52"/>
+      <c r="AB36" s="53"/>
       <c r="AC36" s="16"/>
     </row>
     <row r="37" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9400,27 +9440,27 @@
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
-      <c r="H37" s="49"/>
-      <c r="I37" s="50"/>
-      <c r="J37" s="50"/>
-      <c r="K37" s="50"/>
-      <c r="L37" s="50"/>
-      <c r="M37" s="50"/>
-      <c r="N37" s="50"/>
-      <c r="O37" s="50"/>
-      <c r="P37" s="50"/>
-      <c r="Q37" s="50"/>
-      <c r="R37" s="50"/>
-      <c r="S37" s="50"/>
-      <c r="T37" s="50"/>
-      <c r="U37" s="50"/>
-      <c r="V37" s="50"/>
-      <c r="W37" s="50"/>
-      <c r="X37" s="50"/>
-      <c r="Y37" s="50"/>
-      <c r="Z37" s="50"/>
-      <c r="AA37" s="50"/>
-      <c r="AB37" s="51"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="52"/>
+      <c r="J37" s="52"/>
+      <c r="K37" s="52"/>
+      <c r="L37" s="52"/>
+      <c r="M37" s="52"/>
+      <c r="N37" s="52"/>
+      <c r="O37" s="52"/>
+      <c r="P37" s="52"/>
+      <c r="Q37" s="52"/>
+      <c r="R37" s="52"/>
+      <c r="S37" s="52"/>
+      <c r="T37" s="52"/>
+      <c r="U37" s="52"/>
+      <c r="V37" s="52"/>
+      <c r="W37" s="52"/>
+      <c r="X37" s="52"/>
+      <c r="Y37" s="52"/>
+      <c r="Z37" s="52"/>
+      <c r="AA37" s="52"/>
+      <c r="AB37" s="53"/>
       <c r="AC37" s="16"/>
     </row>
     <row r="38" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9430,27 +9470,27 @@
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
-      <c r="H38" s="49"/>
-      <c r="I38" s="50"/>
-      <c r="J38" s="50"/>
-      <c r="K38" s="50"/>
-      <c r="L38" s="50"/>
-      <c r="M38" s="50"/>
-      <c r="N38" s="50"/>
-      <c r="O38" s="50"/>
-      <c r="P38" s="50"/>
-      <c r="Q38" s="50"/>
-      <c r="R38" s="50"/>
-      <c r="S38" s="50"/>
-      <c r="T38" s="50"/>
-      <c r="U38" s="50"/>
-      <c r="V38" s="50"/>
-      <c r="W38" s="50"/>
-      <c r="X38" s="50"/>
-      <c r="Y38" s="50"/>
-      <c r="Z38" s="50"/>
-      <c r="AA38" s="50"/>
-      <c r="AB38" s="51"/>
+      <c r="H38" s="51"/>
+      <c r="I38" s="52"/>
+      <c r="J38" s="52"/>
+      <c r="K38" s="52"/>
+      <c r="L38" s="52"/>
+      <c r="M38" s="52"/>
+      <c r="N38" s="52"/>
+      <c r="O38" s="52"/>
+      <c r="P38" s="52"/>
+      <c r="Q38" s="52"/>
+      <c r="R38" s="52"/>
+      <c r="S38" s="52"/>
+      <c r="T38" s="52"/>
+      <c r="U38" s="52"/>
+      <c r="V38" s="52"/>
+      <c r="W38" s="52"/>
+      <c r="X38" s="52"/>
+      <c r="Y38" s="52"/>
+      <c r="Z38" s="52"/>
+      <c r="AA38" s="52"/>
+      <c r="AB38" s="53"/>
       <c r="AC38" s="16"/>
     </row>
     <row r="39" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9460,27 +9500,27 @@
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="19"/>
-      <c r="H39" s="49"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="50"/>
-      <c r="L39" s="50"/>
-      <c r="M39" s="50"/>
-      <c r="N39" s="50"/>
-      <c r="O39" s="50"/>
-      <c r="P39" s="50"/>
-      <c r="Q39" s="50"/>
-      <c r="R39" s="50"/>
-      <c r="S39" s="50"/>
-      <c r="T39" s="50"/>
-      <c r="U39" s="50"/>
-      <c r="V39" s="50"/>
-      <c r="W39" s="50"/>
-      <c r="X39" s="50"/>
-      <c r="Y39" s="50"/>
-      <c r="Z39" s="50"/>
-      <c r="AA39" s="50"/>
-      <c r="AB39" s="51"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="52"/>
+      <c r="J39" s="52"/>
+      <c r="K39" s="52"/>
+      <c r="L39" s="52"/>
+      <c r="M39" s="52"/>
+      <c r="N39" s="52"/>
+      <c r="O39" s="52"/>
+      <c r="P39" s="52"/>
+      <c r="Q39" s="52"/>
+      <c r="R39" s="52"/>
+      <c r="S39" s="52"/>
+      <c r="T39" s="52"/>
+      <c r="U39" s="52"/>
+      <c r="V39" s="52"/>
+      <c r="W39" s="52"/>
+      <c r="X39" s="52"/>
+      <c r="Y39" s="52"/>
+      <c r="Z39" s="52"/>
+      <c r="AA39" s="52"/>
+      <c r="AB39" s="53"/>
       <c r="AC39" s="16"/>
     </row>
     <row r="40" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9490,27 +9530,27 @@
       <c r="E40" s="19"/>
       <c r="F40" s="19"/>
       <c r="G40" s="19"/>
-      <c r="H40" s="52"/>
-      <c r="I40" s="53"/>
-      <c r="J40" s="53"/>
-      <c r="K40" s="53"/>
-      <c r="L40" s="53"/>
-      <c r="M40" s="53"/>
-      <c r="N40" s="53"/>
-      <c r="O40" s="53"/>
-      <c r="P40" s="53"/>
-      <c r="Q40" s="53"/>
-      <c r="R40" s="53"/>
-      <c r="S40" s="53"/>
-      <c r="T40" s="53"/>
-      <c r="U40" s="53"/>
-      <c r="V40" s="53"/>
-      <c r="W40" s="53"/>
-      <c r="X40" s="53"/>
-      <c r="Y40" s="53"/>
-      <c r="Z40" s="53"/>
-      <c r="AA40" s="53"/>
-      <c r="AB40" s="54"/>
+      <c r="H40" s="54"/>
+      <c r="I40" s="55"/>
+      <c r="J40" s="55"/>
+      <c r="K40" s="55"/>
+      <c r="L40" s="55"/>
+      <c r="M40" s="55"/>
+      <c r="N40" s="55"/>
+      <c r="O40" s="55"/>
+      <c r="P40" s="55"/>
+      <c r="Q40" s="55"/>
+      <c r="R40" s="55"/>
+      <c r="S40" s="55"/>
+      <c r="T40" s="55"/>
+      <c r="U40" s="55"/>
+      <c r="V40" s="55"/>
+      <c r="W40" s="55"/>
+      <c r="X40" s="55"/>
+      <c r="Y40" s="55"/>
+      <c r="Z40" s="55"/>
+      <c r="AA40" s="55"/>
+      <c r="AB40" s="56"/>
       <c r="AC40" s="16"/>
     </row>
     <row r="41" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9552,27 +9592,27 @@
       <c r="E42" s="19"/>
       <c r="F42" s="19"/>
       <c r="G42" s="19"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="47"/>
-      <c r="J42" s="47"/>
-      <c r="K42" s="47"/>
-      <c r="L42" s="47"/>
-      <c r="M42" s="47"/>
-      <c r="N42" s="47"/>
-      <c r="O42" s="47"/>
-      <c r="P42" s="47"/>
-      <c r="Q42" s="47"/>
-      <c r="R42" s="47"/>
-      <c r="S42" s="47"/>
-      <c r="T42" s="47"/>
-      <c r="U42" s="47"/>
-      <c r="V42" s="47"/>
-      <c r="W42" s="47"/>
-      <c r="X42" s="47"/>
-      <c r="Y42" s="47"/>
-      <c r="Z42" s="47"/>
-      <c r="AA42" s="47"/>
-      <c r="AB42" s="48"/>
+      <c r="H42" s="48"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
+      <c r="M42" s="49"/>
+      <c r="N42" s="49"/>
+      <c r="O42" s="49"/>
+      <c r="P42" s="49"/>
+      <c r="Q42" s="49"/>
+      <c r="R42" s="49"/>
+      <c r="S42" s="49"/>
+      <c r="T42" s="49"/>
+      <c r="U42" s="49"/>
+      <c r="V42" s="49"/>
+      <c r="W42" s="49"/>
+      <c r="X42" s="49"/>
+      <c r="Y42" s="49"/>
+      <c r="Z42" s="49"/>
+      <c r="AA42" s="49"/>
+      <c r="AB42" s="50"/>
       <c r="AC42" s="16"/>
     </row>
     <row r="43" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9582,27 +9622,27 @@
       <c r="E43" s="19"/>
       <c r="F43" s="19"/>
       <c r="G43" s="19"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="50"/>
-      <c r="J43" s="50"/>
-      <c r="K43" s="50"/>
-      <c r="L43" s="50"/>
-      <c r="M43" s="50"/>
-      <c r="N43" s="50"/>
-      <c r="O43" s="50"/>
-      <c r="P43" s="50"/>
-      <c r="Q43" s="50"/>
-      <c r="R43" s="50"/>
-      <c r="S43" s="50"/>
-      <c r="T43" s="50"/>
-      <c r="U43" s="50"/>
-      <c r="V43" s="50"/>
-      <c r="W43" s="50"/>
-      <c r="X43" s="50"/>
-      <c r="Y43" s="50"/>
-      <c r="Z43" s="50"/>
-      <c r="AA43" s="50"/>
-      <c r="AB43" s="51"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="52"/>
+      <c r="J43" s="52"/>
+      <c r="K43" s="52"/>
+      <c r="L43" s="52"/>
+      <c r="M43" s="52"/>
+      <c r="N43" s="52"/>
+      <c r="O43" s="52"/>
+      <c r="P43" s="52"/>
+      <c r="Q43" s="52"/>
+      <c r="R43" s="52"/>
+      <c r="S43" s="52"/>
+      <c r="T43" s="52"/>
+      <c r="U43" s="52"/>
+      <c r="V43" s="52"/>
+      <c r="W43" s="52"/>
+      <c r="X43" s="52"/>
+      <c r="Y43" s="52"/>
+      <c r="Z43" s="52"/>
+      <c r="AA43" s="52"/>
+      <c r="AB43" s="53"/>
       <c r="AC43" s="16"/>
     </row>
     <row r="44" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9612,27 +9652,27 @@
       <c r="E44" s="19"/>
       <c r="F44" s="19"/>
       <c r="G44" s="19"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="50"/>
-      <c r="J44" s="50"/>
-      <c r="K44" s="50"/>
-      <c r="L44" s="50"/>
-      <c r="M44" s="50"/>
-      <c r="N44" s="50"/>
-      <c r="O44" s="50"/>
-      <c r="P44" s="50"/>
-      <c r="Q44" s="50"/>
-      <c r="R44" s="50"/>
-      <c r="S44" s="50"/>
-      <c r="T44" s="50"/>
-      <c r="U44" s="50"/>
-      <c r="V44" s="50"/>
-      <c r="W44" s="50"/>
-      <c r="X44" s="50"/>
-      <c r="Y44" s="50"/>
-      <c r="Z44" s="50"/>
-      <c r="AA44" s="50"/>
-      <c r="AB44" s="51"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="52"/>
+      <c r="J44" s="52"/>
+      <c r="K44" s="52"/>
+      <c r="L44" s="52"/>
+      <c r="M44" s="52"/>
+      <c r="N44" s="52"/>
+      <c r="O44" s="52"/>
+      <c r="P44" s="52"/>
+      <c r="Q44" s="52"/>
+      <c r="R44" s="52"/>
+      <c r="S44" s="52"/>
+      <c r="T44" s="52"/>
+      <c r="U44" s="52"/>
+      <c r="V44" s="52"/>
+      <c r="W44" s="52"/>
+      <c r="X44" s="52"/>
+      <c r="Y44" s="52"/>
+      <c r="Z44" s="52"/>
+      <c r="AA44" s="52"/>
+      <c r="AB44" s="53"/>
       <c r="AC44" s="16"/>
     </row>
     <row r="45" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9642,27 +9682,27 @@
       <c r="E45" s="19"/>
       <c r="F45" s="19"/>
       <c r="G45" s="19"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="50"/>
-      <c r="J45" s="50"/>
-      <c r="K45" s="50"/>
-      <c r="L45" s="50"/>
-      <c r="M45" s="50"/>
-      <c r="N45" s="50"/>
-      <c r="O45" s="50"/>
-      <c r="P45" s="50"/>
-      <c r="Q45" s="50"/>
-      <c r="R45" s="50"/>
-      <c r="S45" s="50"/>
-      <c r="T45" s="50"/>
-      <c r="U45" s="50"/>
-      <c r="V45" s="50"/>
-      <c r="W45" s="50"/>
-      <c r="X45" s="50"/>
-      <c r="Y45" s="50"/>
-      <c r="Z45" s="50"/>
-      <c r="AA45" s="50"/>
-      <c r="AB45" s="51"/>
+      <c r="H45" s="51"/>
+      <c r="I45" s="52"/>
+      <c r="J45" s="52"/>
+      <c r="K45" s="52"/>
+      <c r="L45" s="52"/>
+      <c r="M45" s="52"/>
+      <c r="N45" s="52"/>
+      <c r="O45" s="52"/>
+      <c r="P45" s="52"/>
+      <c r="Q45" s="52"/>
+      <c r="R45" s="52"/>
+      <c r="S45" s="52"/>
+      <c r="T45" s="52"/>
+      <c r="U45" s="52"/>
+      <c r="V45" s="52"/>
+      <c r="W45" s="52"/>
+      <c r="X45" s="52"/>
+      <c r="Y45" s="52"/>
+      <c r="Z45" s="52"/>
+      <c r="AA45" s="52"/>
+      <c r="AB45" s="53"/>
       <c r="AC45" s="16"/>
     </row>
     <row r="46" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9672,27 +9712,27 @@
       <c r="E46" s="19"/>
       <c r="F46" s="19"/>
       <c r="G46" s="19"/>
-      <c r="H46" s="49"/>
-      <c r="I46" s="50"/>
-      <c r="J46" s="50"/>
-      <c r="K46" s="50"/>
-      <c r="L46" s="50"/>
-      <c r="M46" s="50"/>
-      <c r="N46" s="50"/>
-      <c r="O46" s="50"/>
-      <c r="P46" s="50"/>
-      <c r="Q46" s="50"/>
-      <c r="R46" s="50"/>
-      <c r="S46" s="50"/>
-      <c r="T46" s="50"/>
-      <c r="U46" s="50"/>
-      <c r="V46" s="50"/>
-      <c r="W46" s="50"/>
-      <c r="X46" s="50"/>
-      <c r="Y46" s="50"/>
-      <c r="Z46" s="50"/>
-      <c r="AA46" s="50"/>
-      <c r="AB46" s="51"/>
+      <c r="H46" s="51"/>
+      <c r="I46" s="52"/>
+      <c r="J46" s="52"/>
+      <c r="K46" s="52"/>
+      <c r="L46" s="52"/>
+      <c r="M46" s="52"/>
+      <c r="N46" s="52"/>
+      <c r="O46" s="52"/>
+      <c r="P46" s="52"/>
+      <c r="Q46" s="52"/>
+      <c r="R46" s="52"/>
+      <c r="S46" s="52"/>
+      <c r="T46" s="52"/>
+      <c r="U46" s="52"/>
+      <c r="V46" s="52"/>
+      <c r="W46" s="52"/>
+      <c r="X46" s="52"/>
+      <c r="Y46" s="52"/>
+      <c r="Z46" s="52"/>
+      <c r="AA46" s="52"/>
+      <c r="AB46" s="53"/>
       <c r="AC46" s="16"/>
     </row>
     <row r="47" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9702,27 +9742,27 @@
       <c r="E47" s="19"/>
       <c r="F47" s="19"/>
       <c r="G47" s="19"/>
-      <c r="H47" s="49"/>
-      <c r="I47" s="50"/>
-      <c r="J47" s="50"/>
-      <c r="K47" s="50"/>
-      <c r="L47" s="50"/>
-      <c r="M47" s="50"/>
-      <c r="N47" s="50"/>
-      <c r="O47" s="50"/>
-      <c r="P47" s="50"/>
-      <c r="Q47" s="50"/>
-      <c r="R47" s="50"/>
-      <c r="S47" s="50"/>
-      <c r="T47" s="50"/>
-      <c r="U47" s="50"/>
-      <c r="V47" s="50"/>
-      <c r="W47" s="50"/>
-      <c r="X47" s="50"/>
-      <c r="Y47" s="50"/>
-      <c r="Z47" s="50"/>
-      <c r="AA47" s="50"/>
-      <c r="AB47" s="51"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="52"/>
+      <c r="J47" s="52"/>
+      <c r="K47" s="52"/>
+      <c r="L47" s="52"/>
+      <c r="M47" s="52"/>
+      <c r="N47" s="52"/>
+      <c r="O47" s="52"/>
+      <c r="P47" s="52"/>
+      <c r="Q47" s="52"/>
+      <c r="R47" s="52"/>
+      <c r="S47" s="52"/>
+      <c r="T47" s="52"/>
+      <c r="U47" s="52"/>
+      <c r="V47" s="52"/>
+      <c r="W47" s="52"/>
+      <c r="X47" s="52"/>
+      <c r="Y47" s="52"/>
+      <c r="Z47" s="52"/>
+      <c r="AA47" s="52"/>
+      <c r="AB47" s="53"/>
       <c r="AC47" s="16"/>
     </row>
     <row r="48" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9732,27 +9772,27 @@
       <c r="E48" s="19"/>
       <c r="F48" s="19"/>
       <c r="G48" s="19"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="53"/>
-      <c r="J48" s="53"/>
-      <c r="K48" s="53"/>
-      <c r="L48" s="53"/>
-      <c r="M48" s="53"/>
-      <c r="N48" s="53"/>
-      <c r="O48" s="53"/>
-      <c r="P48" s="53"/>
-      <c r="Q48" s="53"/>
-      <c r="R48" s="53"/>
-      <c r="S48" s="53"/>
-      <c r="T48" s="53"/>
-      <c r="U48" s="53"/>
-      <c r="V48" s="53"/>
-      <c r="W48" s="53"/>
-      <c r="X48" s="53"/>
-      <c r="Y48" s="53"/>
-      <c r="Z48" s="53"/>
-      <c r="AA48" s="53"/>
-      <c r="AB48" s="54"/>
+      <c r="H48" s="54"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="55"/>
+      <c r="L48" s="55"/>
+      <c r="M48" s="55"/>
+      <c r="N48" s="55"/>
+      <c r="O48" s="55"/>
+      <c r="P48" s="55"/>
+      <c r="Q48" s="55"/>
+      <c r="R48" s="55"/>
+      <c r="S48" s="55"/>
+      <c r="T48" s="55"/>
+      <c r="U48" s="55"/>
+      <c r="V48" s="55"/>
+      <c r="W48" s="55"/>
+      <c r="X48" s="55"/>
+      <c r="Y48" s="55"/>
+      <c r="Z48" s="55"/>
+      <c r="AA48" s="55"/>
+      <c r="AB48" s="56"/>
       <c r="AC48" s="16"/>
     </row>
     <row r="49" spans="2:29" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -9825,11 +9865,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>28</v>
       </c>
@@ -10634,11 +10674,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>33</v>
       </c>
@@ -11776,11 +11816,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>34</v>
       </c>
@@ -14527,11 +14567,14 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B6:B23"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="H8:AB14"/>
-    <mergeCell ref="H16:AB22"/>
+    <mergeCell ref="B66:B83"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="H68:AB74"/>
+    <mergeCell ref="H76:AB82"/>
+    <mergeCell ref="B86:B103"/>
+    <mergeCell ref="D88:F88"/>
+    <mergeCell ref="H88:AB94"/>
+    <mergeCell ref="H96:AB102"/>
     <mergeCell ref="B26:B43"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="H28:AB34"/>
@@ -14540,14 +14583,11 @@
     <mergeCell ref="D48:F48"/>
     <mergeCell ref="H48:AB54"/>
     <mergeCell ref="H56:AB62"/>
-    <mergeCell ref="B66:B83"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="H68:AB74"/>
-    <mergeCell ref="H76:AB82"/>
-    <mergeCell ref="B86:B103"/>
-    <mergeCell ref="D88:F88"/>
-    <mergeCell ref="H88:AB94"/>
-    <mergeCell ref="H96:AB102"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B6:B23"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="H8:AB14"/>
+    <mergeCell ref="H16:AB22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -14574,11 +14614,11 @@
         <f xml:space="preserve"> '4.2.1'!B3</f>
         <v>.NET MAUI</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="47"/>
       <c r="I3" s="23" t="s">
         <v>41</v>
       </c>

</xml_diff>